<commit_message>
Add Ranking to region selection (catalogue what-if)
- Rank column (S, col 19) added to Scoring_Prod, Scoring_CVAL, Scoring_DR
  Formula: COUNTIF(Candidate_range, >this_candidate)+1; no array formulas
  Non-candidates (Candidate=-1) show blank; Rank 1 = best eligible candidate
- Ranked Candidates table in Result sheet (cols H-P): Prod / CVAL / DR side-by-side
  Uses INDEX/MATCH on Rank column; blank rows auto-suppress where no candidate at rank k
- How_To_Use updated: Rank formula documented, Result sheet map updated
- Verified: LibreOffice recalc 5 geographies, zero errors
  US 4 candidates, EU 4, AU 2, AP 2, ME(explicit-Prod) 1 — all correct
</commit_message>
<xml_diff>
--- a/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
+++ b/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
@@ -132,7 +132,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -204,6 +204,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -916,7 +919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B37"/>
+  <dimension ref="B1:B38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1057,14 +1060,14 @@
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>7. Scoring_Prod / 8. Scoring_CVAL / 9. Scoring_DR — PS component breakdown, AutoSelect flag and winners.</t>
+          <t>7. Scoring_Prod / 8. Scoring_CVAL / 9. Scoring_DR — PS component breakdown (α/β/γ/δ/ε raw + clamped), AutoSelect flag, Candidate (PS if eligible, −1 if not), and Rank (1 = best candidate, blank = not a candidate for that mode). Winner summary in cols T–U.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>10. Result — final placement (Prod / CVAL / DR), readiness, DR sizing (max-not-sum).</t>
+          <t>10. Result — final placement (Prod / CVAL / DR), readiness, DR sizing (max-not-sum), and a Ranked Candidate Regions table (cols H–P) showing all candidate regions ordered by PS for each mode.</t>
         </is>
       </c>
     </row>
@@ -1109,50 +1112,57 @@
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
+          <t>Rank formula (Scoring sheets, col S): Rank=COUNTIF(Candidate_range,"&gt;"&amp;this_candidate)+1. Non-candidates (Candidate=-1) are blank. Rank 1 = region with the highest PS score among eligible candidates. Because PS is a continuous float, ties are effectively impossible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="3" t="inlineStr">
+        <is>
           <t>DR sizing = MAX-NOT-SUM (A.6 / DR-017): DR req = MAX over source regions of (customers × vCPU).</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" s="3" t="inlineStr"/>
-    </row>
     <row r="32">
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>KNOWN GAPS / ASSUMPTIONS (surfaced, not hidden)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="6" t="inlineStr">
-        <is>
-          <t>• Metric = Total Cores. Prod = environment tag 'Prod'; everything else = Non-Prod.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
         <is>
+          <t>• Metric = Total Cores. Prod = environment tag 'Prod'; everything else = Non-Prod.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="6" t="inlineStr">
+        <is>
           <t>• Reserved &amp; Quota are DERIVED planning figures (max of even-share and actual alloc, +8% margin), not billed reservations — edit to model reality.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" s="7" t="inlineStr">
+    <row r="36">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>• Middle East has ~no real usage in the data — its two regions use a flagged SYNTHETIC pool so the geography can be exercised. Japan East (Asia Pacific) is 'pending' in the catalogue and is excluded.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>• total_customers is undefined in baseline v2.4 — mode selector on Policy (Live/Constant/Manual). γ values illustrative.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>• total_customers is undefined in baseline v2.4 — mode selector on Policy (Live/Constant/Manual). γ values illustrative.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>• PS_NonProd δ duplicates its α (baseline design-of-record). DR bootstrap / target are configurable placeholders.</t>
         </is>
@@ -1169,7 +1179,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -1178,6 +1188,15 @@
     <col width="4" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="8" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1202,6 +1221,11 @@
           <t>DR SIZING (max-not-sum, A.6 / DR-017)</t>
         </is>
       </c>
+      <c r="H3" s="29" t="inlineStr">
+        <is>
+          <t>RANKED CANDIDATE REGIONS  (Rank 1 = highest PS; blank = not a candidate for this mode)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
@@ -1213,6 +1237,21 @@
         <f>Setup!B3</f>
         <v/>
       </c>
+      <c r="H4" s="16" t="inlineStr">
+        <is>
+          <t>Prod</t>
+        </is>
+      </c>
+      <c r="K4" s="16" t="inlineStr">
+        <is>
+          <t>CVAL</t>
+        </is>
+      </c>
+      <c r="N4" s="16" t="inlineStr">
+        <is>
+          <t>DR</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
@@ -1233,6 +1272,51 @@
         <f>B11</f>
         <v/>
       </c>
+      <c r="H5" s="10" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="I5" s="10" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="J5" s="10" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="L5" s="10" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="M5" s="10" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
+      <c r="N5" s="10" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+      <c r="O5" s="10" t="inlineStr">
+        <is>
+          <t>Region</t>
+        </is>
+      </c>
+      <c r="P5" s="10" t="inlineStr">
+        <is>
+          <t>PS</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -1253,6 +1337,42 @@
         <f>SUMPRODUCT(MAX((Capacity_Usage!$C$4:$C$17=Setup!$B$11)*Capacity_Usage!$U$4:$U$17))</f>
         <v/>
       </c>
+      <c r="H6" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0))="","",1),"")</f>
+        <v/>
+      </c>
+      <c r="I6" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J6" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0))="","",1),"")</f>
+        <v/>
+      </c>
+      <c r="L6" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M6" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N6" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(1,Scoring_DR!$S$4:$S$17,0))="","",1),"")</f>
+        <v/>
+      </c>
+      <c r="O6" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P6" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="E7" s="14" t="inlineStr">
@@ -1264,6 +1384,42 @@
         <f>Setup!B7</f>
         <v/>
       </c>
+      <c r="H7" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0))="","",2),"")</f>
+        <v/>
+      </c>
+      <c r="I7" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J7" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0))="","",2),"")</f>
+        <v/>
+      </c>
+      <c r="L7" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M7" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(2,Scoring_DR!$S$4:$S$17,0))="","",2),"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P7" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -1286,8 +1442,44 @@
           <t>DR Requirement (max-not-sum)</t>
         </is>
       </c>
-      <c r="F8" s="29">
+      <c r="F8" s="30">
         <f>F6*F7</f>
+        <v/>
+      </c>
+      <c r="H8" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0))="","",3),"")</f>
+        <v/>
+      </c>
+      <c r="I8" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J8" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0))="","",3),"")</f>
+        <v/>
+      </c>
+      <c r="L8" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M8" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(3,Scoring_DR!$S$4:$S$17,0))="","",3),"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P8" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -1314,6 +1506,42 @@
         <f>IFERROR(INDEX(Capacity_Usage!$R$4:$R$17,MATCH(B11,Capacity_Usage!$B$4:$B$17,0)),0)</f>
         <v/>
       </c>
+      <c r="H9" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0))="","",4),"")</f>
+        <v/>
+      </c>
+      <c r="I9" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J9" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0))="","",4),"")</f>
+        <v/>
+      </c>
+      <c r="L9" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(4,Scoring_DR!$S$4:$S$17,0))="","",4),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P9" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
@@ -1338,6 +1566,42 @@
         <f>MAX(0,F8-F9)</f>
         <v/>
       </c>
+      <c r="H10" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0))="","",5),"")</f>
+        <v/>
+      </c>
+      <c r="I10" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0))="","",5),"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M10" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(5,Scoring_DR!$S$4:$S$17,0))="","",5),"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P10" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="14" t="inlineStr">
@@ -1353,10 +1617,84 @@
         <f>Scoring_DR!U3</f>
         <v/>
       </c>
-      <c r="E11" s="30" t="inlineStr">
+      <c r="E11" s="31" t="inlineStr">
         <is>
           <t>Note: illustrative — sources = regions in DR scope geography.</t>
         </is>
+      </c>
+      <c r="H11" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0))="","",6),"")</f>
+        <v/>
+      </c>
+      <c r="I11" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0))="","",6),"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M11" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(6,Scoring_DR!$S$4:$S$17,0))="","",6),"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="H12" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0))="","",7),"")</f>
+        <v/>
+      </c>
+      <c r="I12" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0))="","",7),"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M12" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(7,Scoring_DR!$S$4:$S$17,0))="","",7),"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -1365,8 +1703,82 @@
           <t>Readiness State</t>
         </is>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="30">
         <f>IF(B9="NONE ELIGIBLE","QUOTA_DEFICIT / NEEDS EXPLICIT REGION (Prod)",IF(B10="NONE ELIGIBLE","CAPACITY_UNAVAILABLE (CVAL)",IF(B11="NONE ELIGIBLE","READY_WITH_RISK (no DR region)","READY")))</f>
+        <v/>
+      </c>
+      <c r="H13" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0))="","",8),"")</f>
+        <v/>
+      </c>
+      <c r="I13" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0))="","",8),"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M13" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(8,Scoring_DR!$S$4:$S$17,0))="","",8),"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="H14" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0))="","",9),"")</f>
+        <v/>
+      </c>
+      <c r="I14" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0))="","",9),"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M14" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(9,Scoring_DR!$S$4:$S$17,0))="","",9),"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
     </row>
@@ -1380,11 +1792,203 @@
         <f>"whatif-catalogue-v1  (weights "&amp;TEXT(Policy!B7,"0.00")&amp;" — "&amp;Policy!B8&amp;")"</f>
         <v/>
       </c>
+      <c r="H15" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0))="","",10),"")</f>
+        <v/>
+      </c>
+      <c r="I15" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0))="","",10),"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M15" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(10,Scoring_DR!$S$4:$S$17,0))="","",10),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="H16" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0))="","",11),"")</f>
+        <v/>
+      </c>
+      <c r="I16" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0))="","",11),"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M16" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(11,Scoring_DR!$S$4:$S$17,0))="","",11),"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="H17" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0))="","",12),"")</f>
+        <v/>
+      </c>
+      <c r="I17" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0))="","",12),"")</f>
+        <v/>
+      </c>
+      <c r="L17" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M17" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(12,Scoring_DR!$S$4:$S$17,0))="","",12),"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="H18" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0))="","",13),"")</f>
+        <v/>
+      </c>
+      <c r="I18" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0))="","",13),"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(13,Scoring_DR!$S$4:$S$17,0))="","",13),"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="H19" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_Prod!$S$4:$S$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0))="","",14),"")</f>
+        <v/>
+      </c>
+      <c r="I19" s="11">
+        <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="27">
+        <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_CVAL!$S$4:$S$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0))="","",14),"")</f>
+        <v/>
+      </c>
+      <c r="L19" s="11">
+        <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="M19" s="27">
+        <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="11">
+        <f>IFERROR(IF(INDEX(Scoring_DR!$S$4:$S$17,MATCH(14,Scoring_DR!$S$4:$S$17,0))="","",14),"")</f>
+        <v/>
+      </c>
+      <c r="O19" s="11">
+        <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="27">
+        <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
+    <mergeCell ref="K4:M4"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="H4:J4"/>
+    <mergeCell ref="N4:P4"/>
+    <mergeCell ref="H3:P3"/>
     <mergeCell ref="E3:F3"/>
-    <mergeCell ref="E11:F11"/>
   </mergeCells>
   <conditionalFormatting sqref="B13">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -4740,6 +5344,7 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="6" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
@@ -4858,6 +5463,11 @@
           <t>Candidate</t>
         </is>
       </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
       <c r="T3" s="14" t="inlineStr">
         <is>
           <t>Region</t>
@@ -4941,6 +5551,10 @@
         <f>IF(AND(C4=1,D4=1,E4=1),Q4,-1)</f>
         <v/>
       </c>
+      <c r="S4" s="11">
+        <f>IF(R4&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R4)+1)</f>
+        <v/>
+      </c>
       <c r="T4" s="14" t="inlineStr">
         <is>
           <t>Score</t>
@@ -5024,6 +5638,10 @@
         <f>IF(AND(C5=1,D5=1,E5=1),Q5,-1)</f>
         <v/>
       </c>
+      <c r="S5" s="11">
+        <f>IF(R5&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R5)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11">
@@ -5098,6 +5716,10 @@
         <f>IF(AND(C6=1,D6=1,E6=1),Q6,-1)</f>
         <v/>
       </c>
+      <c r="S6" s="11">
+        <f>IF(R6&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R6)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11">
@@ -5172,6 +5794,10 @@
         <f>IF(AND(C7=1,D7=1,E7=1),Q7,-1)</f>
         <v/>
       </c>
+      <c r="S7" s="11">
+        <f>IF(R7&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R7)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11">
@@ -5246,6 +5872,10 @@
         <f>IF(AND(C8=1,D8=1,E8=1),Q8,-1)</f>
         <v/>
       </c>
+      <c r="S8" s="11">
+        <f>IF(R8&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R8)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11">
@@ -5320,6 +5950,10 @@
         <f>IF(AND(C9=1,D9=1,E9=1),Q9,-1)</f>
         <v/>
       </c>
+      <c r="S9" s="11">
+        <f>IF(R9&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R9)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11">
@@ -5394,6 +6028,10 @@
         <f>IF(AND(C10=1,D10=1,E10=1),Q10,-1)</f>
         <v/>
       </c>
+      <c r="S10" s="11">
+        <f>IF(R10&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R10)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11">
@@ -5468,6 +6106,10 @@
         <f>IF(AND(C11=1,D11=1,E11=1),Q11,-1)</f>
         <v/>
       </c>
+      <c r="S11" s="11">
+        <f>IF(R11&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R11)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11">
@@ -5542,6 +6184,10 @@
         <f>IF(AND(C12=1,D12=1,E12=1),Q12,-1)</f>
         <v/>
       </c>
+      <c r="S12" s="11">
+        <f>IF(R12&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R12)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11">
@@ -5616,6 +6262,10 @@
         <f>IF(AND(C13=1,D13=1,E13=1),Q13,-1)</f>
         <v/>
       </c>
+      <c r="S13" s="11">
+        <f>IF(R13&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R13)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11">
@@ -5690,6 +6340,10 @@
         <f>IF(AND(C14=1,D14=1,E14=1),Q14,-1)</f>
         <v/>
       </c>
+      <c r="S14" s="11">
+        <f>IF(R14&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R14)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11">
@@ -5764,6 +6418,10 @@
         <f>IF(AND(C15=1,D15=1,E15=1),Q15,-1)</f>
         <v/>
       </c>
+      <c r="S15" s="11">
+        <f>IF(R15&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R15)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11">
@@ -5838,6 +6496,10 @@
         <f>IF(AND(C16=1,D16=1,E16=1),Q16,-1)</f>
         <v/>
       </c>
+      <c r="S16" s="11">
+        <f>IF(R16&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R16)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11">
@@ -5910,6 +6572,10 @@
       </c>
       <c r="R17" s="11">
         <f>IF(AND(C17=1,D17=1,E17=1),Q17,-1)</f>
+        <v/>
+      </c>
+      <c r="S17" s="11">
+        <f>IF(R17&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R17)+1)</f>
         <v/>
       </c>
     </row>
@@ -5946,6 +6612,7 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="6" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
@@ -6064,6 +6731,11 @@
           <t>Candidate</t>
         </is>
       </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
       <c r="T3" s="14" t="inlineStr">
         <is>
           <t>Score</t>
@@ -6147,6 +6819,10 @@
         <f>IF(AND(C4=1,D4=1,E4=1,A4&lt;&gt;Scoring_Prod!$U$3),Q4,-1)</f>
         <v/>
       </c>
+      <c r="S4" s="11">
+        <f>IF(R4&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R4)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11">
@@ -6221,6 +6897,10 @@
         <f>IF(AND(C5=1,D5=1,E5=1,A5&lt;&gt;Scoring_Prod!$U$3),Q5,-1)</f>
         <v/>
       </c>
+      <c r="S5" s="11">
+        <f>IF(R5&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R5)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11">
@@ -6295,6 +6975,10 @@
         <f>IF(AND(C6=1,D6=1,E6=1,A6&lt;&gt;Scoring_Prod!$U$3),Q6,-1)</f>
         <v/>
       </c>
+      <c r="S6" s="11">
+        <f>IF(R6&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R6)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11">
@@ -6369,6 +7053,10 @@
         <f>IF(AND(C7=1,D7=1,E7=1,A7&lt;&gt;Scoring_Prod!$U$3),Q7,-1)</f>
         <v/>
       </c>
+      <c r="S7" s="11">
+        <f>IF(R7&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R7)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11">
@@ -6443,6 +7131,10 @@
         <f>IF(AND(C8=1,D8=1,E8=1,A8&lt;&gt;Scoring_Prod!$U$3),Q8,-1)</f>
         <v/>
       </c>
+      <c r="S8" s="11">
+        <f>IF(R8&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R8)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11">
@@ -6517,6 +7209,10 @@
         <f>IF(AND(C9=1,D9=1,E9=1,A9&lt;&gt;Scoring_Prod!$U$3),Q9,-1)</f>
         <v/>
       </c>
+      <c r="S9" s="11">
+        <f>IF(R9&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R9)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11">
@@ -6591,6 +7287,10 @@
         <f>IF(AND(C10=1,D10=1,E10=1,A10&lt;&gt;Scoring_Prod!$U$3),Q10,-1)</f>
         <v/>
       </c>
+      <c r="S10" s="11">
+        <f>IF(R10&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R10)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11">
@@ -6665,6 +7365,10 @@
         <f>IF(AND(C11=1,D11=1,E11=1,A11&lt;&gt;Scoring_Prod!$U$3),Q11,-1)</f>
         <v/>
       </c>
+      <c r="S11" s="11">
+        <f>IF(R11&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R11)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11">
@@ -6739,6 +7443,10 @@
         <f>IF(AND(C12=1,D12=1,E12=1,A12&lt;&gt;Scoring_Prod!$U$3),Q12,-1)</f>
         <v/>
       </c>
+      <c r="S12" s="11">
+        <f>IF(R12&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R12)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11">
@@ -6813,6 +7521,10 @@
         <f>IF(AND(C13=1,D13=1,E13=1,A13&lt;&gt;Scoring_Prod!$U$3),Q13,-1)</f>
         <v/>
       </c>
+      <c r="S13" s="11">
+        <f>IF(R13&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R13)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11">
@@ -6887,6 +7599,10 @@
         <f>IF(AND(C14=1,D14=1,E14=1,A14&lt;&gt;Scoring_Prod!$U$3),Q14,-1)</f>
         <v/>
       </c>
+      <c r="S14" s="11">
+        <f>IF(R14&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R14)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11">
@@ -6961,6 +7677,10 @@
         <f>IF(AND(C15=1,D15=1,E15=1,A15&lt;&gt;Scoring_Prod!$U$3),Q15,-1)</f>
         <v/>
       </c>
+      <c r="S15" s="11">
+        <f>IF(R15&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R15)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11">
@@ -7035,6 +7755,10 @@
         <f>IF(AND(C16=1,D16=1,E16=1,A16&lt;&gt;Scoring_Prod!$U$3),Q16,-1)</f>
         <v/>
       </c>
+      <c r="S16" s="11">
+        <f>IF(R16&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R16)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11">
@@ -7107,6 +7831,10 @@
       </c>
       <c r="R17" s="11">
         <f>IF(AND(C17=1,D17=1,E17=1,A17&lt;&gt;Scoring_Prod!$U$3),Q17,-1)</f>
+        <v/>
+      </c>
+      <c r="S17" s="11">
+        <f>IF(R17&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R17)+1)</f>
         <v/>
       </c>
     </row>
@@ -7142,6 +7870,7 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="6" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
@@ -7260,6 +7989,11 @@
           <t>Candidate</t>
         </is>
       </c>
+      <c r="S3" s="10" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
       <c r="T3" s="14" t="inlineStr">
         <is>
           <t>Score</t>
@@ -7343,6 +8077,10 @@
         <f>IF(AND(C4=1,D4=1,E4=1,A4&lt;&gt;Scoring_Prod!$U$3),Q4,-1)</f>
         <v/>
       </c>
+      <c r="S4" s="11">
+        <f>IF(R4&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R4)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11">
@@ -7417,6 +8155,10 @@
         <f>IF(AND(C5=1,D5=1,E5=1,A5&lt;&gt;Scoring_Prod!$U$3),Q5,-1)</f>
         <v/>
       </c>
+      <c r="S5" s="11">
+        <f>IF(R5&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R5)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11">
@@ -7491,6 +8233,10 @@
         <f>IF(AND(C6=1,D6=1,E6=1,A6&lt;&gt;Scoring_Prod!$U$3),Q6,-1)</f>
         <v/>
       </c>
+      <c r="S6" s="11">
+        <f>IF(R6&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R6)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11">
@@ -7565,6 +8311,10 @@
         <f>IF(AND(C7=1,D7=1,E7=1,A7&lt;&gt;Scoring_Prod!$U$3),Q7,-1)</f>
         <v/>
       </c>
+      <c r="S7" s="11">
+        <f>IF(R7&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R7)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11">
@@ -7639,6 +8389,10 @@
         <f>IF(AND(C8=1,D8=1,E8=1,A8&lt;&gt;Scoring_Prod!$U$3),Q8,-1)</f>
         <v/>
       </c>
+      <c r="S8" s="11">
+        <f>IF(R8&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R8)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11">
@@ -7713,6 +8467,10 @@
         <f>IF(AND(C9=1,D9=1,E9=1,A9&lt;&gt;Scoring_Prod!$U$3),Q9,-1)</f>
         <v/>
       </c>
+      <c r="S9" s="11">
+        <f>IF(R9&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R9)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11">
@@ -7787,6 +8545,10 @@
         <f>IF(AND(C10=1,D10=1,E10=1,A10&lt;&gt;Scoring_Prod!$U$3),Q10,-1)</f>
         <v/>
       </c>
+      <c r="S10" s="11">
+        <f>IF(R10&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R10)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11">
@@ -7861,6 +8623,10 @@
         <f>IF(AND(C11=1,D11=1,E11=1,A11&lt;&gt;Scoring_Prod!$U$3),Q11,-1)</f>
         <v/>
       </c>
+      <c r="S11" s="11">
+        <f>IF(R11&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R11)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11">
@@ -7935,6 +8701,10 @@
         <f>IF(AND(C12=1,D12=1,E12=1,A12&lt;&gt;Scoring_Prod!$U$3),Q12,-1)</f>
         <v/>
       </c>
+      <c r="S12" s="11">
+        <f>IF(R12&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R12)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11">
@@ -8009,6 +8779,10 @@
         <f>IF(AND(C13=1,D13=1,E13=1,A13&lt;&gt;Scoring_Prod!$U$3),Q13,-1)</f>
         <v/>
       </c>
+      <c r="S13" s="11">
+        <f>IF(R13&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R13)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11">
@@ -8083,6 +8857,10 @@
         <f>IF(AND(C14=1,D14=1,E14=1,A14&lt;&gt;Scoring_Prod!$U$3),Q14,-1)</f>
         <v/>
       </c>
+      <c r="S14" s="11">
+        <f>IF(R14&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R14)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11">
@@ -8157,6 +8935,10 @@
         <f>IF(AND(C15=1,D15=1,E15=1,A15&lt;&gt;Scoring_Prod!$U$3),Q15,-1)</f>
         <v/>
       </c>
+      <c r="S15" s="11">
+        <f>IF(R15&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R15)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11">
@@ -8231,6 +9013,10 @@
         <f>IF(AND(C16=1,D16=1,E16=1,A16&lt;&gt;Scoring_Prod!$U$3),Q16,-1)</f>
         <v/>
       </c>
+      <c r="S16" s="11">
+        <f>IF(R16&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R16)+1)</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11">
@@ -8303,6 +9089,10 @@
       </c>
       <c r="R17" s="11">
         <f>IF(AND(C17=1,D17=1,E17=1,A17&lt;&gt;Scoring_Prod!$U$3),Q17,-1)</f>
+        <v/>
+      </c>
+      <c r="S17" s="11">
+        <f>IF(R17&lt;0,"",COUNTIF($R$4:$R$17,"&gt;"&amp;R17)+1)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(catalogue): rename Saudi Arabia Central → Saudi Arabia East; mark as future region (GA target Q4 2026, Eastern Province); add Usage_Source provenance footer for absent ACRME regions
</commit_message>
<xml_diff>
--- a/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
+++ b/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
@@ -28,7 +28,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -56,6 +56,14 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
     </font>
     <font>
       <i val="1"/>
@@ -132,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -171,13 +179,24 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -190,13 +209,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -210,7 +223,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -977,7 +990,7 @@
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>• EXCEPTION: the Middle East regions (Saudi Arabia Central, UAE North) are RESTRICTED — production-only, and NOT auto-selected by the engine unless you explicitly supply one as the Prod region on Setup (cell B8). This matches the baseline 'Restricted deployment regions' definition. So for a Middle East run you must name a Prod region; DR still auto-selects cross-geo in a Standard Europe region.</t>
+          <t>• EXCEPTION: the Middle East regions (Saudi Arabia East, UAE North) are RESTRICTED — production-only, and NOT auto-selected by the engine unless you explicitly supply one as the Prod region on Setup (cell B8). This matches the baseline 'Restricted deployment regions' definition. So for a Middle East run you must name a Prod region; DR still auto-selects cross-geo in a Standard Europe region.</t>
         </is>
       </c>
     </row>
@@ -1150,7 +1163,7 @@
     <row r="36">
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>• Middle East has ~no real usage in the data — its two regions use a flagged SYNTHETIC pool so the geography can be exercised. Japan East (Asia Pacific) is 'pending' in the catalogue and is excluded.</t>
+          <t>• Middle East has ~no real usage in the data — its two regions use a flagged SYNTHETIC pool so the geography can be exercised. Saudi Arabia East is a FUTURE REGION (not yet GA; Microsoft target Q4 2026, Eastern Province; no real usage data will exist until launch). UAE North is GA but absent from ACRME source data. Japan East (Asia Pacific) is 'pending' in the catalogue and is excluded.</t>
         </is>
       </c>
     </row>
@@ -1216,12 +1229,12 @@
         <f>Setup!B9</f>
         <v/>
       </c>
-      <c r="E3" s="26" t="inlineStr">
+      <c r="E3" s="29" t="inlineStr">
         <is>
           <t>DR SIZING (max-not-sum, A.6 / DR-017)</t>
         </is>
       </c>
-      <c r="H3" s="29" t="inlineStr">
+      <c r="H3" s="32" t="inlineStr">
         <is>
           <t>RANKED CANDIDATE REGIONS  (Rank 1 = highest PS; blank = not a candidate for this mode)</t>
         </is>
@@ -1237,17 +1250,17 @@
         <f>Setup!B3</f>
         <v/>
       </c>
-      <c r="H4" s="16" t="inlineStr">
+      <c r="H4" s="22" t="inlineStr">
         <is>
           <t>Prod</t>
         </is>
       </c>
-      <c r="K4" s="16" t="inlineStr">
+      <c r="K4" s="22" t="inlineStr">
         <is>
           <t>CVAL</t>
         </is>
       </c>
-      <c r="N4" s="16" t="inlineStr">
+      <c r="N4" s="22" t="inlineStr">
         <is>
           <t>DR</t>
         </is>
@@ -1345,7 +1358,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1357,7 +1370,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1369,7 +1382,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P6" s="27">
+      <c r="P6" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1392,7 +1405,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1404,7 +1417,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M7" s="27">
+      <c r="M7" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1416,7 +1429,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P7" s="27">
+      <c r="P7" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1442,7 +1455,7 @@
           <t>DR Requirement (max-not-sum)</t>
         </is>
       </c>
-      <c r="F8" s="30">
+      <c r="F8" s="33">
         <f>F6*F7</f>
         <v/>
       </c>
@@ -1454,7 +1467,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1466,7 +1479,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M8" s="27">
+      <c r="M8" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1478,7 +1491,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P8" s="27">
+      <c r="P8" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1493,7 +1506,7 @@
         <f>Scoring_Prod!U3</f>
         <v/>
       </c>
-      <c r="C9" s="27">
+      <c r="C9" s="30">
         <f>Scoring_Prod!U4</f>
         <v/>
       </c>
@@ -1514,7 +1527,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1526,7 +1539,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M9" s="27">
+      <c r="M9" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1538,7 +1551,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P9" s="27">
+      <c r="P9" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1553,7 +1566,7 @@
         <f>Scoring_CVAL!U2</f>
         <v/>
       </c>
-      <c r="C10" s="27">
+      <c r="C10" s="30">
         <f>Scoring_CVAL!U3</f>
         <v/>
       </c>
@@ -1574,7 +1587,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J10" s="27">
+      <c r="J10" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1586,7 +1599,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M10" s="27">
+      <c r="M10" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1598,7 +1611,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P10" s="27">
+      <c r="P10" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1613,11 +1626,11 @@
         <f>Scoring_DR!U2</f>
         <v/>
       </c>
-      <c r="C11" s="27">
+      <c r="C11" s="30">
         <f>Scoring_DR!U3</f>
         <v/>
       </c>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="E11" s="34" t="inlineStr">
         <is>
           <t>Note: illustrative — sources = regions in DR scope geography.</t>
         </is>
@@ -1630,7 +1643,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J11" s="27">
+      <c r="J11" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1642,7 +1655,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M11" s="27">
+      <c r="M11" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1654,7 +1667,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1668,7 +1681,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1680,7 +1693,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M12" s="27">
+      <c r="M12" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1692,7 +1705,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P12" s="27">
+      <c r="P12" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1703,7 +1716,7 @@
           <t>Readiness State</t>
         </is>
       </c>
-      <c r="B13" s="30">
+      <c r="B13" s="33">
         <f>IF(B9="NONE ELIGIBLE","QUOTA_DEFICIT / NEEDS EXPLICIT REGION (Prod)",IF(B10="NONE ELIGIBLE","CAPACITY_UNAVAILABLE (CVAL)",IF(B11="NONE ELIGIBLE","READY_WITH_RISK (no DR region)","READY")))</f>
         <v/>
       </c>
@@ -1715,7 +1728,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J13" s="27">
+      <c r="J13" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1727,7 +1740,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M13" s="27">
+      <c r="M13" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1739,7 +1752,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P13" s="27">
+      <c r="P13" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1753,7 +1766,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J14" s="27">
+      <c r="J14" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1765,7 +1778,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M14" s="27">
+      <c r="M14" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1777,7 +1790,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P14" s="27">
+      <c r="P14" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1800,7 +1813,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J15" s="27">
+      <c r="J15" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1812,7 +1825,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M15" s="27">
+      <c r="M15" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1824,7 +1837,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P15" s="27">
+      <c r="P15" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1838,7 +1851,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J16" s="27">
+      <c r="J16" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1850,7 +1863,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M16" s="27">
+      <c r="M16" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1862,7 +1875,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P16" s="27">
+      <c r="P16" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1876,7 +1889,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J17" s="27">
+      <c r="J17" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1888,7 +1901,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M17" s="27">
+      <c r="M17" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1900,7 +1913,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P17" s="27">
+      <c r="P17" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1914,7 +1927,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J18" s="27">
+      <c r="J18" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1926,7 +1939,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M18" s="27">
+      <c r="M18" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1938,7 +1951,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P18" s="27">
+      <c r="P18" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1952,7 +1965,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J19" s="27">
+      <c r="J19" s="30">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1964,7 +1977,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M19" s="27">
+      <c r="M19" s="30">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1976,7 +1989,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P19" s="27">
+      <c r="P19" s="30">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -2015,7 +2028,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -2039,7 +2052,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Real aggregation from SKU_USage (1).xlsx (Total Cores). Prod = tag 'Prod'; all other tags = Non-Prod. This is provenance; the engine reads the distributed Capacity_Usage sheet.</t>
+          <t>Real aggregation from SKU_USage (1).xlsx (Total Cores). Prod = tag 'Prod'; all other tags = Non-Prod. This is provenance; the engine reads the distributed Capacity_Usage sheet. ACRME catalogue regions absent from source data use SYNTHETIC capacity — see the footer section below. NOTE: Saudi Arabia East is a FUTURE REGION (not yet GA; Microsoft target Q4 2026, Eastern Province) — no real usage data exists; capacity figures are entirely SYNTHETIC.</t>
         </is>
       </c>
     </row>
@@ -2635,10 +2648,102 @@
       <c r="H18" s="14" t="n"/>
       <c r="I18" s="14" t="n"/>
     </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>ACRME CATALOGUE REGIONS — ABSENT FROM SOURCE DATA (capacity figures are SYNTHETIC)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Canada Central</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D21" s="19" t="inlineStr">
+        <is>
+          <t>absent from source data; mock subscription count used; capacity figures SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="E21" s="20" t="n"/>
+      <c r="F21" s="20" t="n"/>
+      <c r="G21" s="20" t="n"/>
+      <c r="H21" s="20" t="n"/>
+      <c r="I21" s="20" t="n"/>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>Saudi Arabia East</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="C22" s="21" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="D22" s="19" t="inlineStr">
+        <is>
+          <t>FUTURE REGION — not yet GA (Microsoft target Q4 2026, Eastern Province); no real usage data; capacity figures SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="E22" s="20" t="n"/>
+      <c r="F22" s="20" t="n"/>
+      <c r="G22" s="20" t="n"/>
+      <c r="H22" s="20" t="n"/>
+      <c r="I22" s="20" t="n"/>
+    </row>
+    <row r="23" ht="30" customHeight="1">
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>UAE North</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>Restricted</t>
+        </is>
+      </c>
+      <c r="D23" s="19" t="inlineStr">
+        <is>
+          <t>GA region — absent from ACRME source data; capacity figures SYNTHETIC</t>
+        </is>
+      </c>
+      <c r="E23" s="20" t="n"/>
+      <c r="F23" s="20" t="n"/>
+      <c r="G23" s="20" t="n"/>
+      <c r="H23" s="20" t="n"/>
+      <c r="I23" s="20" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D22:I22"/>
+    <mergeCell ref="D23:I23"/>
     <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="D21:I21"/>
+    <mergeCell ref="A20:I20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2676,12 +2781,12 @@
       </c>
     </row>
     <row r="2">
-      <c r="E2" s="16" t="inlineStr">
+      <c r="E2" s="22" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="F2" s="16" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>vCPU/VM</t>
         </is>
@@ -2693,17 +2798,17 @@
           <t>Geography</t>
         </is>
       </c>
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E3" s="18" t="inlineStr">
+      <c r="E3" s="20" t="inlineStr">
         <is>
           <t>E16ads_v5</t>
         </is>
       </c>
-      <c r="F3" s="18" t="n">
+      <c r="F3" s="20" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2713,17 +2818,17 @@
           <t>SKU</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B4" s="23" t="inlineStr">
         <is>
           <t>E16ads_v5</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="20" t="inlineStr">
         <is>
           <t>E32ads_v5</t>
         </is>
       </c>
-      <c r="F4" s="18" t="n">
+      <c r="F4" s="20" t="n">
         <v>32</v>
       </c>
     </row>
@@ -2733,15 +2838,15 @@
           <t>VM count</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="E5" s="18" t="inlineStr">
+      <c r="E5" s="20" t="inlineStr">
         <is>
           <t>E8ads_v5</t>
         </is>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="20" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2751,16 +2856,16 @@
           <t>vCPU per VM</t>
         </is>
       </c>
-      <c r="B6" s="19">
+      <c r="B6" s="24">
         <f>VLOOKUP(B4,E3:F10,2,FALSE)</f>
         <v/>
       </c>
-      <c r="E6" s="18" t="inlineStr">
+      <c r="E6" s="20" t="inlineStr">
         <is>
           <t>E4ads_v5</t>
         </is>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="20" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2770,16 +2875,16 @@
           <t>Requested vCPU</t>
         </is>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="25">
         <f>B5*B6</f>
         <v/>
       </c>
-      <c r="E7" s="18" t="inlineStr">
+      <c r="E7" s="20" t="inlineStr">
         <is>
           <t>D8ads_v5</t>
         </is>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="20" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2789,13 +2894,13 @@
           <t>Prod region (req. for Middle East)</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr"/>
-      <c r="E8" s="18" t="inlineStr">
+      <c r="B8" s="23" t="inlineStr"/>
+      <c r="E8" s="20" t="inlineStr">
         <is>
           <t>D4ads_v5</t>
         </is>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="20" t="n">
         <v>4</v>
       </c>
     </row>
@@ -2805,17 +2910,17 @@
           <t>Customer ID</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>CUST-0042</t>
         </is>
       </c>
-      <c r="E9" s="18" t="inlineStr">
+      <c r="E9" s="20" t="inlineStr">
         <is>
           <t>D2ads_v5</t>
         </is>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="20" t="n">
         <v>2</v>
       </c>
     </row>
@@ -2825,16 +2930,16 @@
           <t>Distribution model</t>
         </is>
       </c>
-      <c r="B10" s="19">
+      <c r="B10" s="24">
         <f>VLOOKUP(B3,E13:G17,2,FALSE)</f>
         <v/>
       </c>
-      <c r="E10" s="18" t="inlineStr">
+      <c r="E10" s="20" t="inlineStr">
         <is>
           <t>D16ads_v5</t>
         </is>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="20" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2844,108 +2949,108 @@
           <t>DR scope geography</t>
         </is>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="24">
         <f>VLOOKUP(B3,E13:G17,3,FALSE)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="22" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="G12" s="16" t="inlineStr">
+      <c r="G12" s="22" t="inlineStr">
         <is>
           <t>DR Scope Geo</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="E13" s="18" t="inlineStr">
+      <c r="E13" s="20" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="F13" s="18" t="inlineStr">
+      <c r="F13" s="20" t="inlineStr">
         <is>
           <t>3-region</t>
         </is>
       </c>
-      <c r="G13" s="18" t="inlineStr">
+      <c r="G13" s="20" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="E14" s="18" t="inlineStr">
+      <c r="E14" s="20" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="F14" s="18" t="inlineStr">
+      <c r="F14" s="20" t="inlineStr">
         <is>
           <t>2-region</t>
         </is>
       </c>
-      <c r="G14" s="18" t="inlineStr">
+      <c r="G14" s="20" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="18" t="inlineStr">
+      <c r="E15" s="20" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="F15" s="18" t="inlineStr">
+      <c r="F15" s="20" t="inlineStr">
         <is>
           <t>2-region</t>
         </is>
       </c>
-      <c r="G15" s="18" t="inlineStr">
+      <c r="G15" s="20" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="E16" s="18" t="inlineStr">
+      <c r="E16" s="20" t="inlineStr">
         <is>
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="F16" s="18" t="inlineStr">
+      <c r="F16" s="20" t="inlineStr">
         <is>
           <t>2-region</t>
         </is>
       </c>
-      <c r="G16" s="18" t="inlineStr">
+      <c r="G16" s="20" t="inlineStr">
         <is>
           <t>Asia Pacific</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="18" t="inlineStr">
+      <c r="E17" s="20" t="inlineStr">
         <is>
           <t>Middle East</t>
         </is>
       </c>
-      <c r="F17" s="18" t="inlineStr">
+      <c r="F17" s="20" t="inlineStr">
         <is>
           <t>cross-geo</t>
         </is>
       </c>
-      <c r="G17" s="18" t="inlineStr">
+      <c r="G17" s="20" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
@@ -2996,7 +3101,7 @@
           <t>alpha (α) — Capacity headroom</t>
         </is>
       </c>
-      <c r="B2" s="17" t="n">
+      <c r="B2" s="23" t="n">
         <v>0.3</v>
       </c>
     </row>
@@ -3006,7 +3111,7 @@
           <t>beta (β) — Quota headroom</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3" s="23" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -3016,7 +3121,7 @@
           <t>gamma (γ) — Distribution fairness</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="23" t="n">
         <v>0.25</v>
       </c>
     </row>
@@ -3026,7 +3131,7 @@
           <t>delta (δ) — DR readiness</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="23" t="n">
         <v>0.15</v>
       </c>
     </row>
@@ -3036,7 +3141,7 @@
           <t>epsilon (ε) — Zone diversity</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="23" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -3046,7 +3151,7 @@
           <t>Weight sum</t>
         </is>
       </c>
-      <c r="B7" s="20">
+      <c r="B7" s="25">
         <f>SUM(B2:B6)</f>
         <v/>
       </c>
@@ -3057,7 +3162,7 @@
           <t>Validation</t>
         </is>
       </c>
-      <c r="B8" s="19">
+      <c r="B8" s="24">
         <f>IF(ABS(B7-1)&lt;=0.001,"VALID","INVALID — must sum to 1.0")</f>
         <v/>
       </c>
@@ -3068,15 +3173,15 @@
           <t>total_customers mode (1=Live 2=Constant 3=Manual)</t>
         </is>
       </c>
-      <c r="B10" s="17" t="n">
+      <c r="B10" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>Geography</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="22" t="inlineStr">
         <is>
           <t>Constant</t>
         </is>
@@ -3088,25 +3193,25 @@
           <t>Manual total_customers</t>
         </is>
       </c>
-      <c r="B11" s="17" t="n">
+      <c r="B11" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="D11" s="18" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>US</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="20" t="n">
         <v>150</v>
       </c>
     </row>
     <row r="12">
-      <c r="D12" s="18" t="inlineStr">
+      <c r="D12" s="20" t="inlineStr">
         <is>
           <t>EU</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="20" t="n">
         <v>90</v>
       </c>
     </row>
@@ -3116,15 +3221,15 @@
           <t>DR bootstrap qty (vCPU)</t>
         </is>
       </c>
-      <c r="B13" s="17" t="n">
+      <c r="B13" s="23" t="n">
         <v>40</v>
       </c>
-      <c r="D13" s="18" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="20" t="n">
         <v>40</v>
       </c>
     </row>
@@ -3134,15 +3239,15 @@
           <t>DR coverage target</t>
         </is>
       </c>
-      <c r="B14" s="17" t="n">
+      <c r="B14" s="23" t="n">
         <v>0.8</v>
       </c>
-      <c r="D14" s="18" t="inlineStr">
+      <c r="D14" s="20" t="inlineStr">
         <is>
           <t>Asia Pacific</t>
         </is>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="20" t="n">
         <v>50</v>
       </c>
     </row>
@@ -3152,15 +3257,15 @@
           <t>Min Prod headroom (vCPU)</t>
         </is>
       </c>
-      <c r="B15" s="17" t="n">
+      <c r="B15" s="23" t="n">
         <v>20</v>
       </c>
-      <c r="D15" s="18" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>Middle East</t>
         </is>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="20" t="n">
         <v>10</v>
       </c>
     </row>
@@ -3170,7 +3275,7 @@
           <t>Min NonProd headroom (vCPU)</t>
         </is>
       </c>
-      <c r="B16" s="17" t="n">
+      <c r="B16" s="23" t="n">
         <v>20</v>
       </c>
     </row>
@@ -3180,7 +3285,7 @@
           <t>Min DR headroom (vCPU)</t>
         </is>
       </c>
-      <c r="B17" s="17" t="n">
+      <c r="B17" s="23" t="n">
         <v>16</v>
       </c>
     </row>
@@ -3377,61 +3482,61 @@
           <t>3-region</t>
         </is>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="21" t="n">
+      <c r="F4" s="26" t="n">
         <v>42492</v>
       </c>
-      <c r="G4" s="21" t="n">
+      <c r="G4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="22">
+      <c r="H4" s="27">
         <f>F4-G4</f>
         <v/>
       </c>
-      <c r="I4" s="21" t="n">
+      <c r="I4" s="26" t="n">
         <v>63738</v>
       </c>
-      <c r="J4" s="21" t="n">
+      <c r="J4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="22">
+      <c r="K4" s="27">
         <f>I4-J4</f>
         <v/>
       </c>
-      <c r="L4" s="21" t="n">
+      <c r="L4" s="26" t="n">
         <v>94710</v>
       </c>
-      <c r="M4" s="21" t="n">
+      <c r="M4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="N4" s="21" t="n">
+      <c r="N4" s="26" t="n">
         <v>94708</v>
       </c>
-      <c r="O4" s="21" t="n">
+      <c r="O4" s="26" t="n">
         <v>142064</v>
       </c>
-      <c r="P4" s="21" t="n">
+      <c r="P4" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" s="22">
+      <c r="Q4" s="27">
         <f>O4-P4</f>
         <v/>
       </c>
-      <c r="R4" s="17" t="n">
+      <c r="R4" s="23" t="n">
         <v>19672</v>
       </c>
-      <c r="S4" s="17" t="n">
+      <c r="S4" s="23" t="n">
         <v>16722</v>
       </c>
-      <c r="T4" s="17" t="n">
+      <c r="T4" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U4" s="17" t="n">
+      <c r="U4" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="V4" s="22" t="inlineStr">
+      <c r="V4" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3458,61 +3563,61 @@
           <t>3-region</t>
         </is>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="21" t="n">
+      <c r="F5" s="26" t="n">
         <v>42492</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="26" t="n">
         <v>12292</v>
       </c>
-      <c r="H5" s="22">
+      <c r="H5" s="27">
         <f>F5-G5</f>
         <v/>
       </c>
-      <c r="I5" s="21" t="n">
+      <c r="I5" s="26" t="n">
         <v>63738</v>
       </c>
-      <c r="J5" s="21" t="n">
+      <c r="J5" s="26" t="n">
         <v>12292</v>
       </c>
-      <c r="K5" s="22">
+      <c r="K5" s="27">
         <f>I5-J5</f>
         <v/>
       </c>
-      <c r="L5" s="21" t="n">
+      <c r="L5" s="26" t="n">
         <v>94710</v>
       </c>
-      <c r="M5" s="21" t="n">
+      <c r="M5" s="26" t="n">
         <v>27398</v>
       </c>
-      <c r="N5" s="21" t="n">
+      <c r="N5" s="26" t="n">
         <v>67312</v>
       </c>
-      <c r="O5" s="21" t="n">
+      <c r="O5" s="26" t="n">
         <v>142064</v>
       </c>
-      <c r="P5" s="21" t="n">
+      <c r="P5" s="26" t="n">
         <v>27398</v>
       </c>
-      <c r="Q5" s="22">
+      <c r="Q5" s="27">
         <f>O5-P5</f>
         <v/>
       </c>
-      <c r="R5" s="17" t="n">
+      <c r="R5" s="23" t="n">
         <v>19672</v>
       </c>
-      <c r="S5" s="17" t="n">
+      <c r="S5" s="23" t="n">
         <v>16722</v>
       </c>
-      <c r="T5" s="17" t="n">
+      <c r="T5" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U5" s="17" t="n">
+      <c r="U5" s="23" t="n">
         <v>65</v>
       </c>
-      <c r="V5" s="22" t="inlineStr">
+      <c r="V5" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3539,61 +3644,61 @@
           <t>3-region</t>
         </is>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="26" t="n">
         <v>42492</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="26" t="n">
         <v>2326</v>
       </c>
-      <c r="H6" s="22">
+      <c r="H6" s="27">
         <f>F6-G6</f>
         <v/>
       </c>
-      <c r="I6" s="21" t="n">
+      <c r="I6" s="26" t="n">
         <v>63738</v>
       </c>
-      <c r="J6" s="21" t="n">
+      <c r="J6" s="26" t="n">
         <v>2326</v>
       </c>
-      <c r="K6" s="22">
+      <c r="K6" s="27">
         <f>I6-J6</f>
         <v/>
       </c>
-      <c r="L6" s="21" t="n">
+      <c r="L6" s="26" t="n">
         <v>94710</v>
       </c>
-      <c r="M6" s="21" t="n">
+      <c r="M6" s="26" t="n">
         <v>5186</v>
       </c>
-      <c r="N6" s="21" t="n">
+      <c r="N6" s="26" t="n">
         <v>89524</v>
       </c>
-      <c r="O6" s="21" t="n">
+      <c r="O6" s="26" t="n">
         <v>142064</v>
       </c>
-      <c r="P6" s="21" t="n">
+      <c r="P6" s="26" t="n">
         <v>5186</v>
       </c>
-      <c r="Q6" s="22">
+      <c r="Q6" s="27">
         <f>O6-P6</f>
         <v/>
       </c>
-      <c r="R6" s="17" t="n">
+      <c r="R6" s="23" t="n">
         <v>19672</v>
       </c>
-      <c r="S6" s="17" t="n">
+      <c r="S6" s="23" t="n">
         <v>16722</v>
       </c>
-      <c r="T6" s="17" t="n">
+      <c r="T6" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U6" s="17" t="n">
+      <c r="U6" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="V6" s="22" t="inlineStr">
+      <c r="V6" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3620,61 +3725,61 @@
           <t>3-region</t>
         </is>
       </c>
-      <c r="E7" s="17" t="n">
+      <c r="E7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="26" t="n">
         <v>154178</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="26" t="n">
         <v>142756</v>
       </c>
-      <c r="H7" s="22">
+      <c r="H7" s="27">
         <f>F7-G7</f>
         <v/>
       </c>
-      <c r="I7" s="21" t="n">
+      <c r="I7" s="26" t="n">
         <v>231266</v>
       </c>
-      <c r="J7" s="21" t="n">
+      <c r="J7" s="26" t="n">
         <v>142756</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="27">
         <f>I7-J7</f>
         <v/>
       </c>
-      <c r="L7" s="21" t="n">
+      <c r="L7" s="26" t="n">
         <v>343646</v>
       </c>
-      <c r="M7" s="21" t="n">
+      <c r="M7" s="26" t="n">
         <v>318190</v>
       </c>
-      <c r="N7" s="21" t="n">
+      <c r="N7" s="26" t="n">
         <v>25456</v>
       </c>
-      <c r="O7" s="21" t="n">
+      <c r="O7" s="26" t="n">
         <v>515468</v>
       </c>
-      <c r="P7" s="21" t="n">
+      <c r="P7" s="26" t="n">
         <v>318190</v>
       </c>
-      <c r="Q7" s="22">
+      <c r="Q7" s="27">
         <f>O7-P7</f>
         <v/>
       </c>
-      <c r="R7" s="17" t="n">
+      <c r="R7" s="23" t="n">
         <v>19672</v>
       </c>
-      <c r="S7" s="17" t="n">
+      <c r="S7" s="23" t="n">
         <v>16722</v>
       </c>
-      <c r="T7" s="17" t="n">
+      <c r="T7" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U7" s="17" t="n">
+      <c r="U7" s="23" t="n">
         <v>150</v>
       </c>
-      <c r="V7" s="22" t="inlineStr">
+      <c r="V7" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3701,61 +3806,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E8" s="17" t="n">
+      <c r="E8" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="26" t="n">
         <v>13334</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="26" t="n">
         <v>628</v>
       </c>
-      <c r="H8" s="22">
+      <c r="H8" s="27">
         <f>F8-G8</f>
         <v/>
       </c>
-      <c r="I8" s="21" t="n">
+      <c r="I8" s="26" t="n">
         <v>20002</v>
       </c>
-      <c r="J8" s="21" t="n">
+      <c r="J8" s="26" t="n">
         <v>628</v>
       </c>
-      <c r="K8" s="22">
+      <c r="K8" s="27">
         <f>I8-J8</f>
         <v/>
       </c>
-      <c r="L8" s="21" t="n">
+      <c r="L8" s="26" t="n">
         <v>40456</v>
       </c>
-      <c r="M8" s="21" t="n">
+      <c r="M8" s="26" t="n">
         <v>1902</v>
       </c>
-      <c r="N8" s="21" t="n">
+      <c r="N8" s="26" t="n">
         <v>38554</v>
       </c>
-      <c r="O8" s="21" t="n">
+      <c r="O8" s="26" t="n">
         <v>60684</v>
       </c>
-      <c r="P8" s="21" t="n">
+      <c r="P8" s="26" t="n">
         <v>1902</v>
       </c>
-      <c r="Q8" s="22">
+      <c r="Q8" s="27">
         <f>O8-P8</f>
         <v/>
       </c>
-      <c r="R8" s="17" t="n">
+      <c r="R8" s="23" t="n">
         <v>6174</v>
       </c>
-      <c r="S8" s="17" t="n">
+      <c r="S8" s="23" t="n">
         <v>5248</v>
       </c>
-      <c r="T8" s="17" t="n">
+      <c r="T8" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U8" s="17" t="n">
+      <c r="U8" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="V8" s="22" t="inlineStr">
+      <c r="V8" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3782,61 +3887,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E9" s="17" t="n">
+      <c r="E9" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="21" t="n">
+      <c r="F9" s="26" t="n">
         <v>13334</v>
       </c>
-      <c r="G9" s="21" t="n">
+      <c r="G9" s="26" t="n">
         <v>842</v>
       </c>
-      <c r="H9" s="22">
+      <c r="H9" s="27">
         <f>F9-G9</f>
         <v/>
       </c>
-      <c r="I9" s="21" t="n">
+      <c r="I9" s="26" t="n">
         <v>20002</v>
       </c>
-      <c r="J9" s="21" t="n">
+      <c r="J9" s="26" t="n">
         <v>842</v>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="27">
         <f>I9-J9</f>
         <v/>
       </c>
-      <c r="L9" s="21" t="n">
+      <c r="L9" s="26" t="n">
         <v>40456</v>
       </c>
-      <c r="M9" s="21" t="n">
+      <c r="M9" s="26" t="n">
         <v>2552</v>
       </c>
-      <c r="N9" s="21" t="n">
+      <c r="N9" s="26" t="n">
         <v>37904</v>
       </c>
-      <c r="O9" s="21" t="n">
+      <c r="O9" s="26" t="n">
         <v>60684</v>
       </c>
-      <c r="P9" s="21" t="n">
+      <c r="P9" s="26" t="n">
         <v>2552</v>
       </c>
-      <c r="Q9" s="22">
+      <c r="Q9" s="27">
         <f>O9-P9</f>
         <v/>
       </c>
-      <c r="R9" s="17" t="n">
+      <c r="R9" s="23" t="n">
         <v>6174</v>
       </c>
-      <c r="S9" s="17" t="n">
+      <c r="S9" s="23" t="n">
         <v>5248</v>
       </c>
-      <c r="T9" s="17" t="n">
+      <c r="T9" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U9" s="17" t="n">
+      <c r="U9" s="23" t="n">
         <v>13</v>
       </c>
-      <c r="V9" s="22" t="inlineStr">
+      <c r="V9" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3863,61 +3968,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E10" s="17" t="n">
+      <c r="E10" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="21" t="n">
+      <c r="F10" s="26" t="n">
         <v>13334</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="26" t="n">
         <v>3072</v>
       </c>
-      <c r="H10" s="22">
+      <c r="H10" s="27">
         <f>F10-G10</f>
         <v/>
       </c>
-      <c r="I10" s="21" t="n">
+      <c r="I10" s="26" t="n">
         <v>20002</v>
       </c>
-      <c r="J10" s="21" t="n">
+      <c r="J10" s="26" t="n">
         <v>3072</v>
       </c>
-      <c r="K10" s="22">
+      <c r="K10" s="27">
         <f>I10-J10</f>
         <v/>
       </c>
-      <c r="L10" s="21" t="n">
+      <c r="L10" s="26" t="n">
         <v>40456</v>
       </c>
-      <c r="M10" s="21" t="n">
+      <c r="M10" s="26" t="n">
         <v>9322</v>
       </c>
-      <c r="N10" s="21" t="n">
+      <c r="N10" s="26" t="n">
         <v>31134</v>
       </c>
-      <c r="O10" s="21" t="n">
+      <c r="O10" s="26" t="n">
         <v>60684</v>
       </c>
-      <c r="P10" s="21" t="n">
+      <c r="P10" s="26" t="n">
         <v>9322</v>
       </c>
-      <c r="Q10" s="22">
+      <c r="Q10" s="27">
         <f>O10-P10</f>
         <v/>
       </c>
-      <c r="R10" s="17" t="n">
+      <c r="R10" s="23" t="n">
         <v>6174</v>
       </c>
-      <c r="S10" s="17" t="n">
+      <c r="S10" s="23" t="n">
         <v>5248</v>
       </c>
-      <c r="T10" s="17" t="n">
+      <c r="T10" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U10" s="17" t="n">
+      <c r="U10" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="V10" s="22" t="inlineStr">
+      <c r="V10" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3944,61 +4049,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E11" s="17" t="n">
+      <c r="E11" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="26" t="n">
         <v>48434</v>
       </c>
-      <c r="G11" s="21" t="n">
+      <c r="G11" s="26" t="n">
         <v>44846</v>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="27">
         <f>F11-G11</f>
         <v/>
       </c>
-      <c r="I11" s="21" t="n">
+      <c r="I11" s="26" t="n">
         <v>72650</v>
       </c>
-      <c r="J11" s="21" t="n">
+      <c r="J11" s="26" t="n">
         <v>44846</v>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="27">
         <f>I11-J11</f>
         <v/>
       </c>
-      <c r="L11" s="21" t="n">
+      <c r="L11" s="26" t="n">
         <v>146950</v>
       </c>
-      <c r="M11" s="21" t="n">
+      <c r="M11" s="26" t="n">
         <v>136064</v>
       </c>
-      <c r="N11" s="21" t="n">
+      <c r="N11" s="26" t="n">
         <v>10886</v>
       </c>
-      <c r="O11" s="21" t="n">
+      <c r="O11" s="26" t="n">
         <v>220424</v>
       </c>
-      <c r="P11" s="21" t="n">
+      <c r="P11" s="26" t="n">
         <v>136064</v>
       </c>
-      <c r="Q11" s="22">
+      <c r="Q11" s="27">
         <f>O11-P11</f>
         <v/>
       </c>
-      <c r="R11" s="17" t="n">
+      <c r="R11" s="23" t="n">
         <v>6174</v>
       </c>
-      <c r="S11" s="17" t="n">
+      <c r="S11" s="23" t="n">
         <v>5248</v>
       </c>
-      <c r="T11" s="17" t="n">
+      <c r="T11" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U11" s="17" t="n">
+      <c r="U11" s="23" t="n">
         <v>69</v>
       </c>
-      <c r="V11" s="22" t="inlineStr">
+      <c r="V11" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4025,61 +4130,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E12" s="17" t="n">
+      <c r="E12" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="21" t="n">
+      <c r="F12" s="26" t="n">
         <v>9518</v>
       </c>
-      <c r="G12" s="21" t="n">
+      <c r="G12" s="26" t="n">
         <v>8812</v>
       </c>
-      <c r="H12" s="22">
+      <c r="H12" s="27">
         <f>F12-G12</f>
         <v/>
       </c>
-      <c r="I12" s="21" t="n">
+      <c r="I12" s="26" t="n">
         <v>14276</v>
       </c>
-      <c r="J12" s="21" t="n">
+      <c r="J12" s="26" t="n">
         <v>8812</v>
       </c>
-      <c r="K12" s="22">
+      <c r="K12" s="27">
         <f>I12-J12</f>
         <v/>
       </c>
-      <c r="L12" s="21" t="n">
+      <c r="L12" s="26" t="n">
         <v>17958</v>
       </c>
-      <c r="M12" s="21" t="n">
+      <c r="M12" s="26" t="n">
         <v>16628</v>
       </c>
-      <c r="N12" s="21" t="n">
+      <c r="N12" s="26" t="n">
         <v>1330</v>
       </c>
-      <c r="O12" s="21" t="n">
+      <c r="O12" s="26" t="n">
         <v>26936</v>
       </c>
-      <c r="P12" s="21" t="n">
+      <c r="P12" s="26" t="n">
         <v>16628</v>
       </c>
-      <c r="Q12" s="22">
+      <c r="Q12" s="27">
         <f>O12-P12</f>
         <v/>
       </c>
-      <c r="R12" s="17" t="n">
+      <c r="R12" s="23" t="n">
         <v>2604</v>
       </c>
-      <c r="S12" s="17" t="n">
+      <c r="S12" s="23" t="n">
         <v>2214</v>
       </c>
-      <c r="T12" s="17" t="n">
+      <c r="T12" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U12" s="17" t="n">
+      <c r="U12" s="23" t="n">
         <v>34</v>
       </c>
-      <c r="V12" s="22" t="inlineStr">
+      <c r="V12" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4106,61 +4211,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E13" s="17" t="n">
+      <c r="E13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="21" t="n">
+      <c r="F13" s="26" t="n">
         <v>5624</v>
       </c>
-      <c r="G13" s="21" t="n">
+      <c r="G13" s="26" t="n">
         <v>1602</v>
       </c>
-      <c r="H13" s="22">
+      <c r="H13" s="27">
         <f>F13-G13</f>
         <v/>
       </c>
-      <c r="I13" s="21" t="n">
+      <c r="I13" s="26" t="n">
         <v>8434</v>
       </c>
-      <c r="J13" s="21" t="n">
+      <c r="J13" s="26" t="n">
         <v>1602</v>
       </c>
-      <c r="K13" s="22">
+      <c r="K13" s="27">
         <f>I13-J13</f>
         <v/>
       </c>
-      <c r="L13" s="21" t="n">
+      <c r="L13" s="26" t="n">
         <v>10610</v>
       </c>
-      <c r="M13" s="21" t="n">
+      <c r="M13" s="26" t="n">
         <v>3020</v>
       </c>
-      <c r="N13" s="21" t="n">
+      <c r="N13" s="26" t="n">
         <v>7590</v>
       </c>
-      <c r="O13" s="21" t="n">
+      <c r="O13" s="26" t="n">
         <v>15914</v>
       </c>
-      <c r="P13" s="21" t="n">
+      <c r="P13" s="26" t="n">
         <v>3020</v>
       </c>
-      <c r="Q13" s="22">
+      <c r="Q13" s="27">
         <f>O13-P13</f>
         <v/>
       </c>
-      <c r="R13" s="17" t="n">
+      <c r="R13" s="23" t="n">
         <v>2604</v>
       </c>
-      <c r="S13" s="17" t="n">
+      <c r="S13" s="23" t="n">
         <v>2214</v>
       </c>
-      <c r="T13" s="17" t="n">
+      <c r="T13" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U13" s="17" t="n">
+      <c r="U13" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="V13" s="22" t="inlineStr">
+      <c r="V13" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4187,61 +4292,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E14" s="17" t="n">
+      <c r="E14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="21" t="n">
+      <c r="F14" s="26" t="n">
         <v>12504</v>
       </c>
-      <c r="G14" s="21" t="n">
+      <c r="G14" s="26" t="n">
         <v>2956</v>
       </c>
-      <c r="H14" s="22">
+      <c r="H14" s="27">
         <f>F14-G14</f>
         <v/>
       </c>
-      <c r="I14" s="21" t="n">
+      <c r="I14" s="26" t="n">
         <v>18756</v>
       </c>
-      <c r="J14" s="21" t="n">
+      <c r="J14" s="26" t="n">
         <v>2956</v>
       </c>
-      <c r="K14" s="22">
+      <c r="K14" s="27">
         <f>I14-J14</f>
         <v/>
       </c>
-      <c r="L14" s="21" t="n">
+      <c r="L14" s="26" t="n">
         <v>13968</v>
       </c>
-      <c r="M14" s="21" t="n">
+      <c r="M14" s="26" t="n">
         <v>3302</v>
       </c>
-      <c r="N14" s="21" t="n">
+      <c r="N14" s="26" t="n">
         <v>10666</v>
       </c>
-      <c r="O14" s="21" t="n">
+      <c r="O14" s="26" t="n">
         <v>20952</v>
       </c>
-      <c r="P14" s="21" t="n">
+      <c r="P14" s="26" t="n">
         <v>3302</v>
       </c>
-      <c r="Q14" s="22">
+      <c r="Q14" s="27">
         <f>O14-P14</f>
         <v/>
       </c>
-      <c r="R14" s="17" t="n">
+      <c r="R14" s="23" t="n">
         <v>5790</v>
       </c>
-      <c r="S14" s="17" t="n">
+      <c r="S14" s="23" t="n">
         <v>4922</v>
       </c>
-      <c r="T14" s="17" t="n">
+      <c r="T14" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U14" s="17" t="n">
+      <c r="U14" s="23" t="n">
         <v>21</v>
       </c>
-      <c r="V14" s="22" t="inlineStr">
+      <c r="V14" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4268,61 +4373,61 @@
           <t>2-region</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n">
+      <c r="E15" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F15" s="26" t="n">
         <v>21816</v>
       </c>
-      <c r="G15" s="21" t="n">
+      <c r="G15" s="26" t="n">
         <v>20200</v>
       </c>
-      <c r="H15" s="22">
+      <c r="H15" s="27">
         <f>F15-G15</f>
         <v/>
       </c>
-      <c r="I15" s="21" t="n">
+      <c r="I15" s="26" t="n">
         <v>32722</v>
       </c>
-      <c r="J15" s="21" t="n">
+      <c r="J15" s="26" t="n">
         <v>20200</v>
       </c>
-      <c r="K15" s="22">
+      <c r="K15" s="27">
         <f>I15-J15</f>
         <v/>
       </c>
-      <c r="L15" s="21" t="n">
+      <c r="L15" s="26" t="n">
         <v>24370</v>
       </c>
-      <c r="M15" s="21" t="n">
+      <c r="M15" s="26" t="n">
         <v>22566</v>
       </c>
-      <c r="N15" s="21" t="n">
+      <c r="N15" s="26" t="n">
         <v>1804</v>
       </c>
-      <c r="O15" s="21" t="n">
+      <c r="O15" s="26" t="n">
         <v>36556</v>
       </c>
-      <c r="P15" s="21" t="n">
+      <c r="P15" s="26" t="n">
         <v>22566</v>
       </c>
-      <c r="Q15" s="22">
+      <c r="Q15" s="27">
         <f>O15-P15</f>
         <v/>
       </c>
-      <c r="R15" s="17" t="n">
+      <c r="R15" s="23" t="n">
         <v>5790</v>
       </c>
-      <c r="S15" s="17" t="n">
+      <c r="S15" s="23" t="n">
         <v>4922</v>
       </c>
-      <c r="T15" s="17" t="n">
+      <c r="T15" s="23" t="n">
         <v>0.6</v>
       </c>
-      <c r="U15" s="17" t="n">
+      <c r="U15" s="23" t="n">
         <v>43</v>
       </c>
-      <c r="V15" s="22" t="inlineStr">
+      <c r="V15" s="27" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4331,12 +4436,12 @@
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
         <is>
-          <t>saudicentral</t>
+          <t>saudiarbiaeast</t>
         </is>
       </c>
       <c r="B16" s="11" t="inlineStr">
         <is>
-          <t>Saudi Arabia Central</t>
+          <t>Saudi Arabia East</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -4349,61 +4454,61 @@
           <t>cross-geo</t>
         </is>
       </c>
-      <c r="E16" s="23" t="n">
+      <c r="E16" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="24" t="n">
+      <c r="F16" s="28" t="n">
         <v>1296</v>
       </c>
-      <c r="G16" s="24" t="n">
+      <c r="G16" s="28" t="n">
         <v>1200</v>
       </c>
-      <c r="H16" s="22">
+      <c r="H16" s="27">
         <f>F16-G16</f>
         <v/>
       </c>
-      <c r="I16" s="24" t="n">
+      <c r="I16" s="28" t="n">
         <v>1944</v>
       </c>
-      <c r="J16" s="24" t="n">
+      <c r="J16" s="28" t="n">
         <v>1200</v>
       </c>
-      <c r="K16" s="22">
+      <c r="K16" s="27">
         <f>I16-J16</f>
         <v/>
       </c>
-      <c r="L16" s="24" t="n">
+      <c r="L16" s="28" t="n">
         <v>1838</v>
       </c>
-      <c r="M16" s="24" t="n">
+      <c r="M16" s="28" t="n">
         <v>1700</v>
       </c>
-      <c r="N16" s="24" t="n">
+      <c r="N16" s="28" t="n">
         <v>138</v>
       </c>
-      <c r="O16" s="24" t="n">
+      <c r="O16" s="28" t="n">
         <v>2756</v>
       </c>
-      <c r="P16" s="24" t="n">
+      <c r="P16" s="28" t="n">
         <v>1700</v>
       </c>
-      <c r="Q16" s="22">
+      <c r="Q16" s="27">
         <f>O16-P16</f>
         <v/>
       </c>
-      <c r="R16" s="23" t="n">
+      <c r="R16" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="S16" s="23" t="n">
+      <c r="S16" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="T16" s="23" t="n">
+      <c r="T16" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="U16" s="23" t="n">
+      <c r="U16" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="V16" s="25" t="inlineStr">
+      <c r="V16" s="21" t="inlineStr">
         <is>
           <t>Restricted</t>
         </is>
@@ -4430,61 +4535,61 @@
           <t>cross-geo</t>
         </is>
       </c>
-      <c r="E17" s="23" t="n">
+      <c r="E17" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="24" t="n">
+      <c r="F17" s="28" t="n">
         <v>1296</v>
       </c>
-      <c r="G17" s="24" t="n">
+      <c r="G17" s="28" t="n">
         <v>1200</v>
       </c>
-      <c r="H17" s="22">
+      <c r="H17" s="27">
         <f>F17-G17</f>
         <v/>
       </c>
-      <c r="I17" s="24" t="n">
+      <c r="I17" s="28" t="n">
         <v>1944</v>
       </c>
-      <c r="J17" s="24" t="n">
+      <c r="J17" s="28" t="n">
         <v>1200</v>
       </c>
-      <c r="K17" s="22">
+      <c r="K17" s="27">
         <f>I17-J17</f>
         <v/>
       </c>
-      <c r="L17" s="24" t="n">
+      <c r="L17" s="28" t="n">
         <v>1838</v>
       </c>
-      <c r="M17" s="24" t="n">
+      <c r="M17" s="28" t="n">
         <v>1700</v>
       </c>
-      <c r="N17" s="24" t="n">
+      <c r="N17" s="28" t="n">
         <v>138</v>
       </c>
-      <c r="O17" s="24" t="n">
+      <c r="O17" s="28" t="n">
         <v>2756</v>
       </c>
-      <c r="P17" s="24" t="n">
+      <c r="P17" s="28" t="n">
         <v>1700</v>
       </c>
-      <c r="Q17" s="22">
+      <c r="Q17" s="27">
         <f>O17-P17</f>
         <v/>
       </c>
-      <c r="R17" s="23" t="n">
+      <c r="R17" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="S17" s="23" t="n">
+      <c r="S17" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="T17" s="23" t="n">
+      <c r="T17" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="U17" s="23" t="n">
+      <c r="U17" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="V17" s="25" t="inlineStr">
+      <c r="V17" s="21" t="inlineStr">
         <is>
           <t>Restricted</t>
         </is>
@@ -5355,7 +5460,7 @@
           <t>PS_Prod — Production Placement Score</t>
         </is>
       </c>
-      <c r="T1" s="26" t="inlineStr">
+      <c r="T1" s="29" t="inlineStr">
         <is>
           <t>PROD WINNER</t>
         </is>
@@ -5503,47 +5608,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="30">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!F4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="30">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="30">
         <f>IFERROR(Capacity_Usage!K4/Capacity_Usage!I4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="27">
+      <c r="J4" s="30">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="27">
+      <c r="K4" s="30">
         <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="27">
+      <c r="L4" s="30">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="27">
+      <c r="M4" s="30">
         <f>IFERROR(Capacity_Usage!T4,0)</f>
         <v/>
       </c>
-      <c r="N4" s="27">
+      <c r="N4" s="30">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="27">
+      <c r="O4" s="30">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="27">
+      <c r="P4" s="30">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="30">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -5560,7 +5665,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U4" s="28">
+      <c r="U4" s="31">
         <f>IF(Setup!$B$8&lt;&gt;"",INDEX(Q4:Q17,MATCH(Setup!$B$8,A4:A17,0)),IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -5590,47 +5695,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="30">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!F5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="30">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="27">
+      <c r="I5" s="30">
         <f>IFERROR(Capacity_Usage!K5/Capacity_Usage!I5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="27">
+      <c r="J5" s="30">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="27">
+      <c r="K5" s="30">
         <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="27">
+      <c r="L5" s="30">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="27">
+      <c r="M5" s="30">
         <f>IFERROR(Capacity_Usage!T5,0)</f>
         <v/>
       </c>
-      <c r="N5" s="27">
+      <c r="N5" s="30">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="27">
+      <c r="O5" s="30">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="27">
+      <c r="P5" s="30">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="30">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -5668,47 +5773,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="30">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!F6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="30">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="30">
         <f>IFERROR(Capacity_Usage!K6/Capacity_Usage!I6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="30">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="27">
+      <c r="K6" s="30">
         <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="27">
+      <c r="L6" s="30">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="30">
         <f>IFERROR(Capacity_Usage!T6,0)</f>
         <v/>
       </c>
-      <c r="N6" s="27">
+      <c r="N6" s="30">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="27">
+      <c r="O6" s="30">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="27">
+      <c r="P6" s="30">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="27">
+      <c r="Q6" s="30">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -5746,47 +5851,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="30">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!F7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="30">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="30">
         <f>IFERROR(Capacity_Usage!K7/Capacity_Usage!I7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="30">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="27">
+      <c r="K7" s="30">
         <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
         <v/>
       </c>
-      <c r="L7" s="27">
+      <c r="L7" s="30">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="27">
+      <c r="M7" s="30">
         <f>IFERROR(Capacity_Usage!T7,0)</f>
         <v/>
       </c>
-      <c r="N7" s="27">
+      <c r="N7" s="30">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="27">
+      <c r="O7" s="30">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="27">
+      <c r="P7" s="30">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="27">
+      <c r="Q7" s="30">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -5824,47 +5929,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="30">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!F8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="30">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="27">
+      <c r="I8" s="30">
         <f>IFERROR(Capacity_Usage!K8/Capacity_Usage!I8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="30">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="27">
+      <c r="K8" s="30">
         <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
         <v/>
       </c>
-      <c r="L8" s="27">
+      <c r="L8" s="30">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="27">
+      <c r="M8" s="30">
         <f>IFERROR(Capacity_Usage!T8,0)</f>
         <v/>
       </c>
-      <c r="N8" s="27">
+      <c r="N8" s="30">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="27">
+      <c r="O8" s="30">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="27">
+      <c r="P8" s="30">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="30">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -5902,47 +6007,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="30">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!F9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="30">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="30">
         <f>IFERROR(Capacity_Usage!K9/Capacity_Usage!I9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="30">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="27">
+      <c r="K9" s="30">
         <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
         <v/>
       </c>
-      <c r="L9" s="27">
+      <c r="L9" s="30">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="27">
+      <c r="M9" s="30">
         <f>IFERROR(Capacity_Usage!T9,0)</f>
         <v/>
       </c>
-      <c r="N9" s="27">
+      <c r="N9" s="30">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="27">
+      <c r="O9" s="30">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="27">
+      <c r="P9" s="30">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="30">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -5980,47 +6085,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="30">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!F10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="30">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="27">
+      <c r="I10" s="30">
         <f>IFERROR(Capacity_Usage!K10/Capacity_Usage!I10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="27">
+      <c r="J10" s="30">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="27">
+      <c r="K10" s="30">
         <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
         <v/>
       </c>
-      <c r="L10" s="27">
+      <c r="L10" s="30">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="27">
+      <c r="M10" s="30">
         <f>IFERROR(Capacity_Usage!T10,0)</f>
         <v/>
       </c>
-      <c r="N10" s="27">
+      <c r="N10" s="30">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="27">
+      <c r="O10" s="30">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="27">
+      <c r="P10" s="30">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="30">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -6058,47 +6163,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="30">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!F11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="30">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="27">
+      <c r="I11" s="30">
         <f>IFERROR(Capacity_Usage!K11/Capacity_Usage!I11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="27">
+      <c r="J11" s="30">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="27">
+      <c r="K11" s="30">
         <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="27">
+      <c r="L11" s="30">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="27">
+      <c r="M11" s="30">
         <f>IFERROR(Capacity_Usage!T11,0)</f>
         <v/>
       </c>
-      <c r="N11" s="27">
+      <c r="N11" s="30">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="27">
+      <c r="O11" s="30">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="30">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="30">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -6136,47 +6241,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="30">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!F12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="30">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="30">
         <f>IFERROR(Capacity_Usage!K12/Capacity_Usage!I12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="30">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="27">
+      <c r="K12" s="30">
         <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
         <v/>
       </c>
-      <c r="L12" s="27">
+      <c r="L12" s="30">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="27">
+      <c r="M12" s="30">
         <f>IFERROR(Capacity_Usage!T12,0)</f>
         <v/>
       </c>
-      <c r="N12" s="27">
+      <c r="N12" s="30">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="27">
+      <c r="O12" s="30">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="27">
+      <c r="P12" s="30">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="27">
+      <c r="Q12" s="30">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -6214,47 +6319,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="30">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!F13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="30">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="27">
+      <c r="I13" s="30">
         <f>IFERROR(Capacity_Usage!K13/Capacity_Usage!I13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="27">
+      <c r="J13" s="30">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="27">
+      <c r="K13" s="30">
         <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
         <v/>
       </c>
-      <c r="L13" s="27">
+      <c r="L13" s="30">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="27">
+      <c r="M13" s="30">
         <f>IFERROR(Capacity_Usage!T13,0)</f>
         <v/>
       </c>
-      <c r="N13" s="27">
+      <c r="N13" s="30">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="27">
+      <c r="O13" s="30">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="27">
+      <c r="P13" s="30">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="27">
+      <c r="Q13" s="30">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -6292,47 +6397,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="30">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!F14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="30">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="27">
+      <c r="I14" s="30">
         <f>IFERROR(Capacity_Usage!K14/Capacity_Usage!I14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="27">
+      <c r="J14" s="30">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="27">
+      <c r="K14" s="30">
         <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
         <v/>
       </c>
-      <c r="L14" s="27">
+      <c r="L14" s="30">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="27">
+      <c r="M14" s="30">
         <f>IFERROR(Capacity_Usage!T14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="30">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="27">
+      <c r="O14" s="30">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="27">
+      <c r="P14" s="30">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="27">
+      <c r="Q14" s="30">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -6370,47 +6475,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G15" s="27">
+      <c r="G15" s="30">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!F15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="30">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="27">
+      <c r="I15" s="30">
         <f>IFERROR(Capacity_Usage!K15/Capacity_Usage!I15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="27">
+      <c r="J15" s="30">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="27">
+      <c r="K15" s="30">
         <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
         <v/>
       </c>
-      <c r="L15" s="27">
+      <c r="L15" s="30">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="27">
+      <c r="M15" s="30">
         <f>IFERROR(Capacity_Usage!T15,0)</f>
         <v/>
       </c>
-      <c r="N15" s="27">
+      <c r="N15" s="30">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="27">
+      <c r="O15" s="30">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="27">
+      <c r="P15" s="30">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="27">
+      <c r="Q15" s="30">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -6448,47 +6553,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G16" s="27">
+      <c r="G16" s="30">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!F16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="30">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="27">
+      <c r="I16" s="30">
         <f>IFERROR(Capacity_Usage!K16/Capacity_Usage!I16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="27">
+      <c r="J16" s="30">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="27">
+      <c r="K16" s="30">
         <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
         <v/>
       </c>
-      <c r="L16" s="27">
+      <c r="L16" s="30">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="27">
+      <c r="M16" s="30">
         <f>IFERROR(Capacity_Usage!T16,0)</f>
         <v/>
       </c>
-      <c r="N16" s="27">
+      <c r="N16" s="30">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="27">
+      <c r="O16" s="30">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="27">
+      <c r="P16" s="30">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="27">
+      <c r="Q16" s="30">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -6526,47 +6631,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G17" s="27">
+      <c r="G17" s="30">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!F17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="30">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="27">
+      <c r="I17" s="30">
         <f>IFERROR(Capacity_Usage!K17/Capacity_Usage!I17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="27">
+      <c r="J17" s="30">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="27">
+      <c r="K17" s="30">
         <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
         <v/>
       </c>
-      <c r="L17" s="27">
+      <c r="L17" s="30">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="27">
+      <c r="M17" s="30">
         <f>IFERROR(Capacity_Usage!T17,0)</f>
         <v/>
       </c>
-      <c r="N17" s="27">
+      <c r="N17" s="30">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="27">
+      <c r="O17" s="30">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="27">
+      <c r="P17" s="30">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="27">
+      <c r="Q17" s="30">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>
@@ -6623,7 +6728,7 @@
           <t>PS_NonProd — CVAL Placement Score  (δ duplicates α — known design gap)</t>
         </is>
       </c>
-      <c r="T1" s="26" t="inlineStr">
+      <c r="T1" s="29" t="inlineStr">
         <is>
           <t>CVAL WINNER</t>
         </is>
@@ -6741,7 +6846,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U3" s="28">
+      <c r="U3" s="31">
         <f>IF(Setup!$B$3="Middle East",Scoring_Prod!$U$4,IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -6771,47 +6876,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="30">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!L4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="30">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="30">
         <f>IFERROR(Capacity_Usage!Q4/Capacity_Usage!O4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="27">
+      <c r="J4" s="30">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="27">
+      <c r="K4" s="30">
         <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="27">
+      <c r="L4" s="30">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="27">
+      <c r="M4" s="30">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!L4,0)</f>
         <v/>
       </c>
-      <c r="N4" s="27">
+      <c r="N4" s="30">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="27">
+      <c r="O4" s="30">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="27">
+      <c r="P4" s="30">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="30">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -6849,47 +6954,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="30">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!L5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="30">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="27">
+      <c r="I5" s="30">
         <f>IFERROR(Capacity_Usage!Q5/Capacity_Usage!O5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="27">
+      <c r="J5" s="30">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="27">
+      <c r="K5" s="30">
         <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="27">
+      <c r="L5" s="30">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="27">
+      <c r="M5" s="30">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!L5,0)</f>
         <v/>
       </c>
-      <c r="N5" s="27">
+      <c r="N5" s="30">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="27">
+      <c r="O5" s="30">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="27">
+      <c r="P5" s="30">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="30">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -6927,47 +7032,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="30">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!L6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="30">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="30">
         <f>IFERROR(Capacity_Usage!Q6/Capacity_Usage!O6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="30">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="27">
+      <c r="K6" s="30">
         <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="27">
+      <c r="L6" s="30">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="30">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!L6,0)</f>
         <v/>
       </c>
-      <c r="N6" s="27">
+      <c r="N6" s="30">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="27">
+      <c r="O6" s="30">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="27">
+      <c r="P6" s="30">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="27">
+      <c r="Q6" s="30">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -7005,47 +7110,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="30">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!L7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="30">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="30">
         <f>IFERROR(Capacity_Usage!Q7/Capacity_Usage!O7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="30">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="27">
+      <c r="K7" s="30">
         <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
         <v/>
       </c>
-      <c r="L7" s="27">
+      <c r="L7" s="30">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="27">
+      <c r="M7" s="30">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!L7,0)</f>
         <v/>
       </c>
-      <c r="N7" s="27">
+      <c r="N7" s="30">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="27">
+      <c r="O7" s="30">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="27">
+      <c r="P7" s="30">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="27">
+      <c r="Q7" s="30">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -7083,47 +7188,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="30">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!L8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="30">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="27">
+      <c r="I8" s="30">
         <f>IFERROR(Capacity_Usage!Q8/Capacity_Usage!O8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="30">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="27">
+      <c r="K8" s="30">
         <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
         <v/>
       </c>
-      <c r="L8" s="27">
+      <c r="L8" s="30">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="27">
+      <c r="M8" s="30">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!L8,0)</f>
         <v/>
       </c>
-      <c r="N8" s="27">
+      <c r="N8" s="30">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="27">
+      <c r="O8" s="30">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="27">
+      <c r="P8" s="30">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="30">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -7161,47 +7266,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="30">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!L9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="30">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="30">
         <f>IFERROR(Capacity_Usage!Q9/Capacity_Usage!O9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="30">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="27">
+      <c r="K9" s="30">
         <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
         <v/>
       </c>
-      <c r="L9" s="27">
+      <c r="L9" s="30">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="27">
+      <c r="M9" s="30">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!L9,0)</f>
         <v/>
       </c>
-      <c r="N9" s="27">
+      <c r="N9" s="30">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="27">
+      <c r="O9" s="30">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="27">
+      <c r="P9" s="30">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="30">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -7239,47 +7344,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="30">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!L10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="30">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="27">
+      <c r="I10" s="30">
         <f>IFERROR(Capacity_Usage!Q10/Capacity_Usage!O10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="27">
+      <c r="J10" s="30">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="27">
+      <c r="K10" s="30">
         <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
         <v/>
       </c>
-      <c r="L10" s="27">
+      <c r="L10" s="30">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="27">
+      <c r="M10" s="30">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!L10,0)</f>
         <v/>
       </c>
-      <c r="N10" s="27">
+      <c r="N10" s="30">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="27">
+      <c r="O10" s="30">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="27">
+      <c r="P10" s="30">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="30">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -7317,47 +7422,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="30">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!L11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="30">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="27">
+      <c r="I11" s="30">
         <f>IFERROR(Capacity_Usage!Q11/Capacity_Usage!O11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="27">
+      <c r="J11" s="30">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="27">
+      <c r="K11" s="30">
         <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="27">
+      <c r="L11" s="30">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="27">
+      <c r="M11" s="30">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!L11,0)</f>
         <v/>
       </c>
-      <c r="N11" s="27">
+      <c r="N11" s="30">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="27">
+      <c r="O11" s="30">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="30">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="30">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -7395,47 +7500,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="30">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!L12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="30">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="30">
         <f>IFERROR(Capacity_Usage!Q12/Capacity_Usage!O12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="30">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="27">
+      <c r="K12" s="30">
         <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
         <v/>
       </c>
-      <c r="L12" s="27">
+      <c r="L12" s="30">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="27">
+      <c r="M12" s="30">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!L12,0)</f>
         <v/>
       </c>
-      <c r="N12" s="27">
+      <c r="N12" s="30">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="27">
+      <c r="O12" s="30">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="27">
+      <c r="P12" s="30">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="27">
+      <c r="Q12" s="30">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -7473,47 +7578,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="30">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!L13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="30">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="27">
+      <c r="I13" s="30">
         <f>IFERROR(Capacity_Usage!Q13/Capacity_Usage!O13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="27">
+      <c r="J13" s="30">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="27">
+      <c r="K13" s="30">
         <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
         <v/>
       </c>
-      <c r="L13" s="27">
+      <c r="L13" s="30">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="27">
+      <c r="M13" s="30">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!L13,0)</f>
         <v/>
       </c>
-      <c r="N13" s="27">
+      <c r="N13" s="30">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="27">
+      <c r="O13" s="30">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="27">
+      <c r="P13" s="30">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="27">
+      <c r="Q13" s="30">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -7551,47 +7656,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="30">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!L14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="30">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="27">
+      <c r="I14" s="30">
         <f>IFERROR(Capacity_Usage!Q14/Capacity_Usage!O14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="27">
+      <c r="J14" s="30">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="27">
+      <c r="K14" s="30">
         <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
         <v/>
       </c>
-      <c r="L14" s="27">
+      <c r="L14" s="30">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="27">
+      <c r="M14" s="30">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!L14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="30">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="27">
+      <c r="O14" s="30">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="27">
+      <c r="P14" s="30">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="27">
+      <c r="Q14" s="30">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -7629,47 +7734,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G15" s="27">
+      <c r="G15" s="30">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!L15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="30">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="27">
+      <c r="I15" s="30">
         <f>IFERROR(Capacity_Usage!Q15/Capacity_Usage!O15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="27">
+      <c r="J15" s="30">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="27">
+      <c r="K15" s="30">
         <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
         <v/>
       </c>
-      <c r="L15" s="27">
+      <c r="L15" s="30">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="27">
+      <c r="M15" s="30">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!L15,0)</f>
         <v/>
       </c>
-      <c r="N15" s="27">
+      <c r="N15" s="30">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="27">
+      <c r="O15" s="30">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="27">
+      <c r="P15" s="30">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="27">
+      <c r="Q15" s="30">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -7707,47 +7812,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G16" s="27">
+      <c r="G16" s="30">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!L16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="30">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="27">
+      <c r="I16" s="30">
         <f>IFERROR(Capacity_Usage!Q16/Capacity_Usage!O16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="27">
+      <c r="J16" s="30">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="27">
+      <c r="K16" s="30">
         <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
         <v/>
       </c>
-      <c r="L16" s="27">
+      <c r="L16" s="30">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="27">
+      <c r="M16" s="30">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!L16,0)</f>
         <v/>
       </c>
-      <c r="N16" s="27">
+      <c r="N16" s="30">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="27">
+      <c r="O16" s="30">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="27">
+      <c r="P16" s="30">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="27">
+      <c r="Q16" s="30">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -7785,47 +7890,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G17" s="27">
+      <c r="G17" s="30">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!L17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="30">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="27">
+      <c r="I17" s="30">
         <f>IFERROR(Capacity_Usage!Q17/Capacity_Usage!O17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="27">
+      <c r="J17" s="30">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="27">
+      <c r="K17" s="30">
         <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
         <v/>
       </c>
-      <c r="L17" s="27">
+      <c r="L17" s="30">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="27">
+      <c r="M17" s="30">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!L17,0)</f>
         <v/>
       </c>
-      <c r="N17" s="27">
+      <c r="N17" s="30">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="27">
+      <c r="O17" s="30">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="27">
+      <c r="P17" s="30">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="27">
+      <c r="Q17" s="30">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>
@@ -7881,7 +7986,7 @@
           <t>PS_DR — DR Placement Score  (Middle East scores EU regions cross-geo)</t>
         </is>
       </c>
-      <c r="T1" s="26" t="inlineStr">
+      <c r="T1" s="29" t="inlineStr">
         <is>
           <t>DR WINNER</t>
         </is>
@@ -7999,7 +8104,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U3" s="28">
+      <c r="U3" s="31">
         <f>IF(Setup!$B$10="2-region",Scoring_CVAL!$U$3,IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -8029,47 +8134,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G4" s="27">
+      <c r="G4" s="30">
         <f>IFERROR(Capacity_Usage!S4/Capacity_Usage!R4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="30">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="27">
+      <c r="I4" s="30">
         <f>IFERROR(Capacity_Usage!Q4/Capacity_Usage!O4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="27">
+      <c r="J4" s="30">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="27">
+      <c r="K4" s="30">
         <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="27">
+      <c r="L4" s="30">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="27">
+      <c r="M4" s="30">
         <f>IFERROR(Capacity_Usage!T4/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N4" s="27">
+      <c r="N4" s="30">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="27">
+      <c r="O4" s="30">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="27">
+      <c r="P4" s="30">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="30">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -8107,47 +8212,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G5" s="27">
+      <c r="G5" s="30">
         <f>IFERROR(Capacity_Usage!S5/Capacity_Usage!R5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="30">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="27">
+      <c r="I5" s="30">
         <f>IFERROR(Capacity_Usage!Q5/Capacity_Usage!O5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="27">
+      <c r="J5" s="30">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="27">
+      <c r="K5" s="30">
         <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="27">
+      <c r="L5" s="30">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="27">
+      <c r="M5" s="30">
         <f>IFERROR(Capacity_Usage!T5/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N5" s="27">
+      <c r="N5" s="30">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="27">
+      <c r="O5" s="30">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="27">
+      <c r="P5" s="30">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="30">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -8185,47 +8290,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G6" s="27">
+      <c r="G6" s="30">
         <f>IFERROR(Capacity_Usage!S6/Capacity_Usage!R6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="30">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="27">
+      <c r="I6" s="30">
         <f>IFERROR(Capacity_Usage!Q6/Capacity_Usage!O6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="27">
+      <c r="J6" s="30">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="27">
+      <c r="K6" s="30">
         <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="27">
+      <c r="L6" s="30">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="30">
         <f>IFERROR(Capacity_Usage!T6/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N6" s="27">
+      <c r="N6" s="30">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="27">
+      <c r="O6" s="30">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="27">
+      <c r="P6" s="30">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="27">
+      <c r="Q6" s="30">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -8263,47 +8368,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G7" s="27">
+      <c r="G7" s="30">
         <f>IFERROR(Capacity_Usage!S7/Capacity_Usage!R7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="30">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="30">
         <f>IFERROR(Capacity_Usage!Q7/Capacity_Usage!O7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="30">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="27">
+      <c r="K7" s="30">
         <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
         <v/>
       </c>
-      <c r="L7" s="27">
+      <c r="L7" s="30">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="27">
+      <c r="M7" s="30">
         <f>IFERROR(Capacity_Usage!T7/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N7" s="27">
+      <c r="N7" s="30">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="27">
+      <c r="O7" s="30">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="27">
+      <c r="P7" s="30">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="27">
+      <c r="Q7" s="30">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -8341,47 +8446,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G8" s="27">
+      <c r="G8" s="30">
         <f>IFERROR(Capacity_Usage!S8/Capacity_Usage!R8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="30">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="27">
+      <c r="I8" s="30">
         <f>IFERROR(Capacity_Usage!Q8/Capacity_Usage!O8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="27">
+      <c r="J8" s="30">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="27">
+      <c r="K8" s="30">
         <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
         <v/>
       </c>
-      <c r="L8" s="27">
+      <c r="L8" s="30">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="27">
+      <c r="M8" s="30">
         <f>IFERROR(Capacity_Usage!T8/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N8" s="27">
+      <c r="N8" s="30">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="27">
+      <c r="O8" s="30">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="27">
+      <c r="P8" s="30">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="30">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -8419,47 +8524,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G9" s="27">
+      <c r="G9" s="30">
         <f>IFERROR(Capacity_Usage!S9/Capacity_Usage!R9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="30">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="30">
         <f>IFERROR(Capacity_Usage!Q9/Capacity_Usage!O9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="30">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="27">
+      <c r="K9" s="30">
         <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
         <v/>
       </c>
-      <c r="L9" s="27">
+      <c r="L9" s="30">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="27">
+      <c r="M9" s="30">
         <f>IFERROR(Capacity_Usage!T9/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N9" s="27">
+      <c r="N9" s="30">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="27">
+      <c r="O9" s="30">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="27">
+      <c r="P9" s="30">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="30">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -8497,47 +8602,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G10" s="27">
+      <c r="G10" s="30">
         <f>IFERROR(Capacity_Usage!S10/Capacity_Usage!R10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="30">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="27">
+      <c r="I10" s="30">
         <f>IFERROR(Capacity_Usage!Q10/Capacity_Usage!O10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="27">
+      <c r="J10" s="30">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="27">
+      <c r="K10" s="30">
         <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
         <v/>
       </c>
-      <c r="L10" s="27">
+      <c r="L10" s="30">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="27">
+      <c r="M10" s="30">
         <f>IFERROR(Capacity_Usage!T10/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N10" s="27">
+      <c r="N10" s="30">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="27">
+      <c r="O10" s="30">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="27">
+      <c r="P10" s="30">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="30">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -8575,47 +8680,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G11" s="27">
+      <c r="G11" s="30">
         <f>IFERROR(Capacity_Usage!S11/Capacity_Usage!R11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="30">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="27">
+      <c r="I11" s="30">
         <f>IFERROR(Capacity_Usage!Q11/Capacity_Usage!O11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="27">
+      <c r="J11" s="30">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="27">
+      <c r="K11" s="30">
         <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="27">
+      <c r="L11" s="30">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="27">
+      <c r="M11" s="30">
         <f>IFERROR(Capacity_Usage!T11/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N11" s="27">
+      <c r="N11" s="30">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="27">
+      <c r="O11" s="30">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="30">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="30">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -8653,47 +8758,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G12" s="27">
+      <c r="G12" s="30">
         <f>IFERROR(Capacity_Usage!S12/Capacity_Usage!R12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="30">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="30">
         <f>IFERROR(Capacity_Usage!Q12/Capacity_Usage!O12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="30">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="27">
+      <c r="K12" s="30">
         <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
         <v/>
       </c>
-      <c r="L12" s="27">
+      <c r="L12" s="30">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="27">
+      <c r="M12" s="30">
         <f>IFERROR(Capacity_Usage!T12/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N12" s="27">
+      <c r="N12" s="30">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="27">
+      <c r="O12" s="30">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="27">
+      <c r="P12" s="30">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="27">
+      <c r="Q12" s="30">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -8731,47 +8836,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G13" s="27">
+      <c r="G13" s="30">
         <f>IFERROR(Capacity_Usage!S13/Capacity_Usage!R13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="30">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="27">
+      <c r="I13" s="30">
         <f>IFERROR(Capacity_Usage!Q13/Capacity_Usage!O13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="27">
+      <c r="J13" s="30">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="27">
+      <c r="K13" s="30">
         <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
         <v/>
       </c>
-      <c r="L13" s="27">
+      <c r="L13" s="30">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="27">
+      <c r="M13" s="30">
         <f>IFERROR(Capacity_Usage!T13/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N13" s="27">
+      <c r="N13" s="30">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="27">
+      <c r="O13" s="30">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="27">
+      <c r="P13" s="30">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="27">
+      <c r="Q13" s="30">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -8809,47 +8914,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G14" s="27">
+      <c r="G14" s="30">
         <f>IFERROR(Capacity_Usage!S14/Capacity_Usage!R14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="30">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="27">
+      <c r="I14" s="30">
         <f>IFERROR(Capacity_Usage!Q14/Capacity_Usage!O14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="27">
+      <c r="J14" s="30">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="27">
+      <c r="K14" s="30">
         <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
         <v/>
       </c>
-      <c r="L14" s="27">
+      <c r="L14" s="30">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="27">
+      <c r="M14" s="30">
         <f>IFERROR(Capacity_Usage!T14/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="30">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="27">
+      <c r="O14" s="30">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="27">
+      <c r="P14" s="30">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="27">
+      <c r="Q14" s="30">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -8887,47 +8992,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G15" s="27">
+      <c r="G15" s="30">
         <f>IFERROR(Capacity_Usage!S15/Capacity_Usage!R15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="30">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="27">
+      <c r="I15" s="30">
         <f>IFERROR(Capacity_Usage!Q15/Capacity_Usage!O15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="27">
+      <c r="J15" s="30">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="27">
+      <c r="K15" s="30">
         <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
         <v/>
       </c>
-      <c r="L15" s="27">
+      <c r="L15" s="30">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="27">
+      <c r="M15" s="30">
         <f>IFERROR(Capacity_Usage!T15/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N15" s="27">
+      <c r="N15" s="30">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="27">
+      <c r="O15" s="30">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="27">
+      <c r="P15" s="30">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="27">
+      <c r="Q15" s="30">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -8965,47 +9070,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G16" s="27">
+      <c r="G16" s="30">
         <f>IFERROR(Capacity_Usage!S16/Capacity_Usage!R16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="30">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="27">
+      <c r="I16" s="30">
         <f>IFERROR(Capacity_Usage!Q16/Capacity_Usage!O16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="27">
+      <c r="J16" s="30">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="27">
+      <c r="K16" s="30">
         <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
         <v/>
       </c>
-      <c r="L16" s="27">
+      <c r="L16" s="30">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="27">
+      <c r="M16" s="30">
         <f>IFERROR(Capacity_Usage!T16/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N16" s="27">
+      <c r="N16" s="30">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="27">
+      <c r="O16" s="30">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="27">
+      <c r="P16" s="30">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="27">
+      <c r="Q16" s="30">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -9043,47 +9148,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G17" s="27">
+      <c r="G17" s="30">
         <f>IFERROR(Capacity_Usage!S17/Capacity_Usage!R17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="30">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="27">
+      <c r="I17" s="30">
         <f>IFERROR(Capacity_Usage!Q17/Capacity_Usage!O17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="27">
+      <c r="J17" s="30">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="27">
+      <c r="K17" s="30">
         <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
         <v/>
       </c>
-      <c r="L17" s="27">
+      <c r="L17" s="30">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="27">
+      <c r="M17" s="30">
         <f>IFERROR(Capacity_Usage!T17/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N17" s="27">
+      <c r="N17" s="30">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="27">
+      <c r="O17" s="30">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="27">
+      <c r="P17" s="30">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="27">
+      <c r="Q17" s="30">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Setup: multi-SKU line items per customer/region + 26-SKU dropdown; restore ranked-candidate regions
- Setup sheet replaced single SKU/VM input with an 8-line SKU line-item table:
  one Customer ID + one Geography/Region can request many SKUs. Requested vCPU (B7)
  now = SUM of line vCPUs (VM count x vCPU/VM), feeding the unchanged downstream engine.
- Expanded SKU dropdown to 26 curated standard SKUs (E/D/F families); vCPU counts
  verified against Microsoft Learn size names.
- Restored Ranking: added Rank column (S, COUNTIF) to Scoring_Prod/CVAL/DR and the
  RANKED CANDIDATE REGIONS table (H:P) on Result for Prod/CVAL/DR.
- Result A5 now shows Workload SKUs summary; How_To_Use updated.
- Verified via LibreOffice recalc: zero errors across US/EU/Australia/Asia Pacific/
  Middle East + multi-SKU growth test; ranks ordered by descending PS.
</commit_message>
<xml_diff>
--- a/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
+++ b/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
@@ -140,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -197,10 +197,14 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -212,17 +216,10 @@
     <xf numFmtId="3" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -932,7 +929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B38"/>
+  <dimension ref="B1:B37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1045,7 +1042,7 @@
     <row r="18">
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>3. Setup — pick Geography, SKU, VM count, optional customer-supplied Prod region (required for Middle East), Customer ID.</t>
+          <t>3. Setup — pick Geography, then add one or more SKU line items (SKU + VM count) for the SAME Customer ID &amp; Geography/Region. vCPU/VM auto-fills from the SKU catalogue and Requested vCPU (total) auto-sums across all lines. Optional customer-supplied Prod region (required for Middle East), Customer ID.</t>
         </is>
       </c>
     </row>
@@ -1073,14 +1070,14 @@
     <row r="22">
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>7. Scoring_Prod / 8. Scoring_CVAL / 9. Scoring_DR — PS component breakdown (α/β/γ/δ/ε raw + clamped), AutoSelect flag, Candidate (PS if eligible, −1 if not), and Rank (1 = best candidate, blank = not a candidate for that mode). Winner summary in cols T–U.</t>
+          <t>7. Scoring_Prod / 8. Scoring_CVAL / 9. Scoring_DR — PS component breakdown, AutoSelect flag and winners.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>10. Result — final placement (Prod / CVAL / DR), readiness, DR sizing (max-not-sum), and a Ranked Candidate Regions table (cols H–P) showing all candidate regions ordered by PS for each mode.</t>
+          <t>10. Result — final placement (Prod / CVAL / DR), readiness, DR sizing (max-not-sum), plus a RANKED CANDIDATE REGIONS table (Rank 1 = highest PS) across all catalogue regions for each mode.</t>
         </is>
       </c>
     </row>
@@ -1125,57 +1122,50 @@
     <row r="30">
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Rank formula (Scoring sheets, col S): Rank=COUNTIF(Candidate_range,"&gt;"&amp;this_candidate)+1. Non-candidates (Candidate=-1) are blank. Rank 1 = region with the highest PS score among eligible candidates. Because PS is a continuous float, ties are effectively impossible.</t>
+          <t>DR sizing = MAX-NOT-SUM (A.6 / DR-017): DR req = MAX over source regions of (customers × vCPU).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="3" t="inlineStr">
-        <is>
-          <t>DR sizing = MAX-NOT-SUM (A.6 / DR-017): DR req = MAX over source regions of (customers × vCPU).</t>
-        </is>
-      </c>
+      <c r="B31" s="3" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="B32" s="3" t="inlineStr"/>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>KNOWN GAPS / ASSUMPTIONS (surfaced, not hidden)</t>
+        </is>
+      </c>
     </row>
     <row r="33">
-      <c r="B33" s="4" t="inlineStr">
-        <is>
-          <t>KNOWN GAPS / ASSUMPTIONS (surfaced, not hidden)</t>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>• Metric = Total Cores. Prod = environment tag 'Prod'; everything else = Non-Prod.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>• Metric = Total Cores. Prod = environment tag 'Prod'; everything else = Non-Prod.</t>
+          <t>• Reserved &amp; Quota are DERIVED planning figures (max of even-share and actual alloc, +8% margin), not billed reservations — edit to model reality.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="6" t="inlineStr">
-        <is>
-          <t>• Reserved &amp; Quota are DERIVED planning figures (max of even-share and actual alloc, +8% margin), not billed reservations — edit to model reality.</t>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>• Middle East has ~no real usage in the data — its two regions use a flagged SYNTHETIC pool so the geography can be exercised. Saudi Arabia East is a FUTURE REGION (not yet GA; Microsoft target Q4 2026, Eastern Province; no real usage data will exist until launch). UAE North is GA but absent from ACRME source data. Japan East (Asia Pacific) is 'pending' in the catalogue and is excluded.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="7" t="inlineStr">
-        <is>
-          <t>• Middle East has ~no real usage in the data — its two regions use a flagged SYNTHETIC pool so the geography can be exercised. Saudi Arabia East is a FUTURE REGION (not yet GA; Microsoft target Q4 2026, Eastern Province; no real usage data will exist until launch). UAE North is GA but absent from ACRME source data. Japan East (Asia Pacific) is 'pending' in the catalogue and is excluded.</t>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>• total_customers is undefined in baseline v2.4 — mode selector on Policy (Live/Constant/Manual). γ values illustrative.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>• total_customers is undefined in baseline v2.4 — mode selector on Policy (Live/Constant/Manual). γ values illustrative.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" s="6" t="inlineStr">
         <is>
           <t>• PS_NonProd δ duplicates its α (baseline design-of-record). DR bootstrap / target are configurable placeholders.</t>
         </is>
@@ -1201,15 +1191,16 @@
     <col width="4" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="3" customWidth="1" min="7" max="7"/>
     <col width="6" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
     <col width="6" customWidth="1" min="11" max="11"/>
     <col width="20" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
+    <col width="9" customWidth="1" min="13" max="13"/>
     <col width="6" customWidth="1" min="14" max="14"/>
     <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="8" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1229,12 +1220,12 @@
         <f>Setup!B9</f>
         <v/>
       </c>
-      <c r="E3" s="29" t="inlineStr">
+      <c r="E3" s="25" t="inlineStr">
         <is>
           <t>DR SIZING (max-not-sum, A.6 / DR-017)</t>
         </is>
       </c>
-      <c r="H3" s="32" t="inlineStr">
+      <c r="H3" s="25" t="inlineStr">
         <is>
           <t>RANKED CANDIDATE REGIONS  (Rank 1 = highest PS; blank = not a candidate for this mode)</t>
         </is>
@@ -1269,11 +1260,11 @@
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>SKU</t>
+          <t>Workload SKUs</t>
         </is>
       </c>
       <c r="B5" s="11">
-        <f>Setup!B4</f>
+        <f>Setup!B6</f>
         <v/>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -1358,7 +1349,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(1,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1370,7 +1361,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M6" s="30">
+      <c r="M6" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(1,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1382,7 +1373,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P6" s="30">
+      <c r="P6" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(1,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1405,7 +1396,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(2,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1417,7 +1408,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M7" s="30">
+      <c r="M7" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(2,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1429,7 +1420,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P7" s="30">
+      <c r="P7" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(2,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1455,7 +1446,7 @@
           <t>DR Requirement (max-not-sum)</t>
         </is>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="24">
         <f>F6*F7</f>
         <v/>
       </c>
@@ -1467,7 +1458,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J8" s="30">
+      <c r="J8" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(3,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1479,7 +1470,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M8" s="30">
+      <c r="M8" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(3,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1491,7 +1482,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P8" s="30">
+      <c r="P8" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(3,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1506,7 +1497,7 @@
         <f>Scoring_Prod!U3</f>
         <v/>
       </c>
-      <c r="C9" s="30">
+      <c r="C9" s="31">
         <f>Scoring_Prod!U4</f>
         <v/>
       </c>
@@ -1527,7 +1518,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J9" s="30">
+      <c r="J9" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(4,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1539,7 +1530,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M9" s="30">
+      <c r="M9" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(4,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1551,7 +1542,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P9" s="30">
+      <c r="P9" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(4,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1566,7 +1557,7 @@
         <f>Scoring_CVAL!U2</f>
         <v/>
       </c>
-      <c r="C10" s="30">
+      <c r="C10" s="31">
         <f>Scoring_CVAL!U3</f>
         <v/>
       </c>
@@ -1587,7 +1578,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J10" s="30">
+      <c r="J10" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(5,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1599,7 +1590,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M10" s="30">
+      <c r="M10" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(5,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1611,7 +1602,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P10" s="30">
+      <c r="P10" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(5,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1626,11 +1617,11 @@
         <f>Scoring_DR!U2</f>
         <v/>
       </c>
-      <c r="C11" s="30">
+      <c r="C11" s="31">
         <f>Scoring_DR!U3</f>
         <v/>
       </c>
-      <c r="E11" s="34" t="inlineStr">
+      <c r="E11" s="33" t="inlineStr">
         <is>
           <t>Note: illustrative — sources = regions in DR scope geography.</t>
         </is>
@@ -1643,7 +1634,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(6,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1655,7 +1646,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M11" s="30">
+      <c r="M11" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(6,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1667,7 +1658,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P11" s="30">
+      <c r="P11" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(6,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1681,7 +1672,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(7,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1693,7 +1684,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M12" s="30">
+      <c r="M12" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(7,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1705,7 +1696,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P12" s="30">
+      <c r="P12" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(7,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1716,7 +1707,7 @@
           <t>Readiness State</t>
         </is>
       </c>
-      <c r="B13" s="33">
+      <c r="B13" s="24">
         <f>IF(B9="NONE ELIGIBLE","QUOTA_DEFICIT / NEEDS EXPLICIT REGION (Prod)",IF(B10="NONE ELIGIBLE","CAPACITY_UNAVAILABLE (CVAL)",IF(B11="NONE ELIGIBLE","READY_WITH_RISK (no DR region)","READY")))</f>
         <v/>
       </c>
@@ -1728,7 +1719,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(8,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1740,7 +1731,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M13" s="30">
+      <c r="M13" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(8,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1752,7 +1743,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P13" s="30">
+      <c r="P13" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(8,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1766,7 +1757,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(9,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1778,7 +1769,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M14" s="30">
+      <c r="M14" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(9,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1790,7 +1781,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P14" s="30">
+      <c r="P14" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(9,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1813,7 +1804,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(10,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1825,7 +1816,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M15" s="30">
+      <c r="M15" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(10,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1837,7 +1828,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P15" s="30">
+      <c r="P15" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(10,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1851,7 +1842,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(11,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1863,7 +1854,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M16" s="30">
+      <c r="M16" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(11,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1875,7 +1866,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P16" s="30">
+      <c r="P16" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(11,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1889,7 +1880,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(12,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1901,7 +1892,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M17" s="30">
+      <c r="M17" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(12,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1913,7 +1904,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(12,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1927,7 +1918,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J18" s="30">
+      <c r="J18" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(13,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1939,7 +1930,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M18" s="30">
+      <c r="M18" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(13,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1951,7 +1942,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P18" s="30">
+      <c r="P18" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(13,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1965,7 +1956,7 @@
         <f>IFERROR(INDEX(Scoring_Prod!$A$4:$A$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="J19" s="30">
+      <c r="J19" s="31">
         <f>IFERROR(INDEX(Scoring_Prod!$Q$4:$Q$17,MATCH(14,Scoring_Prod!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1977,7 +1968,7 @@
         <f>IFERROR(INDEX(Scoring_CVAL!$A$4:$A$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="M19" s="30">
+      <c r="M19" s="31">
         <f>IFERROR(INDEX(Scoring_CVAL!$Q$4:$Q$17,MATCH(14,Scoring_CVAL!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -1989,7 +1980,7 @@
         <f>IFERROR(INDEX(Scoring_DR!$A$4:$A$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
-      <c r="P19" s="30">
+      <c r="P19" s="31">
         <f>IFERROR(INDEX(Scoring_DR!$Q$4:$Q$17,MATCH(14,Scoring_DR!$S$4:$S$17,0)),"")</f>
         <v/>
       </c>
@@ -2756,16 +2747,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="3" customWidth="1" min="3" max="3"/>
-    <col width="3" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="3" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="3" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2774,21 +2769,36 @@
           <t>SETUP — Customer &amp; Workload</t>
         </is>
       </c>
-      <c r="E1" s="9" t="inlineStr">
+      <c r="F1" s="9" t="inlineStr">
         <is>
           <t>Lookup tables (do not edit)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="E2" s="22" t="inlineStr">
+      <c r="F2" s="22" t="inlineStr">
         <is>
           <t>SKU</t>
         </is>
       </c>
-      <c r="F2" s="22" t="inlineStr">
+      <c r="G2" s="22" t="inlineStr">
         <is>
           <t>vCPU/VM</t>
+        </is>
+      </c>
+      <c r="I2" s="22" t="inlineStr">
+        <is>
+          <t>Geography</t>
+        </is>
+      </c>
+      <c r="J2" s="22" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="K2" s="22" t="inlineStr">
+        <is>
+          <t>DR Scope Geo</t>
         </is>
       </c>
     </row>
@@ -2803,89 +2813,164 @@
           <t>US</t>
         </is>
       </c>
-      <c r="E3" s="20" t="inlineStr">
-        <is>
-          <t>E16ads_v5</t>
-        </is>
-      </c>
-      <c r="F3" s="20" t="n">
-        <v>16</v>
+      <c r="F3" s="20" t="inlineStr">
+        <is>
+          <t>E64ads_v6</t>
+        </is>
+      </c>
+      <c r="G3" s="20" t="n">
+        <v>64</v>
+      </c>
+      <c r="I3" s="20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="J3" s="20" t="inlineStr">
+        <is>
+          <t>3-region</t>
+        </is>
+      </c>
+      <c r="K3" s="20" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>SKU</t>
-        </is>
-      </c>
-      <c r="B4" s="23" t="inlineStr">
-        <is>
-          <t>E16ads_v5</t>
-        </is>
-      </c>
-      <c r="E4" s="20" t="inlineStr">
-        <is>
-          <t>E32ads_v5</t>
-        </is>
-      </c>
-      <c r="F4" s="20" t="n">
-        <v>32</v>
+          <t>Total VMs (all SKUs)</t>
+        </is>
+      </c>
+      <c r="B4" s="11">
+        <f>SUM(B15:B22)</f>
+        <v/>
+      </c>
+      <c r="F4" s="20" t="inlineStr">
+        <is>
+          <t>E64ads_v5</t>
+        </is>
+      </c>
+      <c r="G4" s="20" t="n">
+        <v>64</v>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>2-region</t>
+        </is>
+      </c>
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>VM count</t>
-        </is>
-      </c>
-      <c r="B5" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="E5" s="20" t="inlineStr">
-        <is>
-          <t>E8ads_v5</t>
-        </is>
-      </c>
-      <c r="F5" s="20" t="n">
-        <v>8</v>
+          <t>SKU line count</t>
+        </is>
+      </c>
+      <c r="B5" s="11">
+        <f>COUNTA(A15:A22)</f>
+        <v/>
+      </c>
+      <c r="F5" s="20" t="inlineStr">
+        <is>
+          <t>E48ads_v5</t>
+        </is>
+      </c>
+      <c r="G5" s="20" t="n">
+        <v>48</v>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="J5" s="20" t="inlineStr">
+        <is>
+          <t>2-region</t>
+        </is>
+      </c>
+      <c r="K5" s="20" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>vCPU per VM</t>
-        </is>
-      </c>
-      <c r="B6" s="24">
-        <f>VLOOKUP(B4,E3:F10,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="E6" s="20" t="inlineStr">
-        <is>
-          <t>E4ads_v5</t>
-        </is>
-      </c>
-      <c r="F6" s="20" t="n">
-        <v>4</v>
+          <t>Workload SKUs</t>
+        </is>
+      </c>
+      <c r="B6" s="11">
+        <f>_xlfn.TEXTJOIN(", ",TRUE,A15:A22)</f>
+        <v/>
+      </c>
+      <c r="F6" s="20" t="inlineStr">
+        <is>
+          <t>E32ads_v6</t>
+        </is>
+      </c>
+      <c r="G6" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="I6" s="20" t="inlineStr">
+        <is>
+          <t>Asia Pacific</t>
+        </is>
+      </c>
+      <c r="J6" s="20" t="inlineStr">
+        <is>
+          <t>2-region</t>
+        </is>
+      </c>
+      <c r="K6" s="20" t="inlineStr">
+        <is>
+          <t>Asia Pacific</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
-          <t>Requested vCPU</t>
-        </is>
-      </c>
-      <c r="B7" s="25">
-        <f>B5*B6</f>
-        <v/>
-      </c>
-      <c r="E7" s="20" t="inlineStr">
-        <is>
-          <t>D8ads_v5</t>
-        </is>
-      </c>
-      <c r="F7" s="20" t="n">
-        <v>8</v>
+          <t>Requested vCPU (total)</t>
+        </is>
+      </c>
+      <c r="B7" s="24">
+        <f>SUM(D15:D22)</f>
+        <v/>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>E32ads_v5</t>
+        </is>
+      </c>
+      <c r="G7" s="20" t="n">
+        <v>32</v>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="J7" s="20" t="inlineStr">
+        <is>
+          <t>cross-geo</t>
+        </is>
+      </c>
+      <c r="K7" s="20" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -2895,13 +2980,13 @@
         </is>
       </c>
       <c r="B8" s="23" t="inlineStr"/>
-      <c r="E8" s="20" t="inlineStr">
-        <is>
-          <t>D4ads_v5</t>
-        </is>
-      </c>
-      <c r="F8" s="20" t="n">
-        <v>4</v>
+      <c r="F8" s="20" t="inlineStr">
+        <is>
+          <t>E20ads_v5</t>
+        </is>
+      </c>
+      <c r="G8" s="20" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -2915,13 +3000,13 @@
           <t>CUST-0042</t>
         </is>
       </c>
-      <c r="E9" s="20" t="inlineStr">
-        <is>
-          <t>D2ads_v5</t>
-        </is>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>2</v>
+      <c r="F9" s="20" t="inlineStr">
+        <is>
+          <t>E16ads_v6</t>
+        </is>
+      </c>
+      <c r="G9" s="20" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="10">
@@ -2930,16 +3015,16 @@
           <t>Distribution model</t>
         </is>
       </c>
-      <c r="B10" s="24">
-        <f>VLOOKUP(B3,E13:G17,2,FALSE)</f>
-        <v/>
-      </c>
-      <c r="E10" s="20" t="inlineStr">
-        <is>
-          <t>D16ads_v5</t>
-        </is>
-      </c>
-      <c r="F10" s="20" t="n">
+      <c r="B10" s="11">
+        <f>VLOOKUP(B3,$I$3:$K$7,2,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>E16ads_v5</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="n">
         <v>16</v>
       </c>
     </row>
@@ -2949,123 +3034,328 @@
           <t>DR scope geography</t>
         </is>
       </c>
-      <c r="B11" s="24">
-        <f>VLOOKUP(B3,E13:G17,3,FALSE)</f>
-        <v/>
+      <c r="B11" s="11">
+        <f>VLOOKUP(B3,$I$3:$K$7,3,FALSE)</f>
+        <v/>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
+        <is>
+          <t>E8ads_v5</t>
+        </is>
+      </c>
+      <c r="G11" s="20" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="22" t="inlineStr">
-        <is>
-          <t>Geography</t>
-        </is>
-      </c>
-      <c r="F12" s="22" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G12" s="22" t="inlineStr">
-        <is>
-          <t>DR Scope Geo</t>
-        </is>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>E4ads_v5</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="13">
-      <c r="E13" s="20" t="inlineStr">
-        <is>
-          <t>US</t>
+      <c r="A13" s="25" t="inlineStr">
+        <is>
+          <t>WORKLOAD — SKU LINE ITEMS  (one Customer ID, one Geography/Region; add as many SKUs as needed)</t>
         </is>
       </c>
       <c r="F13" s="20" t="inlineStr">
         <is>
-          <t>3-region</t>
-        </is>
-      </c>
-      <c r="G13" s="20" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
+          <t>E2ads_v5</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="14">
-      <c r="E14" s="20" t="inlineStr">
-        <is>
-          <t>EU</t>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>SKU</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>VM count</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>vCPU/VM</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>Line vCPU</t>
         </is>
       </c>
       <c r="F14" s="20" t="inlineStr">
         <is>
-          <t>2-region</t>
-        </is>
-      </c>
-      <c r="G14" s="20" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
+          <t>D64ads_v5</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="15">
-      <c r="E15" s="20" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
+      <c r="A15" s="23" t="inlineStr">
+        <is>
+          <t>E16ads_v5</t>
+        </is>
+      </c>
+      <c r="B15" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="11">
+        <f>IF($A15="","",VLOOKUP($A15,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D15" s="11">
+        <f>IF($A15="","",$B15*$C15)</f>
+        <v/>
       </c>
       <c r="F15" s="20" t="inlineStr">
         <is>
-          <t>2-region</t>
-        </is>
-      </c>
-      <c r="G15" s="20" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
+          <t>D32ads_v5</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="16">
-      <c r="E16" s="20" t="inlineStr">
-        <is>
-          <t>Asia Pacific</t>
-        </is>
+      <c r="A16" s="23" t="inlineStr">
+        <is>
+          <t>D8ads_v5</t>
+        </is>
+      </c>
+      <c r="B16" s="23" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="11">
+        <f>IF($A16="","",VLOOKUP($A16,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D16" s="11">
+        <f>IF($A16="","",$B16*$C16)</f>
+        <v/>
       </c>
       <c r="F16" s="20" t="inlineStr">
         <is>
-          <t>2-region</t>
-        </is>
-      </c>
-      <c r="G16" s="20" t="inlineStr">
-        <is>
-          <t>Asia Pacific</t>
-        </is>
+          <t>D16ads_v5</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="17">
-      <c r="E17" s="20" t="inlineStr">
-        <is>
-          <t>Middle East</t>
-        </is>
+      <c r="A17" s="23" t="n"/>
+      <c r="B17" s="23" t="n"/>
+      <c r="C17" s="11">
+        <f>IF($A17="","",VLOOKUP($A17,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D17" s="11">
+        <f>IF($A17="","",$B17*$C17)</f>
+        <v/>
       </c>
       <c r="F17" s="20" t="inlineStr">
         <is>
-          <t>cross-geo</t>
-        </is>
-      </c>
-      <c r="G17" s="20" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
+          <t>D16as_v5</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="23" t="n"/>
+      <c r="B18" s="23" t="n"/>
+      <c r="C18" s="11">
+        <f>IF($A18="","",VLOOKUP($A18,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D18" s="11">
+        <f>IF($A18="","",$B18*$C18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="20" t="inlineStr">
+        <is>
+          <t>D8ads_v5</t>
+        </is>
+      </c>
+      <c r="G18" s="20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="n"/>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="11">
+        <f>IF($A19="","",VLOOKUP($A19,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D19" s="11">
+        <f>IF($A19="","",$B19*$C19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="20" t="inlineStr">
+        <is>
+          <t>D8as_v5</t>
+        </is>
+      </c>
+      <c r="G19" s="20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="n"/>
+      <c r="B20" s="23" t="n"/>
+      <c r="C20" s="11">
+        <f>IF($A20="","",VLOOKUP($A20,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D20" s="11">
+        <f>IF($A20="","",$B20*$C20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="20" t="inlineStr">
+        <is>
+          <t>D4ads_v5</t>
+        </is>
+      </c>
+      <c r="G20" s="20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="23" t="n"/>
+      <c r="B21" s="23" t="n"/>
+      <c r="C21" s="11">
+        <f>IF($A21="","",VLOOKUP($A21,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D21" s="11">
+        <f>IF($A21="","",$B21*$C21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="20" t="inlineStr">
+        <is>
+          <t>D4as_v5</t>
+        </is>
+      </c>
+      <c r="G21" s="20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="n"/>
+      <c r="B22" s="23" t="n"/>
+      <c r="C22" s="11">
+        <f>IF($A22="","",VLOOKUP($A22,$F$3:$G$28,2,FALSE))</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>IF($A22="","",$B22*$C22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="20" t="inlineStr">
+        <is>
+          <t>D2ads_v5</t>
+        </is>
+      </c>
+      <c r="G22" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="C23" s="14" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="D23" s="24">
+        <f>SUM(D15:D22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="20" t="inlineStr">
+        <is>
+          <t>D2as_v5</t>
+        </is>
+      </c>
+      <c r="G23" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="F24" s="20" t="inlineStr">
+        <is>
+          <t>F32s_v2</t>
+        </is>
+      </c>
+      <c r="G24" s="20" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="F25" s="20" t="inlineStr">
+        <is>
+          <t>F16s_v2</t>
+        </is>
+      </c>
+      <c r="G25" s="20" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="F26" s="20" t="inlineStr">
+        <is>
+          <t>F8s_v2</t>
+        </is>
+      </c>
+      <c r="G26" s="20" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="F27" s="20" t="inlineStr">
+        <is>
+          <t>F4s_v2</t>
+        </is>
+      </c>
+      <c r="G27" s="20" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="F28" s="20" t="inlineStr">
+        <is>
+          <t>F2s_v2</t>
+        </is>
+      </c>
+      <c r="G28" s="20" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B3" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"US,EU,Australia,Asia Pacific,Middle East"</formula1>
     </dataValidation>
-    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"E16ads_v5,E32ads_v5,E8ads_v5,E4ads_v5,D8ads_v5,D4ads_v5,D2ads_v5,D16ads_v5"</formula1>
-    </dataValidation>
     <dataValidation sqref="B8" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=Capacity_Usage!$B$4:$B$17</formula1>
+    </dataValidation>
+    <dataValidation sqref="A15:A22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=$F$3:$F$28</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3151,7 +3441,7 @@
           <t>Weight sum</t>
         </is>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="26">
         <f>SUM(B2:B6)</f>
         <v/>
       </c>
@@ -3162,7 +3452,7 @@
           <t>Validation</t>
         </is>
       </c>
-      <c r="B8" s="24">
+      <c r="B8" s="27">
         <f>IF(ABS(B7-1)&lt;=0.001,"VALID","INVALID — must sum to 1.0")</f>
         <v/>
       </c>
@@ -3485,42 +3775,42 @@
       <c r="E4" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="26" t="n">
+      <c r="F4" s="28" t="n">
         <v>42492</v>
       </c>
-      <c r="G4" s="26" t="n">
+      <c r="G4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="H4" s="27">
+      <c r="H4" s="29">
         <f>F4-G4</f>
         <v/>
       </c>
-      <c r="I4" s="26" t="n">
+      <c r="I4" s="28" t="n">
         <v>63738</v>
       </c>
-      <c r="J4" s="26" t="n">
+      <c r="J4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="K4" s="27">
+      <c r="K4" s="29">
         <f>I4-J4</f>
         <v/>
       </c>
-      <c r="L4" s="26" t="n">
+      <c r="L4" s="28" t="n">
         <v>94710</v>
       </c>
-      <c r="M4" s="26" t="n">
+      <c r="M4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="N4" s="26" t="n">
+      <c r="N4" s="28" t="n">
         <v>94708</v>
       </c>
-      <c r="O4" s="26" t="n">
+      <c r="O4" s="28" t="n">
         <v>142064</v>
       </c>
-      <c r="P4" s="26" t="n">
+      <c r="P4" s="28" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" s="27">
+      <c r="Q4" s="29">
         <f>O4-P4</f>
         <v/>
       </c>
@@ -3536,7 +3826,7 @@
       <c r="U4" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="V4" s="27" t="inlineStr">
+      <c r="V4" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3566,42 +3856,42 @@
       <c r="E5" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="28" t="n">
         <v>42492</v>
       </c>
-      <c r="G5" s="26" t="n">
+      <c r="G5" s="28" t="n">
         <v>12292</v>
       </c>
-      <c r="H5" s="27">
+      <c r="H5" s="29">
         <f>F5-G5</f>
         <v/>
       </c>
-      <c r="I5" s="26" t="n">
+      <c r="I5" s="28" t="n">
         <v>63738</v>
       </c>
-      <c r="J5" s="26" t="n">
+      <c r="J5" s="28" t="n">
         <v>12292</v>
       </c>
-      <c r="K5" s="27">
+      <c r="K5" s="29">
         <f>I5-J5</f>
         <v/>
       </c>
-      <c r="L5" s="26" t="n">
+      <c r="L5" s="28" t="n">
         <v>94710</v>
       </c>
-      <c r="M5" s="26" t="n">
+      <c r="M5" s="28" t="n">
         <v>27398</v>
       </c>
-      <c r="N5" s="26" t="n">
+      <c r="N5" s="28" t="n">
         <v>67312</v>
       </c>
-      <c r="O5" s="26" t="n">
+      <c r="O5" s="28" t="n">
         <v>142064</v>
       </c>
-      <c r="P5" s="26" t="n">
+      <c r="P5" s="28" t="n">
         <v>27398</v>
       </c>
-      <c r="Q5" s="27">
+      <c r="Q5" s="29">
         <f>O5-P5</f>
         <v/>
       </c>
@@ -3617,7 +3907,7 @@
       <c r="U5" s="23" t="n">
         <v>65</v>
       </c>
-      <c r="V5" s="27" t="inlineStr">
+      <c r="V5" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3647,42 +3937,42 @@
       <c r="E6" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="26" t="n">
+      <c r="F6" s="28" t="n">
         <v>42492</v>
       </c>
-      <c r="G6" s="26" t="n">
+      <c r="G6" s="28" t="n">
         <v>2326</v>
       </c>
-      <c r="H6" s="27">
+      <c r="H6" s="29">
         <f>F6-G6</f>
         <v/>
       </c>
-      <c r="I6" s="26" t="n">
+      <c r="I6" s="28" t="n">
         <v>63738</v>
       </c>
-      <c r="J6" s="26" t="n">
+      <c r="J6" s="28" t="n">
         <v>2326</v>
       </c>
-      <c r="K6" s="27">
+      <c r="K6" s="29">
         <f>I6-J6</f>
         <v/>
       </c>
-      <c r="L6" s="26" t="n">
+      <c r="L6" s="28" t="n">
         <v>94710</v>
       </c>
-      <c r="M6" s="26" t="n">
+      <c r="M6" s="28" t="n">
         <v>5186</v>
       </c>
-      <c r="N6" s="26" t="n">
+      <c r="N6" s="28" t="n">
         <v>89524</v>
       </c>
-      <c r="O6" s="26" t="n">
+      <c r="O6" s="28" t="n">
         <v>142064</v>
       </c>
-      <c r="P6" s="26" t="n">
+      <c r="P6" s="28" t="n">
         <v>5186</v>
       </c>
-      <c r="Q6" s="27">
+      <c r="Q6" s="29">
         <f>O6-P6</f>
         <v/>
       </c>
@@ -3698,7 +3988,7 @@
       <c r="U6" s="23" t="n">
         <v>10</v>
       </c>
-      <c r="V6" s="27" t="inlineStr">
+      <c r="V6" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3728,42 +4018,42 @@
       <c r="E7" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="28" t="n">
         <v>154178</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="28" t="n">
         <v>142756</v>
       </c>
-      <c r="H7" s="27">
+      <c r="H7" s="29">
         <f>F7-G7</f>
         <v/>
       </c>
-      <c r="I7" s="26" t="n">
+      <c r="I7" s="28" t="n">
         <v>231266</v>
       </c>
-      <c r="J7" s="26" t="n">
+      <c r="J7" s="28" t="n">
         <v>142756</v>
       </c>
-      <c r="K7" s="27">
+      <c r="K7" s="29">
         <f>I7-J7</f>
         <v/>
       </c>
-      <c r="L7" s="26" t="n">
+      <c r="L7" s="28" t="n">
         <v>343646</v>
       </c>
-      <c r="M7" s="26" t="n">
+      <c r="M7" s="28" t="n">
         <v>318190</v>
       </c>
-      <c r="N7" s="26" t="n">
+      <c r="N7" s="28" t="n">
         <v>25456</v>
       </c>
-      <c r="O7" s="26" t="n">
+      <c r="O7" s="28" t="n">
         <v>515468</v>
       </c>
-      <c r="P7" s="26" t="n">
+      <c r="P7" s="28" t="n">
         <v>318190</v>
       </c>
-      <c r="Q7" s="27">
+      <c r="Q7" s="29">
         <f>O7-P7</f>
         <v/>
       </c>
@@ -3779,7 +4069,7 @@
       <c r="U7" s="23" t="n">
         <v>150</v>
       </c>
-      <c r="V7" s="27" t="inlineStr">
+      <c r="V7" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3809,42 +4099,42 @@
       <c r="E8" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F8" s="26" t="n">
+      <c r="F8" s="28" t="n">
         <v>13334</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="28" t="n">
         <v>628</v>
       </c>
-      <c r="H8" s="27">
+      <c r="H8" s="29">
         <f>F8-G8</f>
         <v/>
       </c>
-      <c r="I8" s="26" t="n">
+      <c r="I8" s="28" t="n">
         <v>20002</v>
       </c>
-      <c r="J8" s="26" t="n">
+      <c r="J8" s="28" t="n">
         <v>628</v>
       </c>
-      <c r="K8" s="27">
+      <c r="K8" s="29">
         <f>I8-J8</f>
         <v/>
       </c>
-      <c r="L8" s="26" t="n">
+      <c r="L8" s="28" t="n">
         <v>40456</v>
       </c>
-      <c r="M8" s="26" t="n">
+      <c r="M8" s="28" t="n">
         <v>1902</v>
       </c>
-      <c r="N8" s="26" t="n">
+      <c r="N8" s="28" t="n">
         <v>38554</v>
       </c>
-      <c r="O8" s="26" t="n">
+      <c r="O8" s="28" t="n">
         <v>60684</v>
       </c>
-      <c r="P8" s="26" t="n">
+      <c r="P8" s="28" t="n">
         <v>1902</v>
       </c>
-      <c r="Q8" s="27">
+      <c r="Q8" s="29">
         <f>O8-P8</f>
         <v/>
       </c>
@@ -3860,7 +4150,7 @@
       <c r="U8" s="23" t="n">
         <v>11</v>
       </c>
-      <c r="V8" s="27" t="inlineStr">
+      <c r="V8" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3890,42 +4180,42 @@
       <c r="E9" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F9" s="26" t="n">
+      <c r="F9" s="28" t="n">
         <v>13334</v>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="28" t="n">
         <v>842</v>
       </c>
-      <c r="H9" s="27">
+      <c r="H9" s="29">
         <f>F9-G9</f>
         <v/>
       </c>
-      <c r="I9" s="26" t="n">
+      <c r="I9" s="28" t="n">
         <v>20002</v>
       </c>
-      <c r="J9" s="26" t="n">
+      <c r="J9" s="28" t="n">
         <v>842</v>
       </c>
-      <c r="K9" s="27">
+      <c r="K9" s="29">
         <f>I9-J9</f>
         <v/>
       </c>
-      <c r="L9" s="26" t="n">
+      <c r="L9" s="28" t="n">
         <v>40456</v>
       </c>
-      <c r="M9" s="26" t="n">
+      <c r="M9" s="28" t="n">
         <v>2552</v>
       </c>
-      <c r="N9" s="26" t="n">
+      <c r="N9" s="28" t="n">
         <v>37904</v>
       </c>
-      <c r="O9" s="26" t="n">
+      <c r="O9" s="28" t="n">
         <v>60684</v>
       </c>
-      <c r="P9" s="26" t="n">
+      <c r="P9" s="28" t="n">
         <v>2552</v>
       </c>
-      <c r="Q9" s="27">
+      <c r="Q9" s="29">
         <f>O9-P9</f>
         <v/>
       </c>
@@ -3941,7 +4231,7 @@
       <c r="U9" s="23" t="n">
         <v>13</v>
       </c>
-      <c r="V9" s="27" t="inlineStr">
+      <c r="V9" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -3971,42 +4261,42 @@
       <c r="E10" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F10" s="26" t="n">
+      <c r="F10" s="28" t="n">
         <v>13334</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="28" t="n">
         <v>3072</v>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="29">
         <f>F10-G10</f>
         <v/>
       </c>
-      <c r="I10" s="26" t="n">
+      <c r="I10" s="28" t="n">
         <v>20002</v>
       </c>
-      <c r="J10" s="26" t="n">
+      <c r="J10" s="28" t="n">
         <v>3072</v>
       </c>
-      <c r="K10" s="27">
+      <c r="K10" s="29">
         <f>I10-J10</f>
         <v/>
       </c>
-      <c r="L10" s="26" t="n">
+      <c r="L10" s="28" t="n">
         <v>40456</v>
       </c>
-      <c r="M10" s="26" t="n">
+      <c r="M10" s="28" t="n">
         <v>9322</v>
       </c>
-      <c r="N10" s="26" t="n">
+      <c r="N10" s="28" t="n">
         <v>31134</v>
       </c>
-      <c r="O10" s="26" t="n">
+      <c r="O10" s="28" t="n">
         <v>60684</v>
       </c>
-      <c r="P10" s="26" t="n">
+      <c r="P10" s="28" t="n">
         <v>9322</v>
       </c>
-      <c r="Q10" s="27">
+      <c r="Q10" s="29">
         <f>O10-P10</f>
         <v/>
       </c>
@@ -4022,7 +4312,7 @@
       <c r="U10" s="23" t="n">
         <v>30</v>
       </c>
-      <c r="V10" s="27" t="inlineStr">
+      <c r="V10" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4052,42 +4342,42 @@
       <c r="E11" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="28" t="n">
         <v>48434</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="28" t="n">
         <v>44846</v>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="29">
         <f>F11-G11</f>
         <v/>
       </c>
-      <c r="I11" s="26" t="n">
+      <c r="I11" s="28" t="n">
         <v>72650</v>
       </c>
-      <c r="J11" s="26" t="n">
+      <c r="J11" s="28" t="n">
         <v>44846</v>
       </c>
-      <c r="K11" s="27">
+      <c r="K11" s="29">
         <f>I11-J11</f>
         <v/>
       </c>
-      <c r="L11" s="26" t="n">
+      <c r="L11" s="28" t="n">
         <v>146950</v>
       </c>
-      <c r="M11" s="26" t="n">
+      <c r="M11" s="28" t="n">
         <v>136064</v>
       </c>
-      <c r="N11" s="26" t="n">
+      <c r="N11" s="28" t="n">
         <v>10886</v>
       </c>
-      <c r="O11" s="26" t="n">
+      <c r="O11" s="28" t="n">
         <v>220424</v>
       </c>
-      <c r="P11" s="26" t="n">
+      <c r="P11" s="28" t="n">
         <v>136064</v>
       </c>
-      <c r="Q11" s="27">
+      <c r="Q11" s="29">
         <f>O11-P11</f>
         <v/>
       </c>
@@ -4103,7 +4393,7 @@
       <c r="U11" s="23" t="n">
         <v>69</v>
       </c>
-      <c r="V11" s="27" t="inlineStr">
+      <c r="V11" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4133,42 +4423,42 @@
       <c r="E12" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="26" t="n">
+      <c r="F12" s="28" t="n">
         <v>9518</v>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="28" t="n">
         <v>8812</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="29">
         <f>F12-G12</f>
         <v/>
       </c>
-      <c r="I12" s="26" t="n">
+      <c r="I12" s="28" t="n">
         <v>14276</v>
       </c>
-      <c r="J12" s="26" t="n">
+      <c r="J12" s="28" t="n">
         <v>8812</v>
       </c>
-      <c r="K12" s="27">
+      <c r="K12" s="29">
         <f>I12-J12</f>
         <v/>
       </c>
-      <c r="L12" s="26" t="n">
+      <c r="L12" s="28" t="n">
         <v>17958</v>
       </c>
-      <c r="M12" s="26" t="n">
+      <c r="M12" s="28" t="n">
         <v>16628</v>
       </c>
-      <c r="N12" s="26" t="n">
+      <c r="N12" s="28" t="n">
         <v>1330</v>
       </c>
-      <c r="O12" s="26" t="n">
+      <c r="O12" s="28" t="n">
         <v>26936</v>
       </c>
-      <c r="P12" s="26" t="n">
+      <c r="P12" s="28" t="n">
         <v>16628</v>
       </c>
-      <c r="Q12" s="27">
+      <c r="Q12" s="29">
         <f>O12-P12</f>
         <v/>
       </c>
@@ -4184,7 +4474,7 @@
       <c r="U12" s="23" t="n">
         <v>34</v>
       </c>
-      <c r="V12" s="27" t="inlineStr">
+      <c r="V12" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4214,42 +4504,42 @@
       <c r="E13" s="23" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="28" t="n">
         <v>5624</v>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="28" t="n">
         <v>1602</v>
       </c>
-      <c r="H13" s="27">
+      <c r="H13" s="29">
         <f>F13-G13</f>
         <v/>
       </c>
-      <c r="I13" s="26" t="n">
+      <c r="I13" s="28" t="n">
         <v>8434</v>
       </c>
-      <c r="J13" s="26" t="n">
+      <c r="J13" s="28" t="n">
         <v>1602</v>
       </c>
-      <c r="K13" s="27">
+      <c r="K13" s="29">
         <f>I13-J13</f>
         <v/>
       </c>
-      <c r="L13" s="26" t="n">
+      <c r="L13" s="28" t="n">
         <v>10610</v>
       </c>
-      <c r="M13" s="26" t="n">
+      <c r="M13" s="28" t="n">
         <v>3020</v>
       </c>
-      <c r="N13" s="26" t="n">
+      <c r="N13" s="28" t="n">
         <v>7590</v>
       </c>
-      <c r="O13" s="26" t="n">
+      <c r="O13" s="28" t="n">
         <v>15914</v>
       </c>
-      <c r="P13" s="26" t="n">
+      <c r="P13" s="28" t="n">
         <v>3020</v>
       </c>
-      <c r="Q13" s="27">
+      <c r="Q13" s="29">
         <f>O13-P13</f>
         <v/>
       </c>
@@ -4265,7 +4555,7 @@
       <c r="U13" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="V13" s="27" t="inlineStr">
+      <c r="V13" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4295,42 +4585,42 @@
       <c r="E14" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="28" t="n">
         <v>12504</v>
       </c>
-      <c r="G14" s="26" t="n">
+      <c r="G14" s="28" t="n">
         <v>2956</v>
       </c>
-      <c r="H14" s="27">
+      <c r="H14" s="29">
         <f>F14-G14</f>
         <v/>
       </c>
-      <c r="I14" s="26" t="n">
+      <c r="I14" s="28" t="n">
         <v>18756</v>
       </c>
-      <c r="J14" s="26" t="n">
+      <c r="J14" s="28" t="n">
         <v>2956</v>
       </c>
-      <c r="K14" s="27">
+      <c r="K14" s="29">
         <f>I14-J14</f>
         <v/>
       </c>
-      <c r="L14" s="26" t="n">
+      <c r="L14" s="28" t="n">
         <v>13968</v>
       </c>
-      <c r="M14" s="26" t="n">
+      <c r="M14" s="28" t="n">
         <v>3302</v>
       </c>
-      <c r="N14" s="26" t="n">
+      <c r="N14" s="28" t="n">
         <v>10666</v>
       </c>
-      <c r="O14" s="26" t="n">
+      <c r="O14" s="28" t="n">
         <v>20952</v>
       </c>
-      <c r="P14" s="26" t="n">
+      <c r="P14" s="28" t="n">
         <v>3302</v>
       </c>
-      <c r="Q14" s="27">
+      <c r="Q14" s="29">
         <f>O14-P14</f>
         <v/>
       </c>
@@ -4346,7 +4636,7 @@
       <c r="U14" s="23" t="n">
         <v>21</v>
       </c>
-      <c r="V14" s="27" t="inlineStr">
+      <c r="V14" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4376,42 +4666,42 @@
       <c r="E15" s="23" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="28" t="n">
         <v>21816</v>
       </c>
-      <c r="G15" s="26" t="n">
+      <c r="G15" s="28" t="n">
         <v>20200</v>
       </c>
-      <c r="H15" s="27">
+      <c r="H15" s="29">
         <f>F15-G15</f>
         <v/>
       </c>
-      <c r="I15" s="26" t="n">
+      <c r="I15" s="28" t="n">
         <v>32722</v>
       </c>
-      <c r="J15" s="26" t="n">
+      <c r="J15" s="28" t="n">
         <v>20200</v>
       </c>
-      <c r="K15" s="27">
+      <c r="K15" s="29">
         <f>I15-J15</f>
         <v/>
       </c>
-      <c r="L15" s="26" t="n">
+      <c r="L15" s="28" t="n">
         <v>24370</v>
       </c>
-      <c r="M15" s="26" t="n">
+      <c r="M15" s="28" t="n">
         <v>22566</v>
       </c>
-      <c r="N15" s="26" t="n">
+      <c r="N15" s="28" t="n">
         <v>1804</v>
       </c>
-      <c r="O15" s="26" t="n">
+      <c r="O15" s="28" t="n">
         <v>36556</v>
       </c>
-      <c r="P15" s="26" t="n">
+      <c r="P15" s="28" t="n">
         <v>22566</v>
       </c>
-      <c r="Q15" s="27">
+      <c r="Q15" s="29">
         <f>O15-P15</f>
         <v/>
       </c>
@@ -4427,7 +4717,7 @@
       <c r="U15" s="23" t="n">
         <v>43</v>
       </c>
-      <c r="V15" s="27" t="inlineStr">
+      <c r="V15" s="29" t="inlineStr">
         <is>
           <t>Standard</t>
         </is>
@@ -4457,42 +4747,42 @@
       <c r="E16" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F16" s="28" t="n">
+      <c r="F16" s="30" t="n">
         <v>1296</v>
       </c>
-      <c r="G16" s="28" t="n">
+      <c r="G16" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="H16" s="27">
+      <c r="H16" s="29">
         <f>F16-G16</f>
         <v/>
       </c>
-      <c r="I16" s="28" t="n">
+      <c r="I16" s="30" t="n">
         <v>1944</v>
       </c>
-      <c r="J16" s="28" t="n">
+      <c r="J16" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="K16" s="27">
+      <c r="K16" s="29">
         <f>I16-J16</f>
         <v/>
       </c>
-      <c r="L16" s="28" t="n">
+      <c r="L16" s="30" t="n">
         <v>1838</v>
       </c>
-      <c r="M16" s="28" t="n">
+      <c r="M16" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="N16" s="28" t="n">
+      <c r="N16" s="30" t="n">
         <v>138</v>
       </c>
-      <c r="O16" s="28" t="n">
+      <c r="O16" s="30" t="n">
         <v>2756</v>
       </c>
-      <c r="P16" s="28" t="n">
+      <c r="P16" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="Q16" s="27">
+      <c r="Q16" s="29">
         <f>O16-P16</f>
         <v/>
       </c>
@@ -4538,42 +4828,42 @@
       <c r="E17" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="F17" s="28" t="n">
+      <c r="F17" s="30" t="n">
         <v>1296</v>
       </c>
-      <c r="G17" s="28" t="n">
+      <c r="G17" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="H17" s="27">
+      <c r="H17" s="29">
         <f>F17-G17</f>
         <v/>
       </c>
-      <c r="I17" s="28" t="n">
+      <c r="I17" s="30" t="n">
         <v>1944</v>
       </c>
-      <c r="J17" s="28" t="n">
+      <c r="J17" s="30" t="n">
         <v>1200</v>
       </c>
-      <c r="K17" s="27">
+      <c r="K17" s="29">
         <f>I17-J17</f>
         <v/>
       </c>
-      <c r="L17" s="28" t="n">
+      <c r="L17" s="30" t="n">
         <v>1838</v>
       </c>
-      <c r="M17" s="28" t="n">
+      <c r="M17" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="N17" s="28" t="n">
+      <c r="N17" s="30" t="n">
         <v>138</v>
       </c>
-      <c r="O17" s="28" t="n">
+      <c r="O17" s="30" t="n">
         <v>2756</v>
       </c>
-      <c r="P17" s="28" t="n">
+      <c r="P17" s="30" t="n">
         <v>1700</v>
       </c>
-      <c r="Q17" s="27">
+      <c r="Q17" s="29">
         <f>O17-P17</f>
         <v/>
       </c>
@@ -5449,7 +5739,7 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="6" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
@@ -5460,7 +5750,7 @@
           <t>PS_Prod — Production Placement Score</t>
         </is>
       </c>
-      <c r="T1" s="29" t="inlineStr">
+      <c r="T1" s="25" t="inlineStr">
         <is>
           <t>PROD WINNER</t>
         </is>
@@ -5608,47 +5898,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G4" s="30">
+      <c r="G4" s="31">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!F4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="30">
+      <c r="H4" s="31">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="30">
+      <c r="I4" s="31">
         <f>IFERROR(Capacity_Usage!K4/Capacity_Usage!I4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="30">
+      <c r="J4" s="31">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="30">
+      <c r="K4" s="31">
         <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="30">
+      <c r="L4" s="31">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="30">
+      <c r="M4" s="31">
         <f>IFERROR(Capacity_Usage!T4,0)</f>
         <v/>
       </c>
-      <c r="N4" s="30">
+      <c r="N4" s="31">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="30">
+      <c r="O4" s="31">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="30">
+      <c r="P4" s="31">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="30">
+      <c r="Q4" s="31">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -5665,7 +5955,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U4" s="31">
+      <c r="U4" s="32">
         <f>IF(Setup!$B$8&lt;&gt;"",INDEX(Q4:Q17,MATCH(Setup!$B$8,A4:A17,0)),IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -5695,47 +5985,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="31">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!F5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="31">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="31">
         <f>IFERROR(Capacity_Usage!K5/Capacity_Usage!I5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="31">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="30">
+      <c r="K5" s="31">
         <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="30">
+      <c r="L5" s="31">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="30">
+      <c r="M5" s="31">
         <f>IFERROR(Capacity_Usage!T5,0)</f>
         <v/>
       </c>
-      <c r="N5" s="30">
+      <c r="N5" s="31">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="30">
+      <c r="O5" s="31">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="30">
+      <c r="P5" s="31">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="30">
+      <c r="Q5" s="31">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -5773,47 +6063,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G6" s="30">
+      <c r="G6" s="31">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!F6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="30">
+      <c r="H6" s="31">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="30">
+      <c r="I6" s="31">
         <f>IFERROR(Capacity_Usage!K6/Capacity_Usage!I6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="31">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="30">
+      <c r="K6" s="31">
         <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="30">
+      <c r="L6" s="31">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="30">
+      <c r="M6" s="31">
         <f>IFERROR(Capacity_Usage!T6,0)</f>
         <v/>
       </c>
-      <c r="N6" s="30">
+      <c r="N6" s="31">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="30">
+      <c r="O6" s="31">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="30">
+      <c r="P6" s="31">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="30">
+      <c r="Q6" s="31">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -5851,47 +6141,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G7" s="30">
+      <c r="G7" s="31">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!F7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="31">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="30">
+      <c r="I7" s="31">
         <f>IFERROR(Capacity_Usage!K7/Capacity_Usage!I7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="31">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="30">
+      <c r="K7" s="31">
         <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
         <v/>
       </c>
-      <c r="L7" s="30">
+      <c r="L7" s="31">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="30">
+      <c r="M7" s="31">
         <f>IFERROR(Capacity_Usage!T7,0)</f>
         <v/>
       </c>
-      <c r="N7" s="30">
+      <c r="N7" s="31">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="30">
+      <c r="O7" s="31">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="30">
+      <c r="P7" s="31">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="30">
+      <c r="Q7" s="31">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -5929,47 +6219,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G8" s="30">
+      <c r="G8" s="31">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!F8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="31">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="30">
+      <c r="I8" s="31">
         <f>IFERROR(Capacity_Usage!K8/Capacity_Usage!I8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="30">
+      <c r="J8" s="31">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="30">
+      <c r="K8" s="31">
         <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
         <v/>
       </c>
-      <c r="L8" s="30">
+      <c r="L8" s="31">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="30">
+      <c r="M8" s="31">
         <f>IFERROR(Capacity_Usage!T8,0)</f>
         <v/>
       </c>
-      <c r="N8" s="30">
+      <c r="N8" s="31">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="30">
+      <c r="O8" s="31">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="30">
+      <c r="P8" s="31">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="30">
+      <c r="Q8" s="31">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -6007,47 +6297,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G9" s="30">
+      <c r="G9" s="31">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!F9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="31">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="30">
+      <c r="I9" s="31">
         <f>IFERROR(Capacity_Usage!K9/Capacity_Usage!I9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="30">
+      <c r="J9" s="31">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="30">
+      <c r="K9" s="31">
         <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
         <v/>
       </c>
-      <c r="L9" s="30">
+      <c r="L9" s="31">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="30">
+      <c r="M9" s="31">
         <f>IFERROR(Capacity_Usage!T9,0)</f>
         <v/>
       </c>
-      <c r="N9" s="30">
+      <c r="N9" s="31">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="30">
+      <c r="O9" s="31">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="30">
+      <c r="P9" s="31">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="30">
+      <c r="Q9" s="31">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -6085,47 +6375,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G10" s="30">
+      <c r="G10" s="31">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!F10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="30">
+      <c r="H10" s="31">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="30">
+      <c r="I10" s="31">
         <f>IFERROR(Capacity_Usage!K10/Capacity_Usage!I10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="30">
+      <c r="J10" s="31">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="31">
         <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
         <v/>
       </c>
-      <c r="L10" s="30">
+      <c r="L10" s="31">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="30">
+      <c r="M10" s="31">
         <f>IFERROR(Capacity_Usage!T10,0)</f>
         <v/>
       </c>
-      <c r="N10" s="30">
+      <c r="N10" s="31">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="30">
+      <c r="O10" s="31">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="30">
+      <c r="P10" s="31">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="30">
+      <c r="Q10" s="31">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -6163,47 +6453,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G11" s="30">
+      <c r="G11" s="31">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!F11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="30">
+      <c r="H11" s="31">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="30">
+      <c r="I11" s="31">
         <f>IFERROR(Capacity_Usage!K11/Capacity_Usage!I11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="31">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="30">
+      <c r="K11" s="31">
         <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="30">
+      <c r="L11" s="31">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="30">
+      <c r="M11" s="31">
         <f>IFERROR(Capacity_Usage!T11,0)</f>
         <v/>
       </c>
-      <c r="N11" s="30">
+      <c r="N11" s="31">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="30">
+      <c r="O11" s="31">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="30">
+      <c r="P11" s="31">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="30">
+      <c r="Q11" s="31">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -6241,47 +6531,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G12" s="30">
+      <c r="G12" s="31">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!F12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="31">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="30">
+      <c r="I12" s="31">
         <f>IFERROR(Capacity_Usage!K12/Capacity_Usage!I12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="31">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="30">
+      <c r="K12" s="31">
         <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
         <v/>
       </c>
-      <c r="L12" s="30">
+      <c r="L12" s="31">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="30">
+      <c r="M12" s="31">
         <f>IFERROR(Capacity_Usage!T12,0)</f>
         <v/>
       </c>
-      <c r="N12" s="30">
+      <c r="N12" s="31">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="30">
+      <c r="O12" s="31">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="30">
+      <c r="P12" s="31">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="30">
+      <c r="Q12" s="31">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -6319,47 +6609,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G13" s="30">
+      <c r="G13" s="31">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!F13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="30">
+      <c r="H13" s="31">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="30">
+      <c r="I13" s="31">
         <f>IFERROR(Capacity_Usage!K13/Capacity_Usage!I13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="31">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="30">
+      <c r="K13" s="31">
         <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
         <v/>
       </c>
-      <c r="L13" s="30">
+      <c r="L13" s="31">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="30">
+      <c r="M13" s="31">
         <f>IFERROR(Capacity_Usage!T13,0)</f>
         <v/>
       </c>
-      <c r="N13" s="30">
+      <c r="N13" s="31">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="30">
+      <c r="O13" s="31">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="30">
+      <c r="P13" s="31">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="30">
+      <c r="Q13" s="31">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -6397,47 +6687,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="31">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!F14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="31">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="31">
         <f>IFERROR(Capacity_Usage!K14/Capacity_Usage!I14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="31">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="30">
+      <c r="K14" s="31">
         <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
         <v/>
       </c>
-      <c r="L14" s="30">
+      <c r="L14" s="31">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="30">
+      <c r="M14" s="31">
         <f>IFERROR(Capacity_Usage!T14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="30">
+      <c r="N14" s="31">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="30">
+      <c r="O14" s="31">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="30">
+      <c r="P14" s="31">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="30">
+      <c r="Q14" s="31">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -6475,47 +6765,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="31">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!F15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="31">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="31">
         <f>IFERROR(Capacity_Usage!K15/Capacity_Usage!I15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="31">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="30">
+      <c r="K15" s="31">
         <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
         <v/>
       </c>
-      <c r="L15" s="30">
+      <c r="L15" s="31">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="30">
+      <c r="M15" s="31">
         <f>IFERROR(Capacity_Usage!T15,0)</f>
         <v/>
       </c>
-      <c r="N15" s="30">
+      <c r="N15" s="31">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="30">
+      <c r="O15" s="31">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="30">
+      <c r="P15" s="31">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="30">
+      <c r="Q15" s="31">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -6553,47 +6843,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G16" s="30">
+      <c r="G16" s="31">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!F16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="31">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="31">
         <f>IFERROR(Capacity_Usage!K16/Capacity_Usage!I16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="31">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="30">
+      <c r="K16" s="31">
         <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
         <v/>
       </c>
-      <c r="L16" s="30">
+      <c r="L16" s="31">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="30">
+      <c r="M16" s="31">
         <f>IFERROR(Capacity_Usage!T16,0)</f>
         <v/>
       </c>
-      <c r="N16" s="30">
+      <c r="N16" s="31">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="30">
+      <c r="O16" s="31">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="30">
+      <c r="P16" s="31">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="30">
+      <c r="Q16" s="31">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -6631,47 +6921,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G17" s="30">
+      <c r="G17" s="31">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!F17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="31">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="31">
         <f>IFERROR(Capacity_Usage!K17/Capacity_Usage!I17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="31">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="30">
+      <c r="K17" s="31">
         <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
         <v/>
       </c>
-      <c r="L17" s="30">
+      <c r="L17" s="31">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="30">
+      <c r="M17" s="31">
         <f>IFERROR(Capacity_Usage!T17,0)</f>
         <v/>
       </c>
-      <c r="N17" s="30">
+      <c r="N17" s="31">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="30">
+      <c r="O17" s="31">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="31">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="30">
+      <c r="Q17" s="31">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>
@@ -6717,7 +7007,7 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="6" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
@@ -6728,7 +7018,7 @@
           <t>PS_NonProd — CVAL Placement Score  (δ duplicates α — known design gap)</t>
         </is>
       </c>
-      <c r="T1" s="29" t="inlineStr">
+      <c r="T1" s="25" t="inlineStr">
         <is>
           <t>CVAL WINNER</t>
         </is>
@@ -6846,7 +7136,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U3" s="31">
+      <c r="U3" s="32">
         <f>IF(Setup!$B$3="Middle East",Scoring_Prod!$U$4,IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -6876,47 +7166,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G4" s="30">
+      <c r="G4" s="31">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!L4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="30">
+      <c r="H4" s="31">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="30">
+      <c r="I4" s="31">
         <f>IFERROR(Capacity_Usage!Q4/Capacity_Usage!O4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="30">
+      <c r="J4" s="31">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="30">
+      <c r="K4" s="31">
         <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="30">
+      <c r="L4" s="31">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="30">
+      <c r="M4" s="31">
         <f>IFERROR(Capacity_Usage!N4/Capacity_Usage!L4,0)</f>
         <v/>
       </c>
-      <c r="N4" s="30">
+      <c r="N4" s="31">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="30">
+      <c r="O4" s="31">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="30">
+      <c r="P4" s="31">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="30">
+      <c r="Q4" s="31">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -6954,47 +7244,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="31">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!L5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="31">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="31">
         <f>IFERROR(Capacity_Usage!Q5/Capacity_Usage!O5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="31">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="30">
+      <c r="K5" s="31">
         <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="30">
+      <c r="L5" s="31">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="30">
+      <c r="M5" s="31">
         <f>IFERROR(Capacity_Usage!N5/Capacity_Usage!L5,0)</f>
         <v/>
       </c>
-      <c r="N5" s="30">
+      <c r="N5" s="31">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="30">
+      <c r="O5" s="31">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="30">
+      <c r="P5" s="31">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="30">
+      <c r="Q5" s="31">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -7032,47 +7322,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G6" s="30">
+      <c r="G6" s="31">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!L6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="30">
+      <c r="H6" s="31">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="30">
+      <c r="I6" s="31">
         <f>IFERROR(Capacity_Usage!Q6/Capacity_Usage!O6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="31">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="30">
+      <c r="K6" s="31">
         <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="30">
+      <c r="L6" s="31">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="30">
+      <c r="M6" s="31">
         <f>IFERROR(Capacity_Usage!N6/Capacity_Usage!L6,0)</f>
         <v/>
       </c>
-      <c r="N6" s="30">
+      <c r="N6" s="31">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="30">
+      <c r="O6" s="31">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="30">
+      <c r="P6" s="31">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="30">
+      <c r="Q6" s="31">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -7110,47 +7400,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G7" s="30">
+      <c r="G7" s="31">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!L7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="31">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="30">
+      <c r="I7" s="31">
         <f>IFERROR(Capacity_Usage!Q7/Capacity_Usage!O7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="31">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="30">
+      <c r="K7" s="31">
         <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
         <v/>
       </c>
-      <c r="L7" s="30">
+      <c r="L7" s="31">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="30">
+      <c r="M7" s="31">
         <f>IFERROR(Capacity_Usage!N7/Capacity_Usage!L7,0)</f>
         <v/>
       </c>
-      <c r="N7" s="30">
+      <c r="N7" s="31">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="30">
+      <c r="O7" s="31">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="30">
+      <c r="P7" s="31">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="30">
+      <c r="Q7" s="31">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -7188,47 +7478,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G8" s="30">
+      <c r="G8" s="31">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!L8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="31">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="30">
+      <c r="I8" s="31">
         <f>IFERROR(Capacity_Usage!Q8/Capacity_Usage!O8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="30">
+      <c r="J8" s="31">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="30">
+      <c r="K8" s="31">
         <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
         <v/>
       </c>
-      <c r="L8" s="30">
+      <c r="L8" s="31">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="30">
+      <c r="M8" s="31">
         <f>IFERROR(Capacity_Usage!N8/Capacity_Usage!L8,0)</f>
         <v/>
       </c>
-      <c r="N8" s="30">
+      <c r="N8" s="31">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="30">
+      <c r="O8" s="31">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="30">
+      <c r="P8" s="31">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="30">
+      <c r="Q8" s="31">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -7266,47 +7556,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G9" s="30">
+      <c r="G9" s="31">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!L9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="31">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="30">
+      <c r="I9" s="31">
         <f>IFERROR(Capacity_Usage!Q9/Capacity_Usage!O9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="30">
+      <c r="J9" s="31">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="30">
+      <c r="K9" s="31">
         <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
         <v/>
       </c>
-      <c r="L9" s="30">
+      <c r="L9" s="31">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="30">
+      <c r="M9" s="31">
         <f>IFERROR(Capacity_Usage!N9/Capacity_Usage!L9,0)</f>
         <v/>
       </c>
-      <c r="N9" s="30">
+      <c r="N9" s="31">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="30">
+      <c r="O9" s="31">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="30">
+      <c r="P9" s="31">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="30">
+      <c r="Q9" s="31">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -7344,47 +7634,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G10" s="30">
+      <c r="G10" s="31">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!L10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="30">
+      <c r="H10" s="31">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="30">
+      <c r="I10" s="31">
         <f>IFERROR(Capacity_Usage!Q10/Capacity_Usage!O10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="30">
+      <c r="J10" s="31">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="31">
         <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
         <v/>
       </c>
-      <c r="L10" s="30">
+      <c r="L10" s="31">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="30">
+      <c r="M10" s="31">
         <f>IFERROR(Capacity_Usage!N10/Capacity_Usage!L10,0)</f>
         <v/>
       </c>
-      <c r="N10" s="30">
+      <c r="N10" s="31">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="30">
+      <c r="O10" s="31">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="30">
+      <c r="P10" s="31">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="30">
+      <c r="Q10" s="31">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -7422,47 +7712,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G11" s="30">
+      <c r="G11" s="31">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!L11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="30">
+      <c r="H11" s="31">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="30">
+      <c r="I11" s="31">
         <f>IFERROR(Capacity_Usage!Q11/Capacity_Usage!O11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="31">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="30">
+      <c r="K11" s="31">
         <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="30">
+      <c r="L11" s="31">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="30">
+      <c r="M11" s="31">
         <f>IFERROR(Capacity_Usage!N11/Capacity_Usage!L11,0)</f>
         <v/>
       </c>
-      <c r="N11" s="30">
+      <c r="N11" s="31">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="30">
+      <c r="O11" s="31">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="30">
+      <c r="P11" s="31">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="30">
+      <c r="Q11" s="31">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -7500,47 +7790,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G12" s="30">
+      <c r="G12" s="31">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!L12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="31">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="30">
+      <c r="I12" s="31">
         <f>IFERROR(Capacity_Usage!Q12/Capacity_Usage!O12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="31">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="30">
+      <c r="K12" s="31">
         <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
         <v/>
       </c>
-      <c r="L12" s="30">
+      <c r="L12" s="31">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="30">
+      <c r="M12" s="31">
         <f>IFERROR(Capacity_Usage!N12/Capacity_Usage!L12,0)</f>
         <v/>
       </c>
-      <c r="N12" s="30">
+      <c r="N12" s="31">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="30">
+      <c r="O12" s="31">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="30">
+      <c r="P12" s="31">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="30">
+      <c r="Q12" s="31">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -7578,47 +7868,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G13" s="30">
+      <c r="G13" s="31">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!L13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="30">
+      <c r="H13" s="31">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="30">
+      <c r="I13" s="31">
         <f>IFERROR(Capacity_Usage!Q13/Capacity_Usage!O13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="31">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="30">
+      <c r="K13" s="31">
         <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
         <v/>
       </c>
-      <c r="L13" s="30">
+      <c r="L13" s="31">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="30">
+      <c r="M13" s="31">
         <f>IFERROR(Capacity_Usage!N13/Capacity_Usage!L13,0)</f>
         <v/>
       </c>
-      <c r="N13" s="30">
+      <c r="N13" s="31">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="30">
+      <c r="O13" s="31">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="30">
+      <c r="P13" s="31">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="30">
+      <c r="Q13" s="31">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -7656,47 +7946,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="31">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!L14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="31">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="31">
         <f>IFERROR(Capacity_Usage!Q14/Capacity_Usage!O14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="31">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="30">
+      <c r="K14" s="31">
         <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
         <v/>
       </c>
-      <c r="L14" s="30">
+      <c r="L14" s="31">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="30">
+      <c r="M14" s="31">
         <f>IFERROR(Capacity_Usage!N14/Capacity_Usage!L14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="30">
+      <c r="N14" s="31">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="30">
+      <c r="O14" s="31">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="30">
+      <c r="P14" s="31">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="30">
+      <c r="Q14" s="31">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -7734,47 +8024,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="31">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!L15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="31">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="31">
         <f>IFERROR(Capacity_Usage!Q15/Capacity_Usage!O15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="31">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="30">
+      <c r="K15" s="31">
         <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
         <v/>
       </c>
-      <c r="L15" s="30">
+      <c r="L15" s="31">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="30">
+      <c r="M15" s="31">
         <f>IFERROR(Capacity_Usage!N15/Capacity_Usage!L15,0)</f>
         <v/>
       </c>
-      <c r="N15" s="30">
+      <c r="N15" s="31">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="30">
+      <c r="O15" s="31">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="30">
+      <c r="P15" s="31">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="30">
+      <c r="Q15" s="31">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -7812,47 +8102,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G16" s="30">
+      <c r="G16" s="31">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!L16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="31">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="31">
         <f>IFERROR(Capacity_Usage!Q16/Capacity_Usage!O16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="31">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="30">
+      <c r="K16" s="31">
         <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
         <v/>
       </c>
-      <c r="L16" s="30">
+      <c r="L16" s="31">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="30">
+      <c r="M16" s="31">
         <f>IFERROR(Capacity_Usage!N16/Capacity_Usage!L16,0)</f>
         <v/>
       </c>
-      <c r="N16" s="30">
+      <c r="N16" s="31">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="30">
+      <c r="O16" s="31">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="30">
+      <c r="P16" s="31">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="30">
+      <c r="Q16" s="31">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -7890,47 +8180,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G17" s="30">
+      <c r="G17" s="31">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!L17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="31">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="31">
         <f>IFERROR(Capacity_Usage!Q17/Capacity_Usage!O17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="31">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="30">
+      <c r="K17" s="31">
         <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
         <v/>
       </c>
-      <c r="L17" s="30">
+      <c r="L17" s="31">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="30">
+      <c r="M17" s="31">
         <f>IFERROR(Capacity_Usage!N17/Capacity_Usage!L17,0)</f>
         <v/>
       </c>
-      <c r="N17" s="30">
+      <c r="N17" s="31">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="30">
+      <c r="O17" s="31">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="31">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="30">
+      <c r="Q17" s="31">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>
@@ -7975,7 +8265,7 @@
     <col width="9" customWidth="1" min="16" max="16"/>
     <col width="9" customWidth="1" min="17" max="17"/>
     <col width="9" customWidth="1" min="18" max="18"/>
-    <col width="6" customWidth="1" min="19" max="19"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
     <col width="16" customWidth="1" min="20" max="20"/>
     <col width="18" customWidth="1" min="21" max="21"/>
   </cols>
@@ -7986,7 +8276,7 @@
           <t>PS_DR — DR Placement Score  (Middle East scores EU regions cross-geo)</t>
         </is>
       </c>
-      <c r="T1" s="29" t="inlineStr">
+      <c r="T1" s="25" t="inlineStr">
         <is>
           <t>DR WINNER</t>
         </is>
@@ -8104,7 +8394,7 @@
           <t>Score</t>
         </is>
       </c>
-      <c r="U3" s="31">
+      <c r="U3" s="32">
         <f>IF(Setup!$B$10="2-region",Scoring_CVAL!$U$3,IF(MAX(R4:R17)&lt;0,"",MAX(R4:R17)))</f>
         <v/>
       </c>
@@ -8134,47 +8424,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C4),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C4,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G4" s="30">
+      <c r="G4" s="31">
         <f>IFERROR(Capacity_Usage!S4/Capacity_Usage!R4,0)</f>
         <v/>
       </c>
-      <c r="H4" s="30">
+      <c r="H4" s="31">
         <f>MIN(MAX(G4,0),1)</f>
         <v/>
       </c>
-      <c r="I4" s="30">
+      <c r="I4" s="31">
         <f>IFERROR(Capacity_Usage!Q4/Capacity_Usage!O4,0)</f>
         <v/>
       </c>
-      <c r="J4" s="30">
+      <c r="J4" s="31">
         <f>MIN(MAX(I4,0),1)</f>
         <v/>
       </c>
-      <c r="K4" s="30">
+      <c r="K4" s="31">
         <f>IFERROR(1-Capacity_Usage!U4/F4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="30">
+      <c r="L4" s="31">
         <f>MIN(MAX(K4,0),1)</f>
         <v/>
       </c>
-      <c r="M4" s="30">
+      <c r="M4" s="31">
         <f>IFERROR(Capacity_Usage!T4/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N4" s="30">
+      <c r="N4" s="31">
         <f>MIN(MAX(M4,0),1)</f>
         <v/>
       </c>
-      <c r="O4" s="30">
+      <c r="O4" s="31">
         <f>Capacity_Usage!E4/3</f>
         <v/>
       </c>
-      <c r="P4" s="30">
+      <c r="P4" s="31">
         <f>MIN(MAX(O4,0),1)</f>
         <v/>
       </c>
-      <c r="Q4" s="30">
+      <c r="Q4" s="31">
         <f>Policy!$B$2*H4+Policy!$B$3*J4+Policy!$B$4*L4+Policy!$B$5*N4+Policy!$B$6*P4</f>
         <v/>
       </c>
@@ -8212,47 +8502,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C5),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C5,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G5" s="30">
+      <c r="G5" s="31">
         <f>IFERROR(Capacity_Usage!S5/Capacity_Usage!R5,0)</f>
         <v/>
       </c>
-      <c r="H5" s="30">
+      <c r="H5" s="31">
         <f>MIN(MAX(G5,0),1)</f>
         <v/>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="31">
         <f>IFERROR(Capacity_Usage!Q5/Capacity_Usage!O5,0)</f>
         <v/>
       </c>
-      <c r="J5" s="30">
+      <c r="J5" s="31">
         <f>MIN(MAX(I5,0),1)</f>
         <v/>
       </c>
-      <c r="K5" s="30">
+      <c r="K5" s="31">
         <f>IFERROR(1-Capacity_Usage!U5/F5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="30">
+      <c r="L5" s="31">
         <f>MIN(MAX(K5,0),1)</f>
         <v/>
       </c>
-      <c r="M5" s="30">
+      <c r="M5" s="31">
         <f>IFERROR(Capacity_Usage!T5/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N5" s="30">
+      <c r="N5" s="31">
         <f>MIN(MAX(M5,0),1)</f>
         <v/>
       </c>
-      <c r="O5" s="30">
+      <c r="O5" s="31">
         <f>Capacity_Usage!E5/3</f>
         <v/>
       </c>
-      <c r="P5" s="30">
+      <c r="P5" s="31">
         <f>MIN(MAX(O5,0),1)</f>
         <v/>
       </c>
-      <c r="Q5" s="30">
+      <c r="Q5" s="31">
         <f>Policy!$B$2*H5+Policy!$B$3*J5+Policy!$B$4*L5+Policy!$B$5*N5+Policy!$B$6*P5</f>
         <v/>
       </c>
@@ -8290,47 +8580,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C6),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C6,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G6" s="30">
+      <c r="G6" s="31">
         <f>IFERROR(Capacity_Usage!S6/Capacity_Usage!R6,0)</f>
         <v/>
       </c>
-      <c r="H6" s="30">
+      <c r="H6" s="31">
         <f>MIN(MAX(G6,0),1)</f>
         <v/>
       </c>
-      <c r="I6" s="30">
+      <c r="I6" s="31">
         <f>IFERROR(Capacity_Usage!Q6/Capacity_Usage!O6,0)</f>
         <v/>
       </c>
-      <c r="J6" s="30">
+      <c r="J6" s="31">
         <f>MIN(MAX(I6,0),1)</f>
         <v/>
       </c>
-      <c r="K6" s="30">
+      <c r="K6" s="31">
         <f>IFERROR(1-Capacity_Usage!U6/F6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="30">
+      <c r="L6" s="31">
         <f>MIN(MAX(K6,0),1)</f>
         <v/>
       </c>
-      <c r="M6" s="30">
+      <c r="M6" s="31">
         <f>IFERROR(Capacity_Usage!T6/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N6" s="30">
+      <c r="N6" s="31">
         <f>MIN(MAX(M6,0),1)</f>
         <v/>
       </c>
-      <c r="O6" s="30">
+      <c r="O6" s="31">
         <f>Capacity_Usage!E6/3</f>
         <v/>
       </c>
-      <c r="P6" s="30">
+      <c r="P6" s="31">
         <f>MIN(MAX(O6,0),1)</f>
         <v/>
       </c>
-      <c r="Q6" s="30">
+      <c r="Q6" s="31">
         <f>Policy!$B$2*H6+Policy!$B$3*J6+Policy!$B$4*L6+Policy!$B$5*N6+Policy!$B$6*P6</f>
         <v/>
       </c>
@@ -8368,47 +8658,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C7),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C7,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G7" s="30">
+      <c r="G7" s="31">
         <f>IFERROR(Capacity_Usage!S7/Capacity_Usage!R7,0)</f>
         <v/>
       </c>
-      <c r="H7" s="30">
+      <c r="H7" s="31">
         <f>MIN(MAX(G7,0),1)</f>
         <v/>
       </c>
-      <c r="I7" s="30">
+      <c r="I7" s="31">
         <f>IFERROR(Capacity_Usage!Q7/Capacity_Usage!O7,0)</f>
         <v/>
       </c>
-      <c r="J7" s="30">
+      <c r="J7" s="31">
         <f>MIN(MAX(I7,0),1)</f>
         <v/>
       </c>
-      <c r="K7" s="30">
+      <c r="K7" s="31">
         <f>IFERROR(1-Capacity_Usage!U7/F7,0)</f>
         <v/>
       </c>
-      <c r="L7" s="30">
+      <c r="L7" s="31">
         <f>MIN(MAX(K7,0),1)</f>
         <v/>
       </c>
-      <c r="M7" s="30">
+      <c r="M7" s="31">
         <f>IFERROR(Capacity_Usage!T7/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N7" s="30">
+      <c r="N7" s="31">
         <f>MIN(MAX(M7,0),1)</f>
         <v/>
       </c>
-      <c r="O7" s="30">
+      <c r="O7" s="31">
         <f>Capacity_Usage!E7/3</f>
         <v/>
       </c>
-      <c r="P7" s="30">
+      <c r="P7" s="31">
         <f>MIN(MAX(O7,0),1)</f>
         <v/>
       </c>
-      <c r="Q7" s="30">
+      <c r="Q7" s="31">
         <f>Policy!$B$2*H7+Policy!$B$3*J7+Policy!$B$4*L7+Policy!$B$5*N7+Policy!$B$6*P7</f>
         <v/>
       </c>
@@ -8446,47 +8736,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C8),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C8,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G8" s="30">
+      <c r="G8" s="31">
         <f>IFERROR(Capacity_Usage!S8/Capacity_Usage!R8,0)</f>
         <v/>
       </c>
-      <c r="H8" s="30">
+      <c r="H8" s="31">
         <f>MIN(MAX(G8,0),1)</f>
         <v/>
       </c>
-      <c r="I8" s="30">
+      <c r="I8" s="31">
         <f>IFERROR(Capacity_Usage!Q8/Capacity_Usage!O8,0)</f>
         <v/>
       </c>
-      <c r="J8" s="30">
+      <c r="J8" s="31">
         <f>MIN(MAX(I8,0),1)</f>
         <v/>
       </c>
-      <c r="K8" s="30">
+      <c r="K8" s="31">
         <f>IFERROR(1-Capacity_Usage!U8/F8,0)</f>
         <v/>
       </c>
-      <c r="L8" s="30">
+      <c r="L8" s="31">
         <f>MIN(MAX(K8,0),1)</f>
         <v/>
       </c>
-      <c r="M8" s="30">
+      <c r="M8" s="31">
         <f>IFERROR(Capacity_Usage!T8/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N8" s="30">
+      <c r="N8" s="31">
         <f>MIN(MAX(M8,0),1)</f>
         <v/>
       </c>
-      <c r="O8" s="30">
+      <c r="O8" s="31">
         <f>Capacity_Usage!E8/3</f>
         <v/>
       </c>
-      <c r="P8" s="30">
+      <c r="P8" s="31">
         <f>MIN(MAX(O8,0),1)</f>
         <v/>
       </c>
-      <c r="Q8" s="30">
+      <c r="Q8" s="31">
         <f>Policy!$B$2*H8+Policy!$B$3*J8+Policy!$B$4*L8+Policy!$B$5*N8+Policy!$B$6*P8</f>
         <v/>
       </c>
@@ -8524,47 +8814,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C9),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C9,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G9" s="30">
+      <c r="G9" s="31">
         <f>IFERROR(Capacity_Usage!S9/Capacity_Usage!R9,0)</f>
         <v/>
       </c>
-      <c r="H9" s="30">
+      <c r="H9" s="31">
         <f>MIN(MAX(G9,0),1)</f>
         <v/>
       </c>
-      <c r="I9" s="30">
+      <c r="I9" s="31">
         <f>IFERROR(Capacity_Usage!Q9/Capacity_Usage!O9,0)</f>
         <v/>
       </c>
-      <c r="J9" s="30">
+      <c r="J9" s="31">
         <f>MIN(MAX(I9,0),1)</f>
         <v/>
       </c>
-      <c r="K9" s="30">
+      <c r="K9" s="31">
         <f>IFERROR(1-Capacity_Usage!U9/F9,0)</f>
         <v/>
       </c>
-      <c r="L9" s="30">
+      <c r="L9" s="31">
         <f>MIN(MAX(K9,0),1)</f>
         <v/>
       </c>
-      <c r="M9" s="30">
+      <c r="M9" s="31">
         <f>IFERROR(Capacity_Usage!T9/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N9" s="30">
+      <c r="N9" s="31">
         <f>MIN(MAX(M9,0),1)</f>
         <v/>
       </c>
-      <c r="O9" s="30">
+      <c r="O9" s="31">
         <f>Capacity_Usage!E9/3</f>
         <v/>
       </c>
-      <c r="P9" s="30">
+      <c r="P9" s="31">
         <f>MIN(MAX(O9,0),1)</f>
         <v/>
       </c>
-      <c r="Q9" s="30">
+      <c r="Q9" s="31">
         <f>Policy!$B$2*H9+Policy!$B$3*J9+Policy!$B$4*L9+Policy!$B$5*N9+Policy!$B$6*P9</f>
         <v/>
       </c>
@@ -8602,47 +8892,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C10),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C10,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G10" s="30">
+      <c r="G10" s="31">
         <f>IFERROR(Capacity_Usage!S10/Capacity_Usage!R10,0)</f>
         <v/>
       </c>
-      <c r="H10" s="30">
+      <c r="H10" s="31">
         <f>MIN(MAX(G10,0),1)</f>
         <v/>
       </c>
-      <c r="I10" s="30">
+      <c r="I10" s="31">
         <f>IFERROR(Capacity_Usage!Q10/Capacity_Usage!O10,0)</f>
         <v/>
       </c>
-      <c r="J10" s="30">
+      <c r="J10" s="31">
         <f>MIN(MAX(I10,0),1)</f>
         <v/>
       </c>
-      <c r="K10" s="30">
+      <c r="K10" s="31">
         <f>IFERROR(1-Capacity_Usage!U10/F10,0)</f>
         <v/>
       </c>
-      <c r="L10" s="30">
+      <c r="L10" s="31">
         <f>MIN(MAX(K10,0),1)</f>
         <v/>
       </c>
-      <c r="M10" s="30">
+      <c r="M10" s="31">
         <f>IFERROR(Capacity_Usage!T10/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N10" s="30">
+      <c r="N10" s="31">
         <f>MIN(MAX(M10,0),1)</f>
         <v/>
       </c>
-      <c r="O10" s="30">
+      <c r="O10" s="31">
         <f>Capacity_Usage!E10/3</f>
         <v/>
       </c>
-      <c r="P10" s="30">
+      <c r="P10" s="31">
         <f>MIN(MAX(O10,0),1)</f>
         <v/>
       </c>
-      <c r="Q10" s="30">
+      <c r="Q10" s="31">
         <f>Policy!$B$2*H10+Policy!$B$3*J10+Policy!$B$4*L10+Policy!$B$5*N10+Policy!$B$6*P10</f>
         <v/>
       </c>
@@ -8680,47 +8970,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C11),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C11,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G11" s="30">
+      <c r="G11" s="31">
         <f>IFERROR(Capacity_Usage!S11/Capacity_Usage!R11,0)</f>
         <v/>
       </c>
-      <c r="H11" s="30">
+      <c r="H11" s="31">
         <f>MIN(MAX(G11,0),1)</f>
         <v/>
       </c>
-      <c r="I11" s="30">
+      <c r="I11" s="31">
         <f>IFERROR(Capacity_Usage!Q11/Capacity_Usage!O11,0)</f>
         <v/>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="31">
         <f>MIN(MAX(I11,0),1)</f>
         <v/>
       </c>
-      <c r="K11" s="30">
+      <c r="K11" s="31">
         <f>IFERROR(1-Capacity_Usage!U11/F11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="30">
+      <c r="L11" s="31">
         <f>MIN(MAX(K11,0),1)</f>
         <v/>
       </c>
-      <c r="M11" s="30">
+      <c r="M11" s="31">
         <f>IFERROR(Capacity_Usage!T11/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N11" s="30">
+      <c r="N11" s="31">
         <f>MIN(MAX(M11,0),1)</f>
         <v/>
       </c>
-      <c r="O11" s="30">
+      <c r="O11" s="31">
         <f>Capacity_Usage!E11/3</f>
         <v/>
       </c>
-      <c r="P11" s="30">
+      <c r="P11" s="31">
         <f>MIN(MAX(O11,0),1)</f>
         <v/>
       </c>
-      <c r="Q11" s="30">
+      <c r="Q11" s="31">
         <f>Policy!$B$2*H11+Policy!$B$3*J11+Policy!$B$4*L11+Policy!$B$5*N11+Policy!$B$6*P11</f>
         <v/>
       </c>
@@ -8758,47 +9048,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C12),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C12,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G12" s="30">
+      <c r="G12" s="31">
         <f>IFERROR(Capacity_Usage!S12/Capacity_Usage!R12,0)</f>
         <v/>
       </c>
-      <c r="H12" s="30">
+      <c r="H12" s="31">
         <f>MIN(MAX(G12,0),1)</f>
         <v/>
       </c>
-      <c r="I12" s="30">
+      <c r="I12" s="31">
         <f>IFERROR(Capacity_Usage!Q12/Capacity_Usage!O12,0)</f>
         <v/>
       </c>
-      <c r="J12" s="30">
+      <c r="J12" s="31">
         <f>MIN(MAX(I12,0),1)</f>
         <v/>
       </c>
-      <c r="K12" s="30">
+      <c r="K12" s="31">
         <f>IFERROR(1-Capacity_Usage!U12/F12,0)</f>
         <v/>
       </c>
-      <c r="L12" s="30">
+      <c r="L12" s="31">
         <f>MIN(MAX(K12,0),1)</f>
         <v/>
       </c>
-      <c r="M12" s="30">
+      <c r="M12" s="31">
         <f>IFERROR(Capacity_Usage!T12/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N12" s="30">
+      <c r="N12" s="31">
         <f>MIN(MAX(M12,0),1)</f>
         <v/>
       </c>
-      <c r="O12" s="30">
+      <c r="O12" s="31">
         <f>Capacity_Usage!E12/3</f>
         <v/>
       </c>
-      <c r="P12" s="30">
+      <c r="P12" s="31">
         <f>MIN(MAX(O12,0),1)</f>
         <v/>
       </c>
-      <c r="Q12" s="30">
+      <c r="Q12" s="31">
         <f>Policy!$B$2*H12+Policy!$B$3*J12+Policy!$B$4*L12+Policy!$B$5*N12+Policy!$B$6*P12</f>
         <v/>
       </c>
@@ -8836,47 +9126,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C13),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C13,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G13" s="30">
+      <c r="G13" s="31">
         <f>IFERROR(Capacity_Usage!S13/Capacity_Usage!R13,0)</f>
         <v/>
       </c>
-      <c r="H13" s="30">
+      <c r="H13" s="31">
         <f>MIN(MAX(G13,0),1)</f>
         <v/>
       </c>
-      <c r="I13" s="30">
+      <c r="I13" s="31">
         <f>IFERROR(Capacity_Usage!Q13/Capacity_Usage!O13,0)</f>
         <v/>
       </c>
-      <c r="J13" s="30">
+      <c r="J13" s="31">
         <f>MIN(MAX(I13,0),1)</f>
         <v/>
       </c>
-      <c r="K13" s="30">
+      <c r="K13" s="31">
         <f>IFERROR(1-Capacity_Usage!U13/F13,0)</f>
         <v/>
       </c>
-      <c r="L13" s="30">
+      <c r="L13" s="31">
         <f>MIN(MAX(K13,0),1)</f>
         <v/>
       </c>
-      <c r="M13" s="30">
+      <c r="M13" s="31">
         <f>IFERROR(Capacity_Usage!T13/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N13" s="30">
+      <c r="N13" s="31">
         <f>MIN(MAX(M13,0),1)</f>
         <v/>
       </c>
-      <c r="O13" s="30">
+      <c r="O13" s="31">
         <f>Capacity_Usage!E13/3</f>
         <v/>
       </c>
-      <c r="P13" s="30">
+      <c r="P13" s="31">
         <f>MIN(MAX(O13,0),1)</f>
         <v/>
       </c>
-      <c r="Q13" s="30">
+      <c r="Q13" s="31">
         <f>Policy!$B$2*H13+Policy!$B$3*J13+Policy!$B$4*L13+Policy!$B$5*N13+Policy!$B$6*P13</f>
         <v/>
       </c>
@@ -8914,47 +9204,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C14),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C14,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="31">
         <f>IFERROR(Capacity_Usage!S14/Capacity_Usage!R14,0)</f>
         <v/>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="31">
         <f>MIN(MAX(G14,0),1)</f>
         <v/>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="31">
         <f>IFERROR(Capacity_Usage!Q14/Capacity_Usage!O14,0)</f>
         <v/>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="31">
         <f>MIN(MAX(I14,0),1)</f>
         <v/>
       </c>
-      <c r="K14" s="30">
+      <c r="K14" s="31">
         <f>IFERROR(1-Capacity_Usage!U14/F14,0)</f>
         <v/>
       </c>
-      <c r="L14" s="30">
+      <c r="L14" s="31">
         <f>MIN(MAX(K14,0),1)</f>
         <v/>
       </c>
-      <c r="M14" s="30">
+      <c r="M14" s="31">
         <f>IFERROR(Capacity_Usage!T14/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N14" s="30">
+      <c r="N14" s="31">
         <f>MIN(MAX(M14,0),1)</f>
         <v/>
       </c>
-      <c r="O14" s="30">
+      <c r="O14" s="31">
         <f>Capacity_Usage!E14/3</f>
         <v/>
       </c>
-      <c r="P14" s="30">
+      <c r="P14" s="31">
         <f>MIN(MAX(O14,0),1)</f>
         <v/>
       </c>
-      <c r="Q14" s="30">
+      <c r="Q14" s="31">
         <f>Policy!$B$2*H14+Policy!$B$3*J14+Policy!$B$4*L14+Policy!$B$5*N14+Policy!$B$6*P14</f>
         <v/>
       </c>
@@ -8992,47 +9282,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C15),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C15,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G15" s="30">
+      <c r="G15" s="31">
         <f>IFERROR(Capacity_Usage!S15/Capacity_Usage!R15,0)</f>
         <v/>
       </c>
-      <c r="H15" s="30">
+      <c r="H15" s="31">
         <f>MIN(MAX(G15,0),1)</f>
         <v/>
       </c>
-      <c r="I15" s="30">
+      <c r="I15" s="31">
         <f>IFERROR(Capacity_Usage!Q15/Capacity_Usage!O15,0)</f>
         <v/>
       </c>
-      <c r="J15" s="30">
+      <c r="J15" s="31">
         <f>MIN(MAX(I15,0),1)</f>
         <v/>
       </c>
-      <c r="K15" s="30">
+      <c r="K15" s="31">
         <f>IFERROR(1-Capacity_Usage!U15/F15,0)</f>
         <v/>
       </c>
-      <c r="L15" s="30">
+      <c r="L15" s="31">
         <f>MIN(MAX(K15,0),1)</f>
         <v/>
       </c>
-      <c r="M15" s="30">
+      <c r="M15" s="31">
         <f>IFERROR(Capacity_Usage!T15/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N15" s="30">
+      <c r="N15" s="31">
         <f>MIN(MAX(M15,0),1)</f>
         <v/>
       </c>
-      <c r="O15" s="30">
+      <c r="O15" s="31">
         <f>Capacity_Usage!E15/3</f>
         <v/>
       </c>
-      <c r="P15" s="30">
+      <c r="P15" s="31">
         <f>MIN(MAX(O15,0),1)</f>
         <v/>
       </c>
-      <c r="Q15" s="30">
+      <c r="Q15" s="31">
         <f>Policy!$B$2*H15+Policy!$B$3*J15+Policy!$B$4*L15+Policy!$B$5*N15+Policy!$B$6*P15</f>
         <v/>
       </c>
@@ -9070,47 +9360,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C16),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C16,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G16" s="30">
+      <c r="G16" s="31">
         <f>IFERROR(Capacity_Usage!S16/Capacity_Usage!R16,0)</f>
         <v/>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="31">
         <f>MIN(MAX(G16,0),1)</f>
         <v/>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="31">
         <f>IFERROR(Capacity_Usage!Q16/Capacity_Usage!O16,0)</f>
         <v/>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="31">
         <f>MIN(MAX(I16,0),1)</f>
         <v/>
       </c>
-      <c r="K16" s="30">
+      <c r="K16" s="31">
         <f>IFERROR(1-Capacity_Usage!U16/F16,0)</f>
         <v/>
       </c>
-      <c r="L16" s="30">
+      <c r="L16" s="31">
         <f>MIN(MAX(K16,0),1)</f>
         <v/>
       </c>
-      <c r="M16" s="30">
+      <c r="M16" s="31">
         <f>IFERROR(Capacity_Usage!T16/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N16" s="30">
+      <c r="N16" s="31">
         <f>MIN(MAX(M16,0),1)</f>
         <v/>
       </c>
-      <c r="O16" s="30">
+      <c r="O16" s="31">
         <f>Capacity_Usage!E16/3</f>
         <v/>
       </c>
-      <c r="P16" s="30">
+      <c r="P16" s="31">
         <f>MIN(MAX(O16,0),1)</f>
         <v/>
       </c>
-      <c r="Q16" s="30">
+      <c r="Q16" s="31">
         <f>Policy!$B$2*H16+Policy!$B$3*J16+Policy!$B$4*L16+Policy!$B$5*N16+Policy!$B$6*P16</f>
         <v/>
       </c>
@@ -9148,47 +9438,47 @@
         <f>IF(Policy!$B$10=1,SUMIFS(Capacity_Usage!$U$4:$U$17,Capacity_Usage!$C$4:$C$17,Capacity_Usage!C17),IF(Policy!$B$10=2,VLOOKUP(Capacity_Usage!C17,Policy!$D$11:$E$15,2,FALSE),Policy!$B$11))</f>
         <v/>
       </c>
-      <c r="G17" s="30">
+      <c r="G17" s="31">
         <f>IFERROR(Capacity_Usage!S17/Capacity_Usage!R17,0)</f>
         <v/>
       </c>
-      <c r="H17" s="30">
+      <c r="H17" s="31">
         <f>MIN(MAX(G17,0),1)</f>
         <v/>
       </c>
-      <c r="I17" s="30">
+      <c r="I17" s="31">
         <f>IFERROR(Capacity_Usage!Q17/Capacity_Usage!O17,0)</f>
         <v/>
       </c>
-      <c r="J17" s="30">
+      <c r="J17" s="31">
         <f>MIN(MAX(I17,0),1)</f>
         <v/>
       </c>
-      <c r="K17" s="30">
+      <c r="K17" s="31">
         <f>IFERROR(1-Capacity_Usage!U17/F17,0)</f>
         <v/>
       </c>
-      <c r="L17" s="30">
+      <c r="L17" s="31">
         <f>MIN(MAX(K17,0),1)</f>
         <v/>
       </c>
-      <c r="M17" s="30">
+      <c r="M17" s="31">
         <f>IFERROR(Capacity_Usage!T17/Policy!$B$14,0)</f>
         <v/>
       </c>
-      <c r="N17" s="30">
+      <c r="N17" s="31">
         <f>MIN(MAX(M17,0),1)</f>
         <v/>
       </c>
-      <c r="O17" s="30">
+      <c r="O17" s="31">
         <f>Capacity_Usage!E17/3</f>
         <v/>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="31">
         <f>MIN(MAX(O17,0),1)</f>
         <v/>
       </c>
-      <c r="Q17" s="30">
+      <c r="Q17" s="31">
         <f>Policy!$B$2*H17+Policy!$B$3*J17+Policy!$B$4*L17+Policy!$B$5*N17+Policy!$B$6*P17</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
feat(mockup): add Formula_Reference sheet with comprehensive PS formula tables
- New Formula_Reference sheet explains PS_Prod, PS_NonProd, PS_DR formulas
- Each formula broken down into 5 components (α, β, γ, δ, ε) with:
  * What it measures (purpose)
  * Signal/formula (exact calculation)
  * Weight (contribution to final score)
  * Detailed explanation (rationale and behavior)
  * Excel column references (Capacity_Usage and Scoring sheet mappings)
- Final score rows for each mode with argmax selection logic
- Key notes section covering clamping, weight constraints, model independence,
  open issues (total_customers undefined), and PS_NonProd α/δ duplication
- Addresses user question: why PS_Prod α uses NonProd headroom (regional health
  indicator, not self-referential Prod capacity check)
</commit_message>
<xml_diff>
--- a/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
+++ b/Mockups/acrme_region_selection_whatif_acrme_regions.xlsx
@@ -17,6 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_CVAL" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring_DR" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Result" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Formula_Reference" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +29,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -70,8 +71,28 @@
       <color rgb="00808080"/>
       <sz val="9"/>
     </font>
+    <font>
+      <i val="1"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -113,6 +134,11 @@
         <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -140,7 +166,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -221,6 +247,43 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2013,6 +2076,851 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="35" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>PLACEMENT SCORING FORMULA REFERENCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="34" t="inlineStr">
+        <is>
+          <t>This sheet explains the three placement scoring (PS) formulas used by the ACRME region-selection engine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="34" t="inlineStr">
+        <is>
+          <t>Each formula evaluates candidate regions across five weighted components (α, β, γ, δ, ε) that sum to 1.0.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="34" t="inlineStr">
+        <is>
+          <t>All components are clamped to [0, 1] to prevent outliers from dominating the score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="35" t="inlineStr">
+        <is>
+          <t>PS_Prod — PRODUCTION REGION SCORING</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>What It Measures</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="inlineStr">
+        <is>
+          <t>Signal / Formula</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+      <c r="F8" s="36" t="inlineStr">
+        <is>
+          <t>Excel Column References</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>α</t>
+        </is>
+      </c>
+      <c r="B9" s="38" t="inlineStr">
+        <is>
+          <t>Capacity headroom (forward-looking regional health)</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(nonprod_crg.effective_free / prod_crg.quantity)</t>
+        </is>
+      </c>
+      <c r="D9" s="40" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="E9" s="38" t="inlineStr">
+        <is>
+          <t>Uses NonProd effective free capacity as a regional health indicator. A region with ample NonProd headroom signals overall capacity health, overflow capacity for Prod spikes, and readiness for future CVAL co-location (2-region model). This is NOT self-referential — it evaluates regional capacity resilience, not just Prod-specific capacity.</t>
+        </is>
+      </c>
+      <c r="F9" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: N (NP Eff-Free) ÷ F (Prod Reserved)
+Scoring_Prod: G (α_raw), H (α_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>β</t>
+        </is>
+      </c>
+      <c r="B10" s="38" t="inlineStr">
+        <is>
+          <t>Quota headroom (direct Prod capacity readiness)</t>
+        </is>
+      </c>
+      <c r="C10" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(prod_crg.quota_headroom / prod_crg.quota_limit)</t>
+        </is>
+      </c>
+      <c r="D10" s="40" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="E10" s="38" t="inlineStr">
+        <is>
+          <t>Direct measure of Prod quota availability. High quota headroom means the region can accommodate the Prod workload without quota exhaustion. This complements α by providing a Prod-specific capacity signal while α measures regional health.</t>
+        </is>
+      </c>
+      <c r="F10" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: K (Prod Q-Headroom) ÷ I (Prod Q-Limit)
+Scoring_Prod: I (β_raw), J (β_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="90" customHeight="1">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>γ</t>
+        </is>
+      </c>
+      <c r="B11" s="38" t="inlineStr">
+        <is>
+          <t>Distribution fairness (load balancing)</t>
+        </is>
+      </c>
+      <c r="C11" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(1 - prod_customer_count / total_customers)</t>
+        </is>
+      </c>
+      <c r="D11" s="40" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E11" s="38" t="inlineStr">
+        <is>
+          <t>Rewards regions with fewer existing Prod customers, promoting even distribution of workload across the geography. A region with lower customer count scores higher, preventing concentration in a single region. ⚠️ Note: total_customers is currently UNDEFINED in baseline v2.4 (scope and source unspecified).</t>
+        </is>
+      </c>
+      <c r="F11" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: U (Cust Count)
+Scoring_Prod: F (total_cust for denominator), K (γ_raw), L (γ_c)
+⚠️ total_customers scope: geography-level (most likely) or global (pending clarification)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="90" customHeight="1">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>δ</t>
+        </is>
+      </c>
+      <c r="B12" s="38" t="inlineStr">
+        <is>
+          <t>DR readiness signal (destination DR coverage)</t>
+        </is>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(dr_crg.coverage_ratio)</t>
+        </is>
+      </c>
+      <c r="D12" s="40" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="E12" s="38" t="inlineStr">
+        <is>
+          <t>Measures the region's existing DR coverage ratio — how much of its DR requirement is already met. A region with good DR coverage is more resilient and can potentially host additional DR workloads (multi-source DR hosting, DR-016).</t>
+        </is>
+      </c>
+      <c r="F12" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: T (DR Coverage)
+Scoring_Prod: M (δ_raw), N (δ_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="90" customHeight="1">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>ε</t>
+        </is>
+      </c>
+      <c r="B13" s="38" t="inlineStr">
+        <is>
+          <t>Zone diversity (availability zone count)</t>
+        </is>
+      </c>
+      <c r="C13" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(az_count / 3)</t>
+        </is>
+      </c>
+      <c r="D13" s="40" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="E13" s="38" t="inlineStr">
+        <is>
+          <t>Favors regions with more availability zones (max 3 in Azure). Higher zone count provides better fault isolation and distributes VMs more evenly (PLC-011 even zone-distribution target). A 3-AZ region scores 1.0; 2-AZ scores 0.67; 1-AZ scores 0.33.</t>
+        </is>
+      </c>
+      <c r="F13" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: E (AZ)
+Scoring_Prod: O (ε_raw), P (ε_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="A14" s="42" t="inlineStr">
+        <is>
+          <t>FINAL SCORE</t>
+        </is>
+      </c>
+      <c r="B14" s="43" t="inlineStr">
+        <is>
+          <t>Weighted sum of all five components</t>
+        </is>
+      </c>
+      <c r="C14" s="44" t="inlineStr">
+        <is>
+          <t>PS_Prod = 0.30×α + 0.20×β + 0.25×γ + 0.15×δ + 0.10×ε</t>
+        </is>
+      </c>
+      <c r="D14" s="45" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E14" s="46" t="inlineStr">
+        <is>
+          <t>Range: [0, 1]. Highest score = best candidate. Winner = argmax(PS_Prod) over eligible Standard regions.</t>
+        </is>
+      </c>
+      <c r="F14" s="47" t="inlineStr">
+        <is>
+          <t>Scoring_Prod: Q (PS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>PS_NonProd — CVAL (NON-PRODUCTION) REGION SCORING</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="36" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>What It Measures</t>
+        </is>
+      </c>
+      <c r="C18" s="36" t="inlineStr">
+        <is>
+          <t>Signal / Formula</t>
+        </is>
+      </c>
+      <c r="D18" s="36" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="E18" s="36" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+      <c r="F18" s="36" t="inlineStr">
+        <is>
+          <t>Excel Column References</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="90" customHeight="1">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>α</t>
+        </is>
+      </c>
+      <c r="B19" s="38" t="inlineStr">
+        <is>
+          <t>Capacity headroom (direct NonProd capacity)</t>
+        </is>
+      </c>
+      <c r="C19" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(nonprod_crg.effective_free / nonprod_crg.quantity)</t>
+        </is>
+      </c>
+      <c r="D19" s="40" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="E19" s="38" t="inlineStr">
+        <is>
+          <t>Direct measure of NonProd effective free capacity. Unlike PS_Prod (which uses NonProd as a regional health signal), here we evaluate NonProd capacity directly for CVAL placement. High NonProd headroom = region can accommodate CVAL workload.</t>
+        </is>
+      </c>
+      <c r="F19" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: N (NP Eff-Free) ÷ L (NP Reserved)
+Scoring_CVAL: G (α_raw), H (α_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="90" customHeight="1">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>β</t>
+        </is>
+      </c>
+      <c r="B20" s="38" t="inlineStr">
+        <is>
+          <t>Quota headroom (NonProd quota availability)</t>
+        </is>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(nonprod_crg.quota_headroom / nonprod_crg.quota_limit)</t>
+        </is>
+      </c>
+      <c r="D20" s="40" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="E20" s="38" t="inlineStr">
+        <is>
+          <t>NonProd quota headroom. Ensures the region has sufficient NonProd quota to accommodate the CVAL workload without hitting quota limits.</t>
+        </is>
+      </c>
+      <c r="F20" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: Q (NP Q-Headroom) ÷ O (NP Q-Limit)
+Scoring_CVAL: I (β_raw), J (β_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1">
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>γ</t>
+        </is>
+      </c>
+      <c r="B21" s="38" t="inlineStr">
+        <is>
+          <t>Distribution fairness (load balancing)</t>
+        </is>
+      </c>
+      <c r="C21" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(1 - nonprod_customer_count / total_customers)</t>
+        </is>
+      </c>
+      <c r="D21" s="40" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E21" s="38" t="inlineStr">
+        <is>
+          <t>Rewards regions with fewer existing NonProd customers, promoting even CVAL distribution. Identical logic to PS_Prod but evaluated against NonProd customer counts. ⚠️ total_customers scope undefined.</t>
+        </is>
+      </c>
+      <c r="F21" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: U (Cust Count)
+Scoring_CVAL: F (total_cust for denominator), K (γ_raw), L (γ_c)
+⚠️ total_customers scope: geography-level (most likely) or global (pending clarification)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="90" customHeight="1">
+      <c r="A22" s="37" t="inlineStr">
+        <is>
+          <t>δ</t>
+        </is>
+      </c>
+      <c r="B22" s="38" t="inlineStr">
+        <is>
+          <t>Overflow capacity health (redundant with α)</t>
+        </is>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(nonprod_crg.effective_free / nonprod_crg.quantity)</t>
+        </is>
+      </c>
+      <c r="D22" s="40" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="E22" s="38" t="inlineStr">
+        <is>
+          <t>⚠️ DUPLICATE: This is identical to α. Combined α+δ weight = 0.45. This is the design-of-record formula (baseline v2.4). A pilot variant exists that removes this duplication and reallocates the weight.</t>
+        </is>
+      </c>
+      <c r="F22" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: N (NP Eff-Free) ÷ L (NP Reserved)
+Scoring_CVAL: M (δ_raw), N (δ_c)
+⚠️ Same as α — duplication acknowledged in Calculation Logic Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>ε</t>
+        </is>
+      </c>
+      <c r="B23" s="38" t="inlineStr">
+        <is>
+          <t>Zone diversity (availability zone count)</t>
+        </is>
+      </c>
+      <c r="C23" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(az_count / 3)</t>
+        </is>
+      </c>
+      <c r="D23" s="40" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="E23" s="38" t="inlineStr">
+        <is>
+          <t>Identical to PS_Prod. Favors regions with more availability zones for better fault isolation.</t>
+        </is>
+      </c>
+      <c r="F23" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: E (AZ)
+Scoring_CVAL: O (ε_raw), P (ε_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="42" t="inlineStr">
+        <is>
+          <t>FINAL SCORE</t>
+        </is>
+      </c>
+      <c r="B24" s="43" t="inlineStr">
+        <is>
+          <t>Weighted sum of all five components</t>
+        </is>
+      </c>
+      <c r="C24" s="44" t="inlineStr">
+        <is>
+          <t>PS_NonProd = 0.30×α + 0.20×β + 0.25×γ + 0.15×δ + 0.10×ε</t>
+        </is>
+      </c>
+      <c r="D24" s="45" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E24" s="46" t="inlineStr">
+        <is>
+          <t>Range: [0, 1]. Highest score = best CVAL candidate. Winner = argmax(PS_NonProd) over eligible Standard regions (excluding Prod region). In 2-region model (EU, AU, AP): CVAL placement is deterministic (the other Standard region).</t>
+        </is>
+      </c>
+      <c r="F24" s="47" t="inlineStr">
+        <is>
+          <t>Scoring_CVAL: Q (PS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="35" t="inlineStr">
+        <is>
+          <t>PS_DR — DR (DISASTER RECOVERY) REGION SCORING</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="36" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B28" s="36" t="inlineStr">
+        <is>
+          <t>What It Measures</t>
+        </is>
+      </c>
+      <c r="C28" s="36" t="inlineStr">
+        <is>
+          <t>Signal / Formula</t>
+        </is>
+      </c>
+      <c r="D28" s="36" t="inlineStr">
+        <is>
+          <t>Weight</t>
+        </is>
+      </c>
+      <c r="E28" s="36" t="inlineStr">
+        <is>
+          <t>Explanation</t>
+        </is>
+      </c>
+      <c r="F28" s="36" t="inlineStr">
+        <is>
+          <t>Excel Column References</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="90" customHeight="1">
+      <c r="A29" s="37" t="inlineStr">
+        <is>
+          <t>α</t>
+        </is>
+      </c>
+      <c r="B29" s="38" t="inlineStr">
+        <is>
+          <t>Capacity headroom (DR CRG free slots)</t>
+        </is>
+      </c>
+      <c r="C29" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(dr_crg.free_slots / dr_crg.quantity)</t>
+        </is>
+      </c>
+      <c r="D29" s="40" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="E29" s="38" t="inlineStr">
+        <is>
+          <t>Direct measure of DR capacity headroom. High DR free slots = region can accommodate additional DR workload. This evaluates the region's ability to serve as a DR destination (multi-source DR hosting, DR-016).</t>
+        </is>
+      </c>
+      <c r="F29" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: S (DR Free) ÷ R (DR Reserved)
+Scoring_DR: G (α_raw), H (α_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
+      <c r="A30" s="37" t="inlineStr">
+        <is>
+          <t>β</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>Quota headroom (DR quota availability)</t>
+        </is>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(dr_crg.quota_headroom / dr_crg.quota_limit)</t>
+        </is>
+      </c>
+      <c r="D30" s="40" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="E30" s="38" t="inlineStr">
+        <is>
+          <t>DR quota headroom. In practice, DR uses NonProd quota (DR VMs are in a NonProd environment), so this typically references NP Q-Headroom. Ensures the region has sufficient quota to accommodate the DR workload.</t>
+        </is>
+      </c>
+      <c r="F30" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: Q (NP Q-Headroom) ÷ O (NP Q-Limit)
+Scoring_DR: I (β_raw), J (β_c)
+(DR uses NonProd quota per ENV-002)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="37" t="inlineStr">
+        <is>
+          <t>γ</t>
+        </is>
+      </c>
+      <c r="B31" s="38" t="inlineStr">
+        <is>
+          <t>Distribution fairness (load balancing)</t>
+        </is>
+      </c>
+      <c r="C31" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(1 - dr_customer_count / total_customers)</t>
+        </is>
+      </c>
+      <c r="D31" s="40" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E31" s="38" t="inlineStr">
+        <is>
+          <t>Rewards regions with fewer existing DR customers, promoting even DR distribution. Prevents DR concentration in a single destination region. ⚠️ total_customers scope undefined.</t>
+        </is>
+      </c>
+      <c r="F31" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: U (Cust Count)
+Scoring_DR: F (total_cust for denominator), K (γ_raw), L (γ_c)
+⚠️ total_customers scope: geography-level (most likely) or global (pending clarification)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
+      <c r="A32" s="37" t="inlineStr">
+        <is>
+          <t>δ</t>
+        </is>
+      </c>
+      <c r="B32" s="38" t="inlineStr">
+        <is>
+          <t>Coverage ratio health (DR sizing adequacy)</t>
+        </is>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>min(1.0, dr_crg.coverage_ratio / dr_coverage_target)</t>
+        </is>
+      </c>
+      <c r="D32" s="40" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="E32" s="38" t="inlineStr">
+        <is>
+          <t>Measures how close the region's existing DR coverage is to the configured target. Uses min(1.0, ...) instead of Clamp() for normalization. dr_coverage_target is a configurable scoring reference (per customer/product), NOT the retired 30-40% dr_ratio. DR sizing uses max-not-sum (A.6, DR-017).</t>
+        </is>
+      </c>
+      <c r="F32" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: T (DR Coverage)
+Scoring_DR: M (δ_raw), N (δ_c)
+dr_coverage_target = configurable scoring parameter (Policy sheet or config)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1">
+      <c r="A33" s="37" t="inlineStr">
+        <is>
+          <t>ε</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="inlineStr">
+        <is>
+          <t>Zone diversity (availability zone count)</t>
+        </is>
+      </c>
+      <c r="C33" s="39" t="inlineStr">
+        <is>
+          <t>Clamp(az_count / 3)</t>
+        </is>
+      </c>
+      <c r="D33" s="40" t="inlineStr">
+        <is>
+          <t>0.10</t>
+        </is>
+      </c>
+      <c r="E33" s="38" t="inlineStr">
+        <is>
+          <t>Identical to PS_Prod and PS_NonProd. Favors regions with more availability zones for better DR fault isolation.</t>
+        </is>
+      </c>
+      <c r="F33" s="41" t="inlineStr">
+        <is>
+          <t>Capacity_Usage: E (AZ)
+Scoring_DR: O (ε_raw), P (ε_c)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="60" customHeight="1">
+      <c r="A34" s="42" t="inlineStr">
+        <is>
+          <t>FINAL SCORE</t>
+        </is>
+      </c>
+      <c r="B34" s="43" t="inlineStr">
+        <is>
+          <t>Weighted sum of all five components</t>
+        </is>
+      </c>
+      <c r="C34" s="44" t="inlineStr">
+        <is>
+          <t>PS_DR = 0.30×α + 0.20×β + 0.25×γ + 0.15×δ + 0.10×ε</t>
+        </is>
+      </c>
+      <c r="D34" s="45" t="inlineStr">
+        <is>
+          <t>1.00</t>
+        </is>
+      </c>
+      <c r="E34" s="46" t="inlineStr">
+        <is>
+          <t>Range: [0, 1]. Highest score = best DR candidate. Winner = argmax(PS_DR) over eligible Standard regions (excluding Prod, CVAL). In 2-region model (EU, AU, AP): DR co-locates with CVAL (PLC-010a mandatory). Middle East: DR cross-geo in Europe (weighted-selected).</t>
+        </is>
+      </c>
+      <c r="F34" s="47" t="inlineStr">
+        <is>
+          <t>Scoring_DR: Q (PS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="48" t="inlineStr">
+        <is>
+          <t>KEY NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>1. Clamp(x) = MIN(MAX(x, 0), 1) — ensures all component values stay in [0, 1] range to prevent outliers from dominating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>2. Weight sum constraint: α + β + γ + δ + ε = 1.0 (enforced by Policy sheet validation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>3. The three PS formulas are IDENTICAL across all region models (2-region, 3-region, 4-region, cross-geo). What changes: number of argmax passes, candidate pool, HC gate constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="30" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>4. ⚠️ OPEN ISSUE: total_customers (γ component) is UNDEFINED in baseline v2.4 — no source, scope, or data type specified. Geography-level scope is most likely.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="30" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>5. PS_NonProd α and δ are identical (design-of-record v2.4) — combined weight 0.45. A pilot variant exists that removes this duplication.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>6. PS_DR δ uses min(1.0, ...) instead of Clamp() for coverage-ratio normalization.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>7. Column references: _raw = unclamped component; _c = clamped component; PS = final placement score.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="30" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>8. Winner selection: argmax(PS) over eligible Standard regions (or deterministic in 2-region co-located model).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="16">
+    <mergeCell ref="A38:F38"/>
+    <mergeCell ref="A41:F41"/>
+    <mergeCell ref="A42:F42"/>
+    <mergeCell ref="A36:F36"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A40:F40"/>
+    <mergeCell ref="A4:F4"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A39:F39"/>
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A43:F43"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>